<commit_message>
Registra a San Lazaro Art como sin modificaciones para Ago-26 (respondió 24/08)
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -197,7 +197,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -289,6 +289,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
         <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE9F5"/>
+        <bgColor rgb="00DCE9F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -420,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -545,6 +551,7 @@
     <xf numFmtId="0" fontId="28" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6227,14 +6234,24 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K115" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para agosto</t>
+        </is>
+      </c>
+      <c r="K115" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7038,23 +7055,23 @@
         <v>42</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>15</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G6" s="12" t="n">
         <v>15</v>
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="I6" s="17">
@@ -7177,19 +7194,19 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="19" t="n">
         <v>15</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
@@ -7282,19 +7299,19 @@
         <v>126</v>
       </c>
       <c r="C7" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E7" t="n">
         <v>46</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4603174603174603</v>
+        <v>0.4682539682539683</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Abre el ciclo Septiembre 2026 (Sep-26)
Se duplica el bloque de 42 hoteles del ciclo anterior (Ago-26) con sus
contactos más recientes (incluye el nuevo contacto de Park Lake Luxury),
fecha de envío 02/09/2026, y campos de respuesta/modificaciones neutros.

- HTML: nuevo bloque en allData, aparece automáticamente como pestaña
  "Sep-26" y en el panel de gráficos de la pestaña Métricas.
- Excel: 42 filas nuevas en Consolidado (color rosa, 4to en la rotación),
  nueva fila en Dashboard cumplimiento (insertada arriba, recalculando
  TOTAL) y en Resumen por ciclo.
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -196,8 +196,13 @@
       <color rgb="00006100"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="009D174D"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -295,6 +300,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DCE9F5"/>
         <bgColor rgb="00DCE9F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE7F3"/>
+        <bgColor rgb="00FCE7F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -426,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -552,6 +563,7 @@
     <xf numFmtId="0" fontId="29" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -917,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6873,6 +6885,1560 @@
         </is>
       </c>
       <c r="K129" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Luis Saez</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>luis.saez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K130" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Biohotel</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Maria Del Pilar Narvaez</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>pilar.narvaez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K131" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>calidad.bioxury@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K132" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Geotel Antofagasta</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Nelson Uriel Perez Ortiz</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>nelson.perez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K133" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Katherine Mora</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>katherine.mora@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K134" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>GHL Collection 93</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>James Mendoza</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>james.mendoza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K135" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Armeria Real</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Saray Estrada</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Saray.estrada@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K136" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>GHL Collection Hamilton</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Wilson Bohorquez</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>andres.bohorquez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K137" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>GHL Grand Villavicencio</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Ingrid Mendez</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>jimena.mendez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K138" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>GHL Hotel Capital</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Maira Piza</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>maira.piza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K139" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>GHL Lago Titicaca</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Milagros Velazco Reyes</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>milagros.velazco@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K140" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>GHL Montería</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Jose Medina</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>mauricio.medina@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K141" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>GHL Portón Medellín</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Jose Fernando Villareal</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>jose.villareal@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K142" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Maria Gomez</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>angelica.gomez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K143" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Corales de Indias</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Andres Narvaez</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>andres.narvaez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K144" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Costa Azul</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Marlis Marriaga</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>marlys.marriaga@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K145" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>juan.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K146" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Luis Martinez</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>luis.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K147" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Leidy Cely</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>jrecepcion.bogotaoccidente@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K148" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Carlos Robayo</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>yobani.robayo@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K149" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Mafy Daniela Rodriguez</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>daniela.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K150" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sara Judith Aguirre</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>sara.aguirre@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K151" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Katerine Ospina Gil</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>suprecepcion.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K152" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Jose Carlos Ibañez</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>jose.ibanez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K153" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>LATAM XELA</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Gabriela Rodas</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>gabriela.rodas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K154" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Jose Macea</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>jose.macea@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K155" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Sergio Víctor Alejandro Yevenes Escobar</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>sergio.yevenes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K156" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>San Lazaro Art</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Keilis Mercado</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>keilis.mercado@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K157" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Jeferson Reyes</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>jeferson.reyes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K158" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Sonesta Cali</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Lorena Figueroa</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>lorena.figueroa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K159" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Sonesta Cartagena</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Liliana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>liliana.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K160" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Adolfo Alfaro</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>adolfo.alfaro@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K161" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Andrea Silvana Zevallos</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>andrea.zevallos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K162" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Tania Catacora</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>jefederecepcion.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K163" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Catalina Rojas</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>catalina.rojas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K164" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Sonesta Ibagué</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Wilmer Rodriguez</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>wilmer.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K165" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Sonesta Loja</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Miryam Ramirez</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>miryam.ramirez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K166" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Sonesta Osorno</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Cristina Sanzana</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>cristina.sanzana@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K167" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Edwar Pacanchique</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>edwar.pacanchique@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K168" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Delmy Nuñez</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>delmy.nunez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K169" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Sonesta Yucay</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Monica Chirinos</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>monica.chirinos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K170" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="49" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Sonesta Valledupar</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Emerson David Cotes</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>emerson.cotes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K171" s="44" t="inlineStr">
         <is>
           <t>Sin respuesta</t>
         </is>
@@ -6902,7 +8468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7076,6 +8642,40 @@
       </c>
       <c r="I6" s="17">
         <f>IF(B6&gt;0,C6/B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>42</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I7">
+        <f>IF(B7&gt;0,C7/B7,0)</f>
         <v/>
       </c>
     </row>
@@ -7103,7 +8703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7185,35 +8785,35 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>Ago-26</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>42</v>
       </c>
-      <c r="C4" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="D4" s="19" t="n">
-        <v>22</v>
-      </c>
-      <c r="E4" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F4" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G4" s="20" t="n">
-        <v>0.4761904761904762</v>
-      </c>
-      <c r="H4" s="21" t="inlineStr">
-        <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>42</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -7222,105 +8822,140 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>Ago-26</t>
         </is>
       </c>
       <c r="B5" s="19" t="n">
         <v>42</v>
       </c>
       <c r="C5" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>0.4761904761904762</v>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="C6" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D6" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E6" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F6" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G6" s="20" t="n">
         <v>0.3809523809523809</v>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>███████████░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I5" s="22" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>Jun-26</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
         <v>42</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C7" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D7" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E7" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F7" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G7" s="20" t="n">
         <v>0.5476190476190477</v>
       </c>
-      <c r="H6" s="25" t="inlineStr">
+      <c r="H7" s="25" t="inlineStr">
         <is>
           <t>████████████████░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I6" s="26" t="inlineStr">
+      <c r="I7" s="26" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>126</v>
-      </c>
-      <c r="C7" t="n">
+      <c r="B8" t="n">
+        <v>168</v>
+      </c>
+      <c r="C8" t="n">
         <v>59</v>
       </c>
-      <c r="D7" t="n">
-        <v>67</v>
-      </c>
-      <c r="E7" t="n">
+      <c r="D8" t="n">
+        <v>109</v>
+      </c>
+      <c r="E8" t="n">
         <v>46</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F8" t="n">
         <v>13</v>
       </c>
-      <c r="G7" t="n">
-        <v>0.4682539682539683</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="G8" t="n">
+        <v>0.3511904761904762</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>███████████░░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>Nota: La barra de progreso refleja % de hoteles que respondieron el correo (con o sin modificaciones). Completo = 100% · En progreso = 50-99% · Pendiente = &lt; 50%</t>
         </is>
@@ -7329,9 +8964,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A6"/>
-    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="A9:I9"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Registra respuestas de septiembre (Sep-26): 18 hoteles procesados
10 hoteles con modificaciones (Arsenal, GHL Relax Hotel Sunrise, GHL Style
Yopal, Sonesta Arequipa, Sonesta Bogotá, Sonesta Pereira, GHL Relax Club
Hotel el Puente, GHL Hotel Abadía Plaza, Geotel Calama, Makani Luxury
Wanderlust) y 8 sin modificaciones (Armeria Real, GHL Lago Titicaca, GHL
Relax Hotel Costa Azul, GHL Style Bogotá Occidente, GHL Hotel Grand
Barranquilla, San Lazaro Art, Sonesta Cusco, Sonesta Puno).

Geotel Calama y Makani Luxury Wanderlust con datos parciales (valores
'antes' marcados ⚠ Verificar en correo). Bioxury permanece sin respuesta
real (solo reenvío interno). GHL Style Yopal reporta que ediciones de
ciclos previos no se reflejan en el chatbot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6916,14 +6916,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K130" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>7 diálogos modificados: desayuno, tarifas, objetos perdidos, delivery, taxi, ascensor, teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="K130" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7064,14 +7074,29 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K134" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>11 diálogos modificados: contacto, pago, desayuno, cuna, lavandería, ocupación, horarios, gimnasio, ascensor, transporte</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Respuesta con formato informal — varios diálogos sin número claro o sin valor 'antes'; ver detalle. Diálogo 14-02 con respuesta poco clara ('NO ENTENDI')</t>
+        </is>
+      </c>
+      <c r="K134" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7138,14 +7163,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K136" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K136" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7286,14 +7321,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K140" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K140" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7397,14 +7442,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K143" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: remodelación, day use, mascotas, piscina</t>
+        </is>
+      </c>
+      <c r="K143" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7471,14 +7526,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K145" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K145" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7508,14 +7573,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K146" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>8 diálogos modificados: contacto, reservas, pago, day pass, check-in, desayuno, parqueadero, club infantil</t>
+        </is>
+      </c>
+      <c r="K146" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7582,14 +7657,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K148" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K148" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7656,14 +7741,29 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K150" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>7 diálogos modificados: método de pago, check-in, check-out, desayuno, mascotas, spa</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Reporta que los ajustes enviados en ciclos anteriores no se ven reflejados en el chatbot — verificar</t>
+        </is>
+      </c>
+      <c r="K150" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7730,14 +7830,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K152" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>4 diálogos modificados: cajero, mascotas, reservas restaurante, brunch</t>
+        </is>
+      </c>
+      <c r="K152" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7767,14 +7877,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K153" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K153" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7841,14 +7961,29 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K155" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>12 diálogos actualizados vía PDF adjunto: pases, recepción, check-in, parqueadero, muelle, niños, conserjería, objetos perdidos, transporte, eventos, boutique</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Correcciones enviadas solo en PDF adjunto, sin texto antes/después en el cuerpo del correo — valores 'antes' marcados como Verificar en correo</t>
+        </is>
+      </c>
+      <c r="K155" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7915,14 +8050,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K157" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K157" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8063,14 +8208,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K161" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K161" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8137,14 +8292,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K163" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>9 diálogos modificados: lavandería, fumadores, baño, cama extra, empleo, propinas, reservas restaurante, spa, restaurante</t>
+        </is>
+      </c>
+      <c r="K163" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8174,14 +8339,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K164" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>13 diálogos modificados: clasificación, fumadores, baño, cama extra, contacto, parqueadero, balcón, mascotas, bar, spa, restaurante, delivery, San Valentín</t>
+        </is>
+      </c>
+      <c r="K164" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8322,14 +8497,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K168" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>3 diálogos modificados: desayuno, taxi, restaurante</t>
+        </is>
+      </c>
+      <c r="K168" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8359,14 +8544,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K169" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K169" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8655,23 +8850,23 @@
         <v>42</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="I7">
@@ -8794,26 +8989,26 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+          <t>█████████████░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" s="44" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -8934,23 +9129,23 @@
         <v>168</v>
       </c>
       <c r="C8" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="D8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="E8" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="F8" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3511904761904762</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>███████████░░░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -8965,8 +9160,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A7"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8978,7 +9173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H428"/>
+  <dimension ref="A1:H508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -25212,6 +25407,2566 @@
         </is>
       </c>
       <c r="H428" s="41" t="n"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Nombre del restaurante</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Restaurante Corozo &amp; Timbal</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Restaurante Úrsula; se agrega opción Room Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Precio adulto</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>65000 COP</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>80000 COP visitantes / 60000 COP huéspedes sin desayuno incluido</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>13-42</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Lost &amp; found</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Correo y teléfono</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Solo correo (se retira teléfono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>13-46</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Política de entregas</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Solo hasta 10 KG</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Se aceptan entregas de todas las plataformas; se agrega correo de contacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Precio y tiempo</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Aeropuerto 20000 COP/17min, Hotel 25000 COP/20min</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Aeropuerto-Hotel desde 25000 COP/17min, Hotel-Aeropuerto desde 25000 COP/20min</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Floor arrangement &amp; elevator</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Accesibilidad ascensor</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>No accesible para sillas de ruedas</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Accesible para sillas de ruedas</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>14-04, 15-26, 15-61, 15-62, 15-99, 16-03, 17-44</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>+57 (605) 660 5831</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>+57 316 0107651</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Teléfonos</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Sin línea gratuita</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Se agregan teléfonos gratuitos de recepción y eventos</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>10-04, 10-06</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Reservation modification/cancellation</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Correo y teléfono</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>reservas.sunrise, sin línea gratuita</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>reservas2.sunrise@ghlhoteles.com + teléfono gratuito 3175387071</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Transferencias</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>No mencionadas</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Se agrega transferencia a cuenta bancaria del hotel y Wompi</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>10-41</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Day use / day pass</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Edad tarifa infantil</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Sin rango de edad</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Niños de 3 a 11 años</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Early check-in</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Sin condición</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Sujeto a disponibilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>07:00 a 10:00, sin especificar tipo</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Buffet de 07:00 a 10:00 en restaurante</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Parqueadero cercano</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Sin recomendación</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Se agrega parqueadero Aeropuerto como opción cercana</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Club infantil</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Sin días/horario</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Lu, Mar, Mié, Jue, Vie y Sáb de 13:00 a 21:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Métodos de pago</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Sin Visa; no se acepta efectivo</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Se agrega Visa; se acepta pago en efectivo en recepción</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Early check-in</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>70000 COP</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>70000 COP</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Horario y servicio a la habitación</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>06:00-10:00 todos los días; sin room service</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Lu-Sáb 06:00-10:00, Dom/fest 06:00-10:30; se ofrece con cargo adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Precio adulto</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>48000 COP</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>40000 COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Tasa mascota</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>70000 COP/mascota</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA/mascota</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Horario de spa sin restricciones</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Ya no cuentan con spa</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>13-43</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Tiempo de entrega</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Se devuelve antes de las 10:00</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Se devuelve el mismo día</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Tarifa limpieza por humo</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>700 PEN</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>USD 200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Artículos gratis a petición</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Pantuflas, pasta de dientes, kit de afeitar</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Pantuflas, kit dental, kit de afeitar, costurero, limpia calzados y peine</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>15-24, 15-99</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Extra bed / Specific room request</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Incluía calidad.sonestaarequipa</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Solo reservas.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>16-06</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Jobs &amp; internships</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Contacto RRHH</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>contactenos@ghlhoteles.com / +57 601 3139330</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>laydy.pauca@ghlhoteles.com / +51 054 308 777</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>16-25</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Tips policy</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Política de propinas</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Incluía la línea 'es costumbre dejar propina'</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Se elimina esa línea</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>17-02, 18-02, 18-03, 18-04</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Reservas restaurante/bar</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Solo correo</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Se agrega +51 945 739 921</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>17-10</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Spa</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Política de acceso</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Abierto solo clientes; edad mínima 12 años</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Menores de 12 solo con padres/tutor; masajes con costo adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Descripción restaurante Micaela</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Incluía capacidad, política de niños y tronas</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Descripción simplificada (se retira info de capacidad y niños)</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Clasificación del hotel</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Estrellas</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>5 estrellas</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>4 estrellas</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Detectores de humo</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Las habitaciones no están equipadas con detectores de humo</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Las habitaciones están equipadas con detectores de humo</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Artículos gratis / no disponibles</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Lista distinta</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Se agregan albornoz, pantuflas, gel de ducha, hisopos, cepillo y pasta de dientes; se recorta lista de no disponibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Precio cama extra</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>110000 COP/noche</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Se elimina el precio; solo se indica correo de solicitud</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Teléfono gratuito</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>+57 3052281127 (recepción, reserva y eventos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>10-04, 10-06</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Reservation modification/cancellation</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>reservas.sonetabogota (typo)</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>reservas.sonestabogota@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Política y parqueo de bicis</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Gratuito para todos; sin parqueo de bicis</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Gratuito solo para huéspedes (invitados pagan tarifa); sí hay parqueo de bicis</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Balcón</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Todas las habitaciones tienen balcón</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Ninguna habitación tiene balcón; la suite tiene terraza</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Zonas restringidas</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>Lista extensa de zonas</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Zonas públicas, salas de conferencias, gimnasio, Porterhouse y Cook's</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Nombre y horario</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Cook's PorterHouse, 12:00-22:00 todos los días</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>PorterHouse, horario variable por día (hasta 22:00-22:30 según el día)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>17-11, 17-15</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Spa reservation / hours</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Nombre del servicio</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Spa / Tratamiento de Spa</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Sala de bienestar / Masaje; consultar disponibilidad por correo</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Nombre, horarios y política de niños</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Cook's Porterhouse (no acepta niños); Cook's 6:00-10:00</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Porterhouse (steak house, acepta niños, horario variable); Cook's 6:00-10:00 y 6:30-10:30 fines de semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>18-08</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Takeaway &amp; delivery</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Catering</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Se ofrecía catering</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>No hay catering; solo domicilios</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>18-26</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Valentine's day</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Enlace a oferta específica</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Información general de eventos de temporada</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>06:00 a 10:00</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>06:30 a 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Precio y correo</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Aeropuerto 26000 COP, Centro 28000 COP, recepcion.sonestapereira@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Aeropuerto 40000 COP, Centro 45000 COP, reservas.sonestapereira@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>06:00 a 22:00</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>06:30 a 22:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>10-13</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Opening, closing &amp; renovation</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Fechas y alcance de remodelación</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>01-JUL a 31-AGO</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>01-FEB a 31-OCT; incluye jacuzzi y piscina infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>10-42</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Day use reservation</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>31 de agosto</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>31 de octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Máximo de mascotas</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>2 mascotas por habitación</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>1 mascota por habitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>17-61</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Swimming pool</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>31 de agosto</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>31 de octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>13-45</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Change &amp; ATM</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Ubicación cajero más cercano</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Cra. 7 #25-2, a 6 min a pie</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Cra 8 Clle 19, a 2 min a pie</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Política de mascotas</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>No se aceptan ni animales de apoyo/servicio certificados</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Se aceptan animales de apoyo emocional pequeños con certificado médico y carné de vacunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>18-02, 18-03, 18-04</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Restaurant reservation/cancellation/modification</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>reservas.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>eventos.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>18-11</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Brunch</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Recomendación externa</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>MARDIWI (Pereira)</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira - Visus</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Teléfonos</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>+56 996795687 / +56 931909316</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Pago en efectivo</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>No se acepta efectivo en moneda local ni USD; disponible link de pago en pesos chilenos</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Verificar en correo (el hotel no envió el valor 'después')</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Horario y restaurante</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Lu-Sáb 06:00-10:00, Dom 06:00-10:30, Restaurante Entre Piedras</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>13-25</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Cribs</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Cuna</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Cuna gratis con previa reserva, sujeto a disponibilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>13-43</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Servicio regular/express</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Regular: entrega al día siguiente después de 13:00; Express: mismo día después de 19:30 (+50%); sin servicio en feriados</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>14-02</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Connecting rooms</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Verificar en correo — respuesta poco clara del hotel ('NO ENTENDI'), menciona connecting entre Queen y Junior Suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Room occupancy</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Ocupación máxima</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Queen: 2 adultos + 1 niño &lt;=6 años; Suite Especial: 4 adultos + 2 niños &lt;=6 años</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Horario de atención</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Lunes a domingo de 06:00 a 22:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Sala de ejercicios y dispensador de agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Floor arrangement &amp; elevator</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Ascensor y habitaciones por piso</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Verificar en correo (el hotel escribió '17-432', probable error de digitación)</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Sin ascensor; Queen 3/piso, Junior Suite 1/piso, Suite Especial 1/piso; total 15 habitaciones/torre</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>19-10</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Public transport tickets</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Venta de tickets</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>No se venden tickets de transporte público (Calama no tiene metro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>10-31</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Minimum stay</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Pases de un día</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Live Makani Adulto 280000 COP; Live MANA+Almuerzo 440000 COP; Live Makani ELUA X2 1160000 COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>11-31</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Front desk</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Horario recepción</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Abierta hasta las 5:00 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>3:00 pm a 5:00 pm; sin early check-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Parqueadero</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Sin parqueadero propio; el más cercano en el parque de la Marina</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>13-05</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Marina &amp; boat dock</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Horario de llegada en embarcación</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Hasta las 4:00 pm; barcos grandes requieren transbordo</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Tarifa infantil</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Gratis hasta 3 años; 450000 COP/noche de 3 a 11 años; sin club infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>13-41</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Concierge</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Horario y servicio</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>8:00 am a 10:00 pm, inglés y español, sin membresía Clefs d'Or</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>13-42</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Lost &amp; found</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>+57 318 335 6186; entrega en muelle de la Bodeguita</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>13-50</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Airport &amp; train station public transport</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Tiempo de traslado</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>20 min terrestre + 25 min marítimo desde el aeropuerto</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>16-15</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Social &amp; photoshoot</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>laura.molina@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>17-91</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Bloqueador, vestidos de baño, sombreros, bolsos, sandalias</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>20-02, 20-21, 20-22</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Business meeting / Celebration</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Salas de reunión y eventos</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Verificar en correo</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Sin salas de reuniones; eventos vía camila.dickens@ghlhoteles.com / eventos.makani@ghlhoteles.com</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:H227"/>

</xml_diff>

<commit_message>
Marcar como Actualizado los 10 hoteles con modificaciones de Sep-26
Los cambios reportados por Arsenal, Geotel Calama, GHL Relax Club Hotel
el Puente, GHL Relax Hotel Sunrise, GHL Style Yopal, GHL Hotel Abadía
Plaza, Makani Luxury Wanderlust, Sonesta Arequipa, Sonesta Bogotá y
Sonesta Pereira ya fueron aplicados en el chatbot (Velma). Se actualiza
estado, fecha y responsable en el HTML y en el Excel, y se agregan las
80 filas de detalle de Sep-26 que faltaban en la hoja "Modificaciones
detalle".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6931,9 +6931,14 @@
           <t>7 diálogos modificados: desayuno, tarifas, objetos perdidos, delivery, taxi, ascensor, teléfono de contacto</t>
         </is>
       </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K130" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7089,6 +7094,11 @@
           <t>11 diálogos modificados: contacto, pago, desayuno, cuna, lavandería, ocupación, horarios, gimnasio, ascensor, transporte</t>
         </is>
       </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="J134" t="inlineStr">
         <is>
           <t>Respuesta con formato informal — varios diálogos sin número claro o sin valor 'antes'; ver detalle. Diálogo 14-02 con respuesta poco clara ('NO ENTENDI')</t>
@@ -7096,7 +7106,7 @@
       </c>
       <c r="K134" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7457,9 +7467,14 @@
           <t>4 diálogos modificados: remodelación, day use, mascotas, piscina</t>
         </is>
       </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K143" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7588,9 +7603,14 @@
           <t>8 diálogos modificados: contacto, reservas, pago, day pass, check-in, desayuno, parqueadero, club infantil</t>
         </is>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K146" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7756,6 +7776,11 @@
           <t>7 diálogos modificados: método de pago, check-in, check-out, desayuno, mascotas, spa</t>
         </is>
       </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="J150" t="inlineStr">
         <is>
           <t>Reporta que los ajustes enviados en ciclos anteriores no se ven reflejados en el chatbot — verificar</t>
@@ -7763,7 +7788,7 @@
       </c>
       <c r="K150" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7845,9 +7870,14 @@
           <t>4 diálogos modificados: cajero, mascotas, reservas restaurante, brunch</t>
         </is>
       </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K152" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7976,6 +8006,11 @@
           <t>12 diálogos actualizados vía PDF adjunto: pases, recepción, check-in, parqueadero, muelle, niños, conserjería, objetos perdidos, transporte, eventos, boutique</t>
         </is>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="J155" t="inlineStr">
         <is>
           <t>Correcciones enviadas solo en PDF adjunto, sin texto antes/después en el cuerpo del correo — valores 'antes' marcados como Verificar en correo</t>
@@ -7983,7 +8018,7 @@
       </c>
       <c r="K155" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8307,9 +8342,14 @@
           <t>9 diálogos modificados: lavandería, fumadores, baño, cama extra, empleo, propinas, reservas restaurante, spa, restaurante</t>
         </is>
       </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K163" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8354,9 +8394,14 @@
           <t>13 diálogos modificados: clasificación, fumadores, baño, cama extra, contacto, parqueadero, balcón, mascotas, bar, spa, restaurante, delivery, San Valentín</t>
         </is>
       </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K164" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8512,9 +8557,14 @@
           <t>3 diálogos modificados: desayuno, taxi, restaurante</t>
         </is>
       </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
       <c r="K168" s="46" t="inlineStr">
         <is>
-          <t>Pendiente actualización</t>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8862,7 +8912,7 @@
         <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -9173,7 +9223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H508"/>
+  <dimension ref="A1:H588"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27965,6 +28015,2966 @@
       <c r="F508" t="inlineStr">
         <is>
           <t>Sin salas de reuniones; eventos vía camila.dickens@ghlhoteles.com / eventos.makani@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Nombre del restaurante</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Restaurante Corozo &amp; Timbal</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>Restaurante Úrsula; se agrega opción Room Service</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Precio adulto</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>65000 COP</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>80000 COP visitantes / 60000 COP huéspedes sin desayuno incluido</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>13-42</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Lost &amp; found</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Correo y teléfono</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>Solo correo (se retira teléfono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>13-46</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Política de entregas</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Solo hasta 10 KG</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>Se aceptan entregas de todas las plataformas; se agrega correo de contacto</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Precio y tiempo</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Aeropuerto 20000 COP/17min, Hotel 25000 COP/20min</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Aeropuerto-Hotel desde 25000 COP/17min, Hotel-Aeropuerto desde 25000 COP/20min</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Floor arrangement &amp; elevator</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Accesibilidad ascensor</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>No accesible para sillas de ruedas</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>Accesible para sillas de ruedas</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>14-04, 15-26, 15-61, 15-62, 15-99, 16-03, 17-44</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>+57 (605) 660 5831</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>+57 316 0107651</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Teléfonos</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>+56 996795687 / +56 931909316</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Pago en efectivo</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>No se acepta efectivo en moneda local ni USD; disponible link de pago en pesos chilenos</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo (el hotel no envió el valor 'después')</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Horario y restaurante</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>Lu-Sáb 06:00-10:00, Dom 06:00-10:30, Restaurante Entre Piedras</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>13-25</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Cribs</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Cuna</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>Cuna gratis con previa reserva, sujeto a disponibilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>13-43</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Servicio regular/express</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>Regular: entrega al día siguiente después de 13:00; Express: mismo día después de 19:30 (+50%); sin servicio en feriados</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>14-02</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Connecting rooms</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo — respuesta poco clara del hotel ('NO ENTENDI'), menciona connecting entre Queen y Junior Suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Room occupancy</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Ocupación máxima</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>Queen: 2 adultos + 1 niño ≤6 años; Suite Especial: 4 adultos + 2 niños ≤6 años</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Horario de atención</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>Lunes a domingo de 06:00 a 22:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>17-31</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Fitness gym</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>Sala de ejercicios y dispensador de agua</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>17-43</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Floor arrangement &amp; elevator</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Ascensor y habitaciones por piso</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo (el hotel escribió '17-432', probable error de digitación)</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>Sin ascensor; Queen 3/piso, Junior Suite 1/piso, Suite Especial 1/piso; total 15 habitaciones/torre</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>19-10</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Public transport tickets</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Venta de tickets</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>No se venden tickets de transporte público (Calama no tiene metro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>10-13</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Opening, closing &amp; renovation</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Fechas y alcance de remodelación</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>01-JUL a 31-AGO</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
+          <t>01-FEB a 31-OCT; incluye jacuzzi y piscina infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>10-42</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Day use reservation</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>31 de agosto</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>31 de octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Máximo de mascotas</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>2 mascotas por habitación</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>1 mascota por habitación</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>17-61</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Swimming pool</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Fecha fin remodelación</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>31 de agosto</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>31 de octubre</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Teléfonos</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Sin línea gratuita</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>Se agregan teléfonos gratuitos de recepción y eventos</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>10-04, 10-06</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Reservation modification/cancellation</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Correo y teléfono</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>reservas2.sunrise sin línea gratuita</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>reservas2.sunrise@ghlhoteles.com + teléfono gratuito 3175387071</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Transferencias</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>No mencionadas</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>Se agrega transferencia a cuenta bancaria del hotel y Wompi</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>10-41</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Day use / day pass</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Edad tarifa infantil</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Sin rango de edad</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>Niños de 3 a 11 años</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Early check-in</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>Sin condición</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>Sujeto a disponibilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>07:00 a 10:00, sin especificar tipo</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>Buffet de 07:00 a 10:00 en restaurante</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Parqueadero cercano</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>Sin recomendación</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>Se agrega parqueadero Aeropuerto como opción cercana</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Club infantil</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>Sin días/horario</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>Lu, Mar, Mié, Jue, Vie y Sáb de 13:00 a 21:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Métodos de pago</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>Sin Visa; no se acepta efectivo</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>Se agrega Visa; se acepta pago en efectivo en recepción</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Early check-in</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>70000 COP</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>11-11</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Check-out time</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>70000 COP</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>Horario y servicio a la habitación</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>06:00-10:00 todos los días; sin room service</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>Lu-Sáb 06:00-10:00, Dom/fest 06:00-10:30; se ofrece con cargo adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>12-02</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Breakfast rates</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>Precio adulto</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>48000 COP</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>40000 COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>Tasa mascota</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>70000 COP/mascota</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>70000 COP + IVA/mascota</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Spa hours</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>Horario de spa sin restricciones</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>Ya no cuentan con spa</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>13-45</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Change &amp; ATM</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>Ubicación cajero más cercano</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>Cra. 7 #25-2, a 6 min a pie</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>Cra 8 Clle 19, a 2 min a pie</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>Política de mascotas</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>No se aceptan ni animales de apoyo/servicio certificados</t>
+        </is>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>Se aceptan animales de apoyo emocional pequeños con certificado médico y carné de vacunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>18-02, 18-03, 18-04</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>Restaurant reservation/cancellation/modification</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>reservas.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G549" t="inlineStr">
+        <is>
+          <t>eventos.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>18-11</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Brunch</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>Recomendación externa</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>MARDIWI (Pereira)</t>
+        </is>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira - Visus</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>10-31</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Minimum stay</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>Pases de un día</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>Live Makani Adulto 280000 COP; Live MANA+Almuerzo 440000 COP; Live Makani ELUA X2 1160000 COP</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>11-31</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Front desk</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>Horario recepción</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>Abierta hasta las 5:00 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>11-01</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Check-in time</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>3:00 pm a 5:00 pm; sin early check-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>Parqueadero</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>Sin parqueadero propio; el más cercano en el parque de la Marina</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>13-05</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Marina &amp; boat dock</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>Horario de llegada en embarcación</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>Hasta las 4:00 pm; barcos grandes requieren transbordo</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>13-21</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Kids</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>Tarifa infantil</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>Gratis hasta 3 años; 450000 COP/noche de 3 a 11 años; sin club infantil</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>13-41</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Concierge</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>Horario y servicio</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>8:00 am a 10:00 pm, inglés y español, sin membresía Clefs d'Or</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>13-42</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Lost &amp; found</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>+57 318 335 6186; entrega en muelle de la Bodeguita</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>13-50</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Airport &amp; train station public transport</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>Tiempo de traslado</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>20 min terrestre + 25 min marítimo desde el aeropuerto</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>16-15</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Social &amp; photoshoot</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>Contacto</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>laura.molina@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>17-91</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Boutique</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>Productos</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Bloqueador, vestidos de baño, sombreros, bolsos, sandalias</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>20-02, 20-21, 20-22</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Business meeting / Celebration</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>Salas de reunión y eventos</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>Sin salas de reuniones; eventos vía camila.dickens@ghlhoteles.com / eventos.makani@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>13-43</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>Tiempo de entrega</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>Se devuelve antes de las 10:00</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Se devuelve el mismo día</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Tarifa limpieza por humo</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>700 PEN</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>USD 200.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>Artículos gratis a petición</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>Pantuflas, pasta de dientes, kit de afeitar</t>
+        </is>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>Pantuflas, kit dental, kit de afeitar, costurero, limpia calzados y peine</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>15-24, 15-99</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Extra bed / Specific room request</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>Correo de contacto</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>Incluía calidad.sonestaarequipa</t>
+        </is>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>Solo reservas.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>16-06</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Jobs &amp; internships</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Contacto RRHH</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>contactenos@ghlhoteles.com / +57 601 3139330</t>
+        </is>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>laydy.pauca@ghlhoteles.com / +51 054 308 777</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>16-25</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Tips policy</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>Política de propinas</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>Incluía la línea 'es costumbre dejar propina'</t>
+        </is>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Se elimina esa línea</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>17-02, 18-02, 18-03, 18-04</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Reservas restaurante/bar</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>Teléfono de contacto</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>Solo correo</t>
+        </is>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Se agrega +51 945 739 921</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>17-10</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Spa</t>
+        </is>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>Política de acceso</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>Abierto solo clientes; edad mínima 12 años</t>
+        </is>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Menores de 12 solo con padres/tutor; masajes con costo adicional</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>Descripción restaurante Micaela</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>Incluía capacidad, política de niños y tronas</t>
+        </is>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>Descripción simplificada (se retira info de capacidad y niños)</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Clasificación del hotel</t>
+        </is>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>Estrellas</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>5 estrellas</t>
+        </is>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>4 estrellas</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>14-04</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Smoking</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>Detectores de humo</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>Las habitaciones no están equipadas con detectores de humo</t>
+        </is>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>Las habitaciones están equipadas con detectores de humo</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>15-06</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Bathroom equipment</t>
+        </is>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>Artículos gratis / no disponibles</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>Lista distinta</t>
+        </is>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>Se agregan albornoz, pantuflas, gel de ducha, hisopos, cepillo y pasta de dientes; se recorta lista de no disponibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>Precio cama extra</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>110000 COP/noche</t>
+        </is>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>Se elimina el precio; solo se indica correo de solicitud</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>16-02</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>Teléfono gratuito</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>+57 3052281127 (recepción, reserva y eventos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>10-04, 10-06</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Reservation modification/cancellation</t>
+        </is>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>reservas.sonetabogota (typo)</t>
+        </is>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>reservas.sonestabogota@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>13-01</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>Política y parqueo de bicis</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>Gratuito para todos; sin parqueo de bicis</t>
+        </is>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>Gratuito solo para huéspedes (invitados pagan tarifa); sí hay parqueo de bicis</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>15-61</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Balcony &amp; windows</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>Balcón</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>Todas las habitaciones tienen balcón</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>Ninguna habitación tiene balcón; la suite tiene terraza</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>Zonas restringidas</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>Lista extensa de zonas</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>Zonas públicas, salas de conferencias, gimnasio, Porterhouse y Cook's</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>Nombre y horario</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>Cook's PorterHouse, 12:00-22:00 todos los días</t>
+        </is>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>PorterHouse, horario variable por día (hasta 22:00-22:30 según el día)</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>17-11, 17-15</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Spa reservation / hours</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>Nombre del servicio</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>Spa / Tratamiento de Spa</t>
+        </is>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>Sala de bienestar / Masaje; consultar disponibilidad por correo</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>Nombre, horarios y política de niños</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>Cook's Porterhouse (no acepta niños); Cook's 6:00-10:00</t>
+        </is>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>Porterhouse (steak house, acepta niños, horario variable); Cook's 6:00-10:00 y 6:30-10:30 fines de semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>18-08</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Takeaway &amp; delivery</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>Catering</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>Se ofrecía catering</t>
+        </is>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>No hay catering; solo domicilios</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>18-26</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Valentine's day</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>Enlace a oferta específica</t>
+        </is>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>Información general de eventos de temporada</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>12-01</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Breakfast time</t>
+        </is>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>06:00 a 10:00</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>06:30 a 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>13-53</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>Precio y correo</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>Aeropuerto 26000 COP, Centro 28000 COP, recepcion.sonestapereira@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>Aeropuerto 40000 COP, Centro 45000 COP, reservas.sonestapereira@ghlhoteles.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>18-01</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Restaurant</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Horario</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>06:00 a 22:00</t>
+        </is>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>06:30 a 22:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Marcar como Actualizado los 10 hoteles con modificaciones de Sep-26"
This reverts commit 4be13d890da52c781f59f8d991cf4603a762c04a.
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6931,14 +6931,9 @@
           <t>7 diálogos modificados: desayuno, tarifas, objetos perdidos, delivery, taxi, ascensor, teléfono de contacto</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K130" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7094,11 +7089,6 @@
           <t>11 diálogos modificados: contacto, pago, desayuno, cuna, lavandería, ocupación, horarios, gimnasio, ascensor, transporte</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="J134" t="inlineStr">
         <is>
           <t>Respuesta con formato informal — varios diálogos sin número claro o sin valor 'antes'; ver detalle. Diálogo 14-02 con respuesta poco clara ('NO ENTENDI')</t>
@@ -7106,7 +7096,7 @@
       </c>
       <c r="K134" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7467,14 +7457,9 @@
           <t>4 diálogos modificados: remodelación, day use, mascotas, piscina</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K143" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7603,14 +7588,9 @@
           <t>8 diálogos modificados: contacto, reservas, pago, day pass, check-in, desayuno, parqueadero, club infantil</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K146" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7776,11 +7756,6 @@
           <t>7 diálogos modificados: método de pago, check-in, check-out, desayuno, mascotas, spa</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="J150" t="inlineStr">
         <is>
           <t>Reporta que los ajustes enviados en ciclos anteriores no se ven reflejados en el chatbot — verificar</t>
@@ -7788,7 +7763,7 @@
       </c>
       <c r="K150" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -7870,14 +7845,9 @@
           <t>4 diálogos modificados: cajero, mascotas, reservas restaurante, brunch</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K152" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8006,11 +7976,6 @@
           <t>12 diálogos actualizados vía PDF adjunto: pases, recepción, check-in, parqueadero, muelle, niños, conserjería, objetos perdidos, transporte, eventos, boutique</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="J155" t="inlineStr">
         <is>
           <t>Correcciones enviadas solo en PDF adjunto, sin texto antes/después en el cuerpo del correo — valores 'antes' marcados como Verificar en correo</t>
@@ -8018,7 +7983,7 @@
       </c>
       <c r="K155" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8342,14 +8307,9 @@
           <t>9 diálogos modificados: lavandería, fumadores, baño, cama extra, empleo, propinas, reservas restaurante, spa, restaurante</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K163" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8394,14 +8354,9 @@
           <t>13 diálogos modificados: clasificación, fumadores, baño, cama extra, contacto, parqueadero, balcón, mascotas, bar, spa, restaurante, delivery, San Valentín</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K164" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8557,14 +8512,9 @@
           <t>3 diálogos modificados: desayuno, taxi, restaurante</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
       <c r="K168" s="46" t="inlineStr">
         <is>
-          <t>Actualizado</t>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8862,7 @@
         <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -9223,7 +9173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H588"/>
+  <dimension ref="A1:H508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28015,2966 +27965,6 @@
       <c r="F508" t="inlineStr">
         <is>
           <t>Sin salas de reuniones; eventos vía camila.dickens@ghlhoteles.com / eventos.makani@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="509">
-      <c r="A509" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B509" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C509" t="inlineStr">
-        <is>
-          <t>12-01</t>
-        </is>
-      </c>
-      <c r="D509" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E509" t="inlineStr">
-        <is>
-          <t>Nombre del restaurante</t>
-        </is>
-      </c>
-      <c r="F509" t="inlineStr">
-        <is>
-          <t>Restaurante Corozo &amp; Timbal</t>
-        </is>
-      </c>
-      <c r="G509" t="inlineStr">
-        <is>
-          <t>Restaurante Úrsula; se agrega opción Room Service</t>
-        </is>
-      </c>
-    </row>
-    <row r="510">
-      <c r="A510" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B510" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C510" t="inlineStr">
-        <is>
-          <t>12-02</t>
-        </is>
-      </c>
-      <c r="D510" t="inlineStr">
-        <is>
-          <t>Breakfast rates</t>
-        </is>
-      </c>
-      <c r="E510" t="inlineStr">
-        <is>
-          <t>Precio adulto</t>
-        </is>
-      </c>
-      <c r="F510" t="inlineStr">
-        <is>
-          <t>65000 COP</t>
-        </is>
-      </c>
-      <c r="G510" t="inlineStr">
-        <is>
-          <t>80000 COP visitantes / 60000 COP huéspedes sin desayuno incluido</t>
-        </is>
-      </c>
-    </row>
-    <row r="511">
-      <c r="A511" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B511" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C511" t="inlineStr">
-        <is>
-          <t>13-42</t>
-        </is>
-      </c>
-      <c r="D511" t="inlineStr">
-        <is>
-          <t>Lost &amp; found</t>
-        </is>
-      </c>
-      <c r="E511" t="inlineStr">
-        <is>
-          <t>Contacto</t>
-        </is>
-      </c>
-      <c r="F511" t="inlineStr">
-        <is>
-          <t>Correo y teléfono</t>
-        </is>
-      </c>
-      <c r="G511" t="inlineStr">
-        <is>
-          <t>Solo correo (se retira teléfono)</t>
-        </is>
-      </c>
-    </row>
-    <row r="512">
-      <c r="A512" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B512" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C512" t="inlineStr">
-        <is>
-          <t>13-46</t>
-        </is>
-      </c>
-      <c r="D512" t="inlineStr">
-        <is>
-          <t>Delivery</t>
-        </is>
-      </c>
-      <c r="E512" t="inlineStr">
-        <is>
-          <t>Política de entregas</t>
-        </is>
-      </c>
-      <c r="F512" t="inlineStr">
-        <is>
-          <t>Solo hasta 10 KG</t>
-        </is>
-      </c>
-      <c r="G512" t="inlineStr">
-        <is>
-          <t>Se aceptan entregas de todas las plataformas; se agrega correo de contacto</t>
-        </is>
-      </c>
-    </row>
-    <row r="513">
-      <c r="A513" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B513" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C513" t="inlineStr">
-        <is>
-          <t>13-53</t>
-        </is>
-      </c>
-      <c r="D513" t="inlineStr">
-        <is>
-          <t>Taxi</t>
-        </is>
-      </c>
-      <c r="E513" t="inlineStr">
-        <is>
-          <t>Precio y tiempo</t>
-        </is>
-      </c>
-      <c r="F513" t="inlineStr">
-        <is>
-          <t>Aeropuerto 20000 COP/17min, Hotel 25000 COP/20min</t>
-        </is>
-      </c>
-      <c r="G513" t="inlineStr">
-        <is>
-          <t>Aeropuerto-Hotel desde 25000 COP/17min, Hotel-Aeropuerto desde 25000 COP/20min</t>
-        </is>
-      </c>
-    </row>
-    <row r="514">
-      <c r="A514" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B514" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C514" t="inlineStr">
-        <is>
-          <t>17-43</t>
-        </is>
-      </c>
-      <c r="D514" t="inlineStr">
-        <is>
-          <t>Floor arrangement &amp; elevator</t>
-        </is>
-      </c>
-      <c r="E514" t="inlineStr">
-        <is>
-          <t>Accesibilidad ascensor</t>
-        </is>
-      </c>
-      <c r="F514" t="inlineStr">
-        <is>
-          <t>No accesible para sillas de ruedas</t>
-        </is>
-      </c>
-      <c r="G514" t="inlineStr">
-        <is>
-          <t>Accesible para sillas de ruedas</t>
-        </is>
-      </c>
-    </row>
-    <row r="515">
-      <c r="A515" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B515" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="C515" t="inlineStr">
-        <is>
-          <t>14-04, 15-26, 15-61, 15-62, 15-99, 16-03, 17-44</t>
-        </is>
-      </c>
-      <c r="D515" t="inlineStr">
-        <is>
-          <t>Varios</t>
-        </is>
-      </c>
-      <c r="E515" t="inlineStr">
-        <is>
-          <t>Teléfono de contacto</t>
-        </is>
-      </c>
-      <c r="F515" t="inlineStr">
-        <is>
-          <t>+57 (605) 660 5831</t>
-        </is>
-      </c>
-      <c r="G515" t="inlineStr">
-        <is>
-          <t>+57 316 0107651</t>
-        </is>
-      </c>
-    </row>
-    <row r="516">
-      <c r="A516" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B516" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C516" t="inlineStr">
-        <is>
-          <t>16-02</t>
-        </is>
-      </c>
-      <c r="D516" t="inlineStr">
-        <is>
-          <t>Contact staff</t>
-        </is>
-      </c>
-      <c r="E516" t="inlineStr">
-        <is>
-          <t>Teléfonos</t>
-        </is>
-      </c>
-      <c r="F516" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G516" t="inlineStr">
-        <is>
-          <t>+56 996795687 / +56 931909316</t>
-        </is>
-      </c>
-    </row>
-    <row r="517">
-      <c r="A517" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B517" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C517" t="inlineStr">
-        <is>
-          <t>10-71</t>
-        </is>
-      </c>
-      <c r="D517" t="inlineStr">
-        <is>
-          <t>Payment method</t>
-        </is>
-      </c>
-      <c r="E517" t="inlineStr">
-        <is>
-          <t>Pago en efectivo</t>
-        </is>
-      </c>
-      <c r="F517" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G517" t="inlineStr">
-        <is>
-          <t>No se acepta efectivo en moneda local ni USD; disponible link de pago en pesos chilenos</t>
-        </is>
-      </c>
-    </row>
-    <row r="518">
-      <c r="A518" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B518" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C518" t="inlineStr">
-        <is>
-          <t>11-11</t>
-        </is>
-      </c>
-      <c r="D518" t="inlineStr">
-        <is>
-          <t>Check-out time</t>
-        </is>
-      </c>
-      <c r="E518" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F518" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G518" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo (el hotel no envió el valor 'después')</t>
-        </is>
-      </c>
-    </row>
-    <row r="519">
-      <c r="A519" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B519" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C519" t="inlineStr">
-        <is>
-          <t>12-01</t>
-        </is>
-      </c>
-      <c r="D519" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E519" t="inlineStr">
-        <is>
-          <t>Horario y restaurante</t>
-        </is>
-      </c>
-      <c r="F519" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G519" t="inlineStr">
-        <is>
-          <t>Lu-Sáb 06:00-10:00, Dom 06:00-10:30, Restaurante Entre Piedras</t>
-        </is>
-      </c>
-    </row>
-    <row r="520">
-      <c r="A520" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B520" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C520" t="inlineStr">
-        <is>
-          <t>13-25</t>
-        </is>
-      </c>
-      <c r="D520" t="inlineStr">
-        <is>
-          <t>Cribs</t>
-        </is>
-      </c>
-      <c r="E520" t="inlineStr">
-        <is>
-          <t>Cuna</t>
-        </is>
-      </c>
-      <c r="F520" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G520" t="inlineStr">
-        <is>
-          <t>Cuna gratis con previa reserva, sujeto a disponibilidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="521">
-      <c r="A521" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B521" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C521" t="inlineStr">
-        <is>
-          <t>13-43</t>
-        </is>
-      </c>
-      <c r="D521" t="inlineStr">
-        <is>
-          <t>Laundry</t>
-        </is>
-      </c>
-      <c r="E521" t="inlineStr">
-        <is>
-          <t>Servicio regular/express</t>
-        </is>
-      </c>
-      <c r="F521" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G521" t="inlineStr">
-        <is>
-          <t>Regular: entrega al día siguiente después de 13:00; Express: mismo día después de 19:30 (+50%); sin servicio en feriados</t>
-        </is>
-      </c>
-    </row>
-    <row r="522">
-      <c r="A522" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B522" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C522" t="inlineStr">
-        <is>
-          <t>14-02</t>
-        </is>
-      </c>
-      <c r="D522" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E522" t="inlineStr">
-        <is>
-          <t>Connecting rooms</t>
-        </is>
-      </c>
-      <c r="F522" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G522" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo — respuesta poco clara del hotel ('NO ENTENDI'), menciona connecting entre Queen y Junior Suite</t>
-        </is>
-      </c>
-    </row>
-    <row r="523">
-      <c r="A523" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B523" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C523" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D523" t="inlineStr">
-        <is>
-          <t>Room occupancy</t>
-        </is>
-      </c>
-      <c r="E523" t="inlineStr">
-        <is>
-          <t>Ocupación máxima</t>
-        </is>
-      </c>
-      <c r="F523" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G523" t="inlineStr">
-        <is>
-          <t>Queen: 2 adultos + 1 niño ≤6 años; Suite Especial: 4 adultos + 2 niños ≤6 años</t>
-        </is>
-      </c>
-    </row>
-    <row r="524">
-      <c r="A524" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B524" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C524" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D524" t="inlineStr">
-        <is>
-          <t>Horario</t>
-        </is>
-      </c>
-      <c r="E524" t="inlineStr">
-        <is>
-          <t>Horario de atención</t>
-        </is>
-      </c>
-      <c r="F524" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G524" t="inlineStr">
-        <is>
-          <t>Lunes a domingo de 06:00 a 22:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="525">
-      <c r="A525" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B525" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C525" t="inlineStr">
-        <is>
-          <t>17-31</t>
-        </is>
-      </c>
-      <c r="D525" t="inlineStr">
-        <is>
-          <t>Fitness gym</t>
-        </is>
-      </c>
-      <c r="E525" t="inlineStr">
-        <is>
-          <t>Equipamiento</t>
-        </is>
-      </c>
-      <c r="F525" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G525" t="inlineStr">
-        <is>
-          <t>Sala de ejercicios y dispensador de agua</t>
-        </is>
-      </c>
-    </row>
-    <row r="526">
-      <c r="A526" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B526" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C526" t="inlineStr">
-        <is>
-          <t>17-43</t>
-        </is>
-      </c>
-      <c r="D526" t="inlineStr">
-        <is>
-          <t>Floor arrangement &amp; elevator</t>
-        </is>
-      </c>
-      <c r="E526" t="inlineStr">
-        <is>
-          <t>Ascensor y habitaciones por piso</t>
-        </is>
-      </c>
-      <c r="F526" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo (el hotel escribió '17-432', probable error de digitación)</t>
-        </is>
-      </c>
-      <c r="G526" t="inlineStr">
-        <is>
-          <t>Sin ascensor; Queen 3/piso, Junior Suite 1/piso, Suite Especial 1/piso; total 15 habitaciones/torre</t>
-        </is>
-      </c>
-    </row>
-    <row r="527">
-      <c r="A527" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B527" t="inlineStr">
-        <is>
-          <t>Geotel Calama</t>
-        </is>
-      </c>
-      <c r="C527" t="inlineStr">
-        <is>
-          <t>19-10</t>
-        </is>
-      </c>
-      <c r="D527" t="inlineStr">
-        <is>
-          <t>Public transport tickets</t>
-        </is>
-      </c>
-      <c r="E527" t="inlineStr">
-        <is>
-          <t>Venta de tickets</t>
-        </is>
-      </c>
-      <c r="F527" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G527" t="inlineStr">
-        <is>
-          <t>No se venden tickets de transporte público (Calama no tiene metro)</t>
-        </is>
-      </c>
-    </row>
-    <row r="528">
-      <c r="A528" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B528" t="inlineStr">
-        <is>
-          <t>GHL Relax Club Hotel el Puente</t>
-        </is>
-      </c>
-      <c r="C528" t="inlineStr">
-        <is>
-          <t>10-13</t>
-        </is>
-      </c>
-      <c r="D528" t="inlineStr">
-        <is>
-          <t>Opening, closing &amp; renovation</t>
-        </is>
-      </c>
-      <c r="E528" t="inlineStr">
-        <is>
-          <t>Fechas y alcance de remodelación</t>
-        </is>
-      </c>
-      <c r="F528" t="inlineStr">
-        <is>
-          <t>01-JUL a 31-AGO</t>
-        </is>
-      </c>
-      <c r="G528" t="inlineStr">
-        <is>
-          <t>01-FEB a 31-OCT; incluye jacuzzi y piscina infantil</t>
-        </is>
-      </c>
-    </row>
-    <row r="529">
-      <c r="A529" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B529" t="inlineStr">
-        <is>
-          <t>GHL Relax Club Hotel el Puente</t>
-        </is>
-      </c>
-      <c r="C529" t="inlineStr">
-        <is>
-          <t>10-42</t>
-        </is>
-      </c>
-      <c r="D529" t="inlineStr">
-        <is>
-          <t>Day use reservation</t>
-        </is>
-      </c>
-      <c r="E529" t="inlineStr">
-        <is>
-          <t>Fecha fin remodelación</t>
-        </is>
-      </c>
-      <c r="F529" t="inlineStr">
-        <is>
-          <t>31 de agosto</t>
-        </is>
-      </c>
-      <c r="G529" t="inlineStr">
-        <is>
-          <t>31 de octubre</t>
-        </is>
-      </c>
-    </row>
-    <row r="530">
-      <c r="A530" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B530" t="inlineStr">
-        <is>
-          <t>GHL Relax Club Hotel el Puente</t>
-        </is>
-      </c>
-      <c r="C530" t="inlineStr">
-        <is>
-          <t>16-10</t>
-        </is>
-      </c>
-      <c r="D530" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="E530" t="inlineStr">
-        <is>
-          <t>Máximo de mascotas</t>
-        </is>
-      </c>
-      <c r="F530" t="inlineStr">
-        <is>
-          <t>2 mascotas por habitación</t>
-        </is>
-      </c>
-      <c r="G530" t="inlineStr">
-        <is>
-          <t>1 mascota por habitación</t>
-        </is>
-      </c>
-    </row>
-    <row r="531">
-      <c r="A531" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B531" t="inlineStr">
-        <is>
-          <t>GHL Relax Club Hotel el Puente</t>
-        </is>
-      </c>
-      <c r="C531" t="inlineStr">
-        <is>
-          <t>17-61</t>
-        </is>
-      </c>
-      <c r="D531" t="inlineStr">
-        <is>
-          <t>Swimming pool</t>
-        </is>
-      </c>
-      <c r="E531" t="inlineStr">
-        <is>
-          <t>Fecha fin remodelación</t>
-        </is>
-      </c>
-      <c r="F531" t="inlineStr">
-        <is>
-          <t>31 de agosto</t>
-        </is>
-      </c>
-      <c r="G531" t="inlineStr">
-        <is>
-          <t>31 de octubre</t>
-        </is>
-      </c>
-    </row>
-    <row r="532">
-      <c r="A532" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B532" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C532" t="inlineStr">
-        <is>
-          <t>16-02</t>
-        </is>
-      </c>
-      <c r="D532" t="inlineStr">
-        <is>
-          <t>Contact staff</t>
-        </is>
-      </c>
-      <c r="E532" t="inlineStr">
-        <is>
-          <t>Teléfonos</t>
-        </is>
-      </c>
-      <c r="F532" t="inlineStr">
-        <is>
-          <t>Sin línea gratuita</t>
-        </is>
-      </c>
-      <c r="G532" t="inlineStr">
-        <is>
-          <t>Se agregan teléfonos gratuitos de recepción y eventos</t>
-        </is>
-      </c>
-    </row>
-    <row r="533">
-      <c r="A533" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B533" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C533" t="inlineStr">
-        <is>
-          <t>10-04, 10-06</t>
-        </is>
-      </c>
-      <c r="D533" t="inlineStr">
-        <is>
-          <t>Reservation modification/cancellation</t>
-        </is>
-      </c>
-      <c r="E533" t="inlineStr">
-        <is>
-          <t>Correo y teléfono</t>
-        </is>
-      </c>
-      <c r="F533" t="inlineStr">
-        <is>
-          <t>reservas2.sunrise sin línea gratuita</t>
-        </is>
-      </c>
-      <c r="G533" t="inlineStr">
-        <is>
-          <t>reservas2.sunrise@ghlhoteles.com + teléfono gratuito 3175387071</t>
-        </is>
-      </c>
-    </row>
-    <row r="534">
-      <c r="A534" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B534" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C534" t="inlineStr">
-        <is>
-          <t>10-71</t>
-        </is>
-      </c>
-      <c r="D534" t="inlineStr">
-        <is>
-          <t>Payment method</t>
-        </is>
-      </c>
-      <c r="E534" t="inlineStr">
-        <is>
-          <t>Transferencias</t>
-        </is>
-      </c>
-      <c r="F534" t="inlineStr">
-        <is>
-          <t>No mencionadas</t>
-        </is>
-      </c>
-      <c r="G534" t="inlineStr">
-        <is>
-          <t>Se agrega transferencia a cuenta bancaria del hotel y Wompi</t>
-        </is>
-      </c>
-    </row>
-    <row r="535">
-      <c r="A535" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C535" t="inlineStr">
-        <is>
-          <t>10-41</t>
-        </is>
-      </c>
-      <c r="D535" t="inlineStr">
-        <is>
-          <t>Day use / day pass</t>
-        </is>
-      </c>
-      <c r="E535" t="inlineStr">
-        <is>
-          <t>Edad tarifa infantil</t>
-        </is>
-      </c>
-      <c r="F535" t="inlineStr">
-        <is>
-          <t>Sin rango de edad</t>
-        </is>
-      </c>
-      <c r="G535" t="inlineStr">
-        <is>
-          <t>Niños de 3 a 11 años</t>
-        </is>
-      </c>
-    </row>
-    <row r="536">
-      <c r="A536" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B536" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C536" t="inlineStr">
-        <is>
-          <t>11-01</t>
-        </is>
-      </c>
-      <c r="D536" t="inlineStr">
-        <is>
-          <t>Check-in time</t>
-        </is>
-      </c>
-      <c r="E536" t="inlineStr">
-        <is>
-          <t>Early check-in</t>
-        </is>
-      </c>
-      <c r="F536" t="inlineStr">
-        <is>
-          <t>Sin condición</t>
-        </is>
-      </c>
-      <c r="G536" t="inlineStr">
-        <is>
-          <t>Sujeto a disponibilidad</t>
-        </is>
-      </c>
-    </row>
-    <row r="537">
-      <c r="A537" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B537" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C537" t="inlineStr">
-        <is>
-          <t>12-01</t>
-        </is>
-      </c>
-      <c r="D537" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E537" t="inlineStr">
-        <is>
-          <t>Horario</t>
-        </is>
-      </c>
-      <c r="F537" t="inlineStr">
-        <is>
-          <t>07:00 a 10:00, sin especificar tipo</t>
-        </is>
-      </c>
-      <c r="G537" t="inlineStr">
-        <is>
-          <t>Buffet de 07:00 a 10:00 en restaurante</t>
-        </is>
-      </c>
-    </row>
-    <row r="538">
-      <c r="A538" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B538" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C538" t="inlineStr">
-        <is>
-          <t>13-01</t>
-        </is>
-      </c>
-      <c r="D538" t="inlineStr">
-        <is>
-          <t>Parking</t>
-        </is>
-      </c>
-      <c r="E538" t="inlineStr">
-        <is>
-          <t>Parqueadero cercano</t>
-        </is>
-      </c>
-      <c r="F538" t="inlineStr">
-        <is>
-          <t>Sin recomendación</t>
-        </is>
-      </c>
-      <c r="G538" t="inlineStr">
-        <is>
-          <t>Se agrega parqueadero Aeropuerto como opción cercana</t>
-        </is>
-      </c>
-    </row>
-    <row r="539">
-      <c r="A539" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B539" t="inlineStr">
-        <is>
-          <t>GHL Relax Hotel Sunrise</t>
-        </is>
-      </c>
-      <c r="C539" t="inlineStr">
-        <is>
-          <t>13-21</t>
-        </is>
-      </c>
-      <c r="D539" t="inlineStr">
-        <is>
-          <t>Kids</t>
-        </is>
-      </c>
-      <c r="E539" t="inlineStr">
-        <is>
-          <t>Club infantil</t>
-        </is>
-      </c>
-      <c r="F539" t="inlineStr">
-        <is>
-          <t>Sin días/horario</t>
-        </is>
-      </c>
-      <c r="G539" t="inlineStr">
-        <is>
-          <t>Lu, Mar, Mié, Jue, Vie y Sáb de 13:00 a 21:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="540">
-      <c r="A540" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B540" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C540" t="inlineStr">
-        <is>
-          <t>10-71</t>
-        </is>
-      </c>
-      <c r="D540" t="inlineStr">
-        <is>
-          <t>Payment method</t>
-        </is>
-      </c>
-      <c r="E540" t="inlineStr">
-        <is>
-          <t>Métodos de pago</t>
-        </is>
-      </c>
-      <c r="F540" t="inlineStr">
-        <is>
-          <t>Sin Visa; no se acepta efectivo</t>
-        </is>
-      </c>
-      <c r="G540" t="inlineStr">
-        <is>
-          <t>Se agrega Visa; se acepta pago en efectivo en recepción</t>
-        </is>
-      </c>
-    </row>
-    <row r="541">
-      <c r="A541" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B541" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C541" t="inlineStr">
-        <is>
-          <t>11-01</t>
-        </is>
-      </c>
-      <c r="D541" t="inlineStr">
-        <is>
-          <t>Check-in time</t>
-        </is>
-      </c>
-      <c r="E541" t="inlineStr">
-        <is>
-          <t>Early check-in</t>
-        </is>
-      </c>
-      <c r="F541" t="inlineStr">
-        <is>
-          <t>70000 COP</t>
-        </is>
-      </c>
-      <c r="G541" t="inlineStr">
-        <is>
-          <t>70000 COP + IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B542" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C542" t="inlineStr">
-        <is>
-          <t>11-11</t>
-        </is>
-      </c>
-      <c r="D542" t="inlineStr">
-        <is>
-          <t>Check-out time</t>
-        </is>
-      </c>
-      <c r="E542" t="inlineStr">
-        <is>
-          <t>Late check-out</t>
-        </is>
-      </c>
-      <c r="F542" t="inlineStr">
-        <is>
-          <t>70000 COP</t>
-        </is>
-      </c>
-      <c r="G542" t="inlineStr">
-        <is>
-          <t>70000 COP + IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="543">
-      <c r="A543" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B543" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C543" t="inlineStr">
-        <is>
-          <t>12-01</t>
-        </is>
-      </c>
-      <c r="D543" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E543" t="inlineStr">
-        <is>
-          <t>Horario y servicio a la habitación</t>
-        </is>
-      </c>
-      <c r="F543" t="inlineStr">
-        <is>
-          <t>06:00-10:00 todos los días; sin room service</t>
-        </is>
-      </c>
-      <c r="G543" t="inlineStr">
-        <is>
-          <t>Lu-Sáb 06:00-10:00, Dom/fest 06:00-10:30; se ofrece con cargo adicional</t>
-        </is>
-      </c>
-    </row>
-    <row r="544">
-      <c r="A544" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B544" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C544" t="inlineStr">
-        <is>
-          <t>12-02</t>
-        </is>
-      </c>
-      <c r="D544" t="inlineStr">
-        <is>
-          <t>Breakfast rates</t>
-        </is>
-      </c>
-      <c r="E544" t="inlineStr">
-        <is>
-          <t>Precio adulto</t>
-        </is>
-      </c>
-      <c r="F544" t="inlineStr">
-        <is>
-          <t>48000 COP</t>
-        </is>
-      </c>
-      <c r="G544" t="inlineStr">
-        <is>
-          <t>40000 COP</t>
-        </is>
-      </c>
-    </row>
-    <row r="545">
-      <c r="A545" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B545" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C545" t="inlineStr">
-        <is>
-          <t>16-10</t>
-        </is>
-      </c>
-      <c r="D545" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="E545" t="inlineStr">
-        <is>
-          <t>Tasa mascota</t>
-        </is>
-      </c>
-      <c r="F545" t="inlineStr">
-        <is>
-          <t>70000 COP/mascota</t>
-        </is>
-      </c>
-      <c r="G545" t="inlineStr">
-        <is>
-          <t>70000 COP + IVA/mascota</t>
-        </is>
-      </c>
-    </row>
-    <row r="546">
-      <c r="A546" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B546" t="inlineStr">
-        <is>
-          <t>GHL Style Yopal</t>
-        </is>
-      </c>
-      <c r="C546" t="inlineStr">
-        <is>
-          <t>17-15</t>
-        </is>
-      </c>
-      <c r="D546" t="inlineStr">
-        <is>
-          <t>Spa hours</t>
-        </is>
-      </c>
-      <c r="E546" t="inlineStr">
-        <is>
-          <t>Disponibilidad</t>
-        </is>
-      </c>
-      <c r="F546" t="inlineStr">
-        <is>
-          <t>Horario de spa sin restricciones</t>
-        </is>
-      </c>
-      <c r="G546" t="inlineStr">
-        <is>
-          <t>Ya no cuentan con spa</t>
-        </is>
-      </c>
-    </row>
-    <row r="547">
-      <c r="A547" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B547" t="inlineStr">
-        <is>
-          <t>GHL Hotel Abadía Plaza</t>
-        </is>
-      </c>
-      <c r="C547" t="inlineStr">
-        <is>
-          <t>13-45</t>
-        </is>
-      </c>
-      <c r="D547" t="inlineStr">
-        <is>
-          <t>Change &amp; ATM</t>
-        </is>
-      </c>
-      <c r="E547" t="inlineStr">
-        <is>
-          <t>Ubicación cajero más cercano</t>
-        </is>
-      </c>
-      <c r="F547" t="inlineStr">
-        <is>
-          <t>Cra. 7 #25-2, a 6 min a pie</t>
-        </is>
-      </c>
-      <c r="G547" t="inlineStr">
-        <is>
-          <t>Cra 8 Clle 19, a 2 min a pie</t>
-        </is>
-      </c>
-    </row>
-    <row r="548">
-      <c r="A548" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B548" t="inlineStr">
-        <is>
-          <t>GHL Hotel Abadía Plaza</t>
-        </is>
-      </c>
-      <c r="C548" t="inlineStr">
-        <is>
-          <t>16-10</t>
-        </is>
-      </c>
-      <c r="D548" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="E548" t="inlineStr">
-        <is>
-          <t>Política de mascotas</t>
-        </is>
-      </c>
-      <c r="F548" t="inlineStr">
-        <is>
-          <t>No se aceptan ni animales de apoyo/servicio certificados</t>
-        </is>
-      </c>
-      <c r="G548" t="inlineStr">
-        <is>
-          <t>Se aceptan animales de apoyo emocional pequeños con certificado médico y carné de vacunas</t>
-        </is>
-      </c>
-    </row>
-    <row r="549">
-      <c r="A549" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B549" t="inlineStr">
-        <is>
-          <t>GHL Hotel Abadía Plaza</t>
-        </is>
-      </c>
-      <c r="C549" t="inlineStr">
-        <is>
-          <t>18-02, 18-03, 18-04</t>
-        </is>
-      </c>
-      <c r="D549" t="inlineStr">
-        <is>
-          <t>Restaurant reservation/cancellation/modification</t>
-        </is>
-      </c>
-      <c r="E549" t="inlineStr">
-        <is>
-          <t>Correo de contacto</t>
-        </is>
-      </c>
-      <c r="F549" t="inlineStr">
-        <is>
-          <t>reservas.abadiaplaza@ghlhoteles.com</t>
-        </is>
-      </c>
-      <c r="G549" t="inlineStr">
-        <is>
-          <t>eventos.abadiaplaza@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="550">
-      <c r="A550" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B550" t="inlineStr">
-        <is>
-          <t>GHL Hotel Abadía Plaza</t>
-        </is>
-      </c>
-      <c r="C550" t="inlineStr">
-        <is>
-          <t>18-11</t>
-        </is>
-      </c>
-      <c r="D550" t="inlineStr">
-        <is>
-          <t>Brunch</t>
-        </is>
-      </c>
-      <c r="E550" t="inlineStr">
-        <is>
-          <t>Recomendación externa</t>
-        </is>
-      </c>
-      <c r="F550" t="inlineStr">
-        <is>
-          <t>MARDIWI (Pereira)</t>
-        </is>
-      </c>
-      <c r="G550" t="inlineStr">
-        <is>
-          <t>Sonesta Pereira - Visus</t>
-        </is>
-      </c>
-    </row>
-    <row r="551">
-      <c r="A551" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B551" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C551" t="inlineStr">
-        <is>
-          <t>10-31</t>
-        </is>
-      </c>
-      <c r="D551" t="inlineStr">
-        <is>
-          <t>Minimum stay</t>
-        </is>
-      </c>
-      <c r="E551" t="inlineStr">
-        <is>
-          <t>Pases de un día</t>
-        </is>
-      </c>
-      <c r="F551" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G551" t="inlineStr">
-        <is>
-          <t>Live Makani Adulto 280000 COP; Live MANA+Almuerzo 440000 COP; Live Makani ELUA X2 1160000 COP</t>
-        </is>
-      </c>
-    </row>
-    <row r="552">
-      <c r="A552" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B552" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C552" t="inlineStr">
-        <is>
-          <t>11-31</t>
-        </is>
-      </c>
-      <c r="D552" t="inlineStr">
-        <is>
-          <t>Front desk</t>
-        </is>
-      </c>
-      <c r="E552" t="inlineStr">
-        <is>
-          <t>Horario recepción</t>
-        </is>
-      </c>
-      <c r="F552" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G552" t="inlineStr">
-        <is>
-          <t>Abierta hasta las 5:00 pm</t>
-        </is>
-      </c>
-    </row>
-    <row r="553">
-      <c r="A553" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B553" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C553" t="inlineStr">
-        <is>
-          <t>11-01</t>
-        </is>
-      </c>
-      <c r="D553" t="inlineStr">
-        <is>
-          <t>Check-in time</t>
-        </is>
-      </c>
-      <c r="E553" t="inlineStr">
-        <is>
-          <t>Horario</t>
-        </is>
-      </c>
-      <c r="F553" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G553" t="inlineStr">
-        <is>
-          <t>3:00 pm a 5:00 pm; sin early check-in</t>
-        </is>
-      </c>
-    </row>
-    <row r="554">
-      <c r="A554" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B554" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C554" t="inlineStr">
-        <is>
-          <t>13-01</t>
-        </is>
-      </c>
-      <c r="D554" t="inlineStr">
-        <is>
-          <t>Parking</t>
-        </is>
-      </c>
-      <c r="E554" t="inlineStr">
-        <is>
-          <t>Parqueadero</t>
-        </is>
-      </c>
-      <c r="F554" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G554" t="inlineStr">
-        <is>
-          <t>Sin parqueadero propio; el más cercano en el parque de la Marina</t>
-        </is>
-      </c>
-    </row>
-    <row r="555">
-      <c r="A555" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B555" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C555" t="inlineStr">
-        <is>
-          <t>13-05</t>
-        </is>
-      </c>
-      <c r="D555" t="inlineStr">
-        <is>
-          <t>Marina &amp; boat dock</t>
-        </is>
-      </c>
-      <c r="E555" t="inlineStr">
-        <is>
-          <t>Horario de llegada en embarcación</t>
-        </is>
-      </c>
-      <c r="F555" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G555" t="inlineStr">
-        <is>
-          <t>Hasta las 4:00 pm; barcos grandes requieren transbordo</t>
-        </is>
-      </c>
-    </row>
-    <row r="556">
-      <c r="A556" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B556" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C556" t="inlineStr">
-        <is>
-          <t>13-21</t>
-        </is>
-      </c>
-      <c r="D556" t="inlineStr">
-        <is>
-          <t>Kids</t>
-        </is>
-      </c>
-      <c r="E556" t="inlineStr">
-        <is>
-          <t>Tarifa infantil</t>
-        </is>
-      </c>
-      <c r="F556" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G556" t="inlineStr">
-        <is>
-          <t>Gratis hasta 3 años; 450000 COP/noche de 3 a 11 años; sin club infantil</t>
-        </is>
-      </c>
-    </row>
-    <row r="557">
-      <c r="A557" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B557" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C557" t="inlineStr">
-        <is>
-          <t>13-41</t>
-        </is>
-      </c>
-      <c r="D557" t="inlineStr">
-        <is>
-          <t>Concierge</t>
-        </is>
-      </c>
-      <c r="E557" t="inlineStr">
-        <is>
-          <t>Horario y servicio</t>
-        </is>
-      </c>
-      <c r="F557" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G557" t="inlineStr">
-        <is>
-          <t>8:00 am a 10:00 pm, inglés y español, sin membresía Clefs d'Or</t>
-        </is>
-      </c>
-    </row>
-    <row r="558">
-      <c r="A558" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B558" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C558" t="inlineStr">
-        <is>
-          <t>13-42</t>
-        </is>
-      </c>
-      <c r="D558" t="inlineStr">
-        <is>
-          <t>Lost &amp; found</t>
-        </is>
-      </c>
-      <c r="E558" t="inlineStr">
-        <is>
-          <t>Contacto</t>
-        </is>
-      </c>
-      <c r="F558" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G558" t="inlineStr">
-        <is>
-          <t>+57 318 335 6186; entrega en muelle de la Bodeguita</t>
-        </is>
-      </c>
-    </row>
-    <row r="559">
-      <c r="A559" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B559" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C559" t="inlineStr">
-        <is>
-          <t>13-50</t>
-        </is>
-      </c>
-      <c r="D559" t="inlineStr">
-        <is>
-          <t>Airport &amp; train station public transport</t>
-        </is>
-      </c>
-      <c r="E559" t="inlineStr">
-        <is>
-          <t>Tiempo de traslado</t>
-        </is>
-      </c>
-      <c r="F559" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G559" t="inlineStr">
-        <is>
-          <t>20 min terrestre + 25 min marítimo desde el aeropuerto</t>
-        </is>
-      </c>
-    </row>
-    <row r="560">
-      <c r="A560" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B560" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C560" t="inlineStr">
-        <is>
-          <t>16-15</t>
-        </is>
-      </c>
-      <c r="D560" t="inlineStr">
-        <is>
-          <t>Social &amp; photoshoot</t>
-        </is>
-      </c>
-      <c r="E560" t="inlineStr">
-        <is>
-          <t>Contacto</t>
-        </is>
-      </c>
-      <c r="F560" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G560" t="inlineStr">
-        <is>
-          <t>laura.molina@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="561">
-      <c r="A561" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B561" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C561" t="inlineStr">
-        <is>
-          <t>17-91</t>
-        </is>
-      </c>
-      <c r="D561" t="inlineStr">
-        <is>
-          <t>Boutique</t>
-        </is>
-      </c>
-      <c r="E561" t="inlineStr">
-        <is>
-          <t>Productos</t>
-        </is>
-      </c>
-      <c r="F561" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G561" t="inlineStr">
-        <is>
-          <t>Bloqueador, vestidos de baño, sombreros, bolsos, sandalias</t>
-        </is>
-      </c>
-    </row>
-    <row r="562">
-      <c r="A562" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B562" t="inlineStr">
-        <is>
-          <t>Makani Luxury Wanderlust</t>
-        </is>
-      </c>
-      <c r="C562" t="inlineStr">
-        <is>
-          <t>20-02, 20-21, 20-22</t>
-        </is>
-      </c>
-      <c r="D562" t="inlineStr">
-        <is>
-          <t>Business meeting / Celebration</t>
-        </is>
-      </c>
-      <c r="E562" t="inlineStr">
-        <is>
-          <t>Salas de reunión y eventos</t>
-        </is>
-      </c>
-      <c r="F562" t="inlineStr">
-        <is>
-          <t>⚠ Verificar en correo</t>
-        </is>
-      </c>
-      <c r="G562" t="inlineStr">
-        <is>
-          <t>Sin salas de reuniones; eventos vía camila.dickens@ghlhoteles.com / eventos.makani@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="563">
-      <c r="A563" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B563" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C563" t="inlineStr">
-        <is>
-          <t>13-43</t>
-        </is>
-      </c>
-      <c r="D563" t="inlineStr">
-        <is>
-          <t>Laundry</t>
-        </is>
-      </c>
-      <c r="E563" t="inlineStr">
-        <is>
-          <t>Tiempo de entrega</t>
-        </is>
-      </c>
-      <c r="F563" t="inlineStr">
-        <is>
-          <t>Se devuelve antes de las 10:00</t>
-        </is>
-      </c>
-      <c r="G563" t="inlineStr">
-        <is>
-          <t>Se devuelve el mismo día</t>
-        </is>
-      </c>
-    </row>
-    <row r="564">
-      <c r="A564" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B564" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C564" t="inlineStr">
-        <is>
-          <t>14-04</t>
-        </is>
-      </c>
-      <c r="D564" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="E564" t="inlineStr">
-        <is>
-          <t>Tarifa limpieza por humo</t>
-        </is>
-      </c>
-      <c r="F564" t="inlineStr">
-        <is>
-          <t>700 PEN</t>
-        </is>
-      </c>
-      <c r="G564" t="inlineStr">
-        <is>
-          <t>USD 200.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="565">
-      <c r="A565" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B565" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C565" t="inlineStr">
-        <is>
-          <t>15-06</t>
-        </is>
-      </c>
-      <c r="D565" t="inlineStr">
-        <is>
-          <t>Bathroom equipment</t>
-        </is>
-      </c>
-      <c r="E565" t="inlineStr">
-        <is>
-          <t>Artículos gratis a petición</t>
-        </is>
-      </c>
-      <c r="F565" t="inlineStr">
-        <is>
-          <t>Pantuflas, pasta de dientes, kit de afeitar</t>
-        </is>
-      </c>
-      <c r="G565" t="inlineStr">
-        <is>
-          <t>Pantuflas, kit dental, kit de afeitar, costurero, limpia calzados y peine</t>
-        </is>
-      </c>
-    </row>
-    <row r="566">
-      <c r="A566" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B566" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C566" t="inlineStr">
-        <is>
-          <t>15-24, 15-99</t>
-        </is>
-      </c>
-      <c r="D566" t="inlineStr">
-        <is>
-          <t>Extra bed / Specific room request</t>
-        </is>
-      </c>
-      <c r="E566" t="inlineStr">
-        <is>
-          <t>Correo de contacto</t>
-        </is>
-      </c>
-      <c r="F566" t="inlineStr">
-        <is>
-          <t>Incluía calidad.sonestaarequipa</t>
-        </is>
-      </c>
-      <c r="G566" t="inlineStr">
-        <is>
-          <t>Solo reservas.sonestaarequipa@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="567">
-      <c r="A567" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B567" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C567" t="inlineStr">
-        <is>
-          <t>16-06</t>
-        </is>
-      </c>
-      <c r="D567" t="inlineStr">
-        <is>
-          <t>Jobs &amp; internships</t>
-        </is>
-      </c>
-      <c r="E567" t="inlineStr">
-        <is>
-          <t>Contacto RRHH</t>
-        </is>
-      </c>
-      <c r="F567" t="inlineStr">
-        <is>
-          <t>contactenos@ghlhoteles.com / +57 601 3139330</t>
-        </is>
-      </c>
-      <c r="G567" t="inlineStr">
-        <is>
-          <t>laydy.pauca@ghlhoteles.com / +51 054 308 777</t>
-        </is>
-      </c>
-    </row>
-    <row r="568">
-      <c r="A568" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B568" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C568" t="inlineStr">
-        <is>
-          <t>16-25</t>
-        </is>
-      </c>
-      <c r="D568" t="inlineStr">
-        <is>
-          <t>Tips policy</t>
-        </is>
-      </c>
-      <c r="E568" t="inlineStr">
-        <is>
-          <t>Política de propinas</t>
-        </is>
-      </c>
-      <c r="F568" t="inlineStr">
-        <is>
-          <t>Incluía la línea 'es costumbre dejar propina'</t>
-        </is>
-      </c>
-      <c r="G568" t="inlineStr">
-        <is>
-          <t>Se elimina esa línea</t>
-        </is>
-      </c>
-    </row>
-    <row r="569">
-      <c r="A569" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B569" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C569" t="inlineStr">
-        <is>
-          <t>17-02, 18-02, 18-03, 18-04</t>
-        </is>
-      </c>
-      <c r="D569" t="inlineStr">
-        <is>
-          <t>Reservas restaurante/bar</t>
-        </is>
-      </c>
-      <c r="E569" t="inlineStr">
-        <is>
-          <t>Teléfono de contacto</t>
-        </is>
-      </c>
-      <c r="F569" t="inlineStr">
-        <is>
-          <t>Solo correo</t>
-        </is>
-      </c>
-      <c r="G569" t="inlineStr">
-        <is>
-          <t>Se agrega +51 945 739 921</t>
-        </is>
-      </c>
-    </row>
-    <row r="570">
-      <c r="A570" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B570" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C570" t="inlineStr">
-        <is>
-          <t>17-10</t>
-        </is>
-      </c>
-      <c r="D570" t="inlineStr">
-        <is>
-          <t>Spa</t>
-        </is>
-      </c>
-      <c r="E570" t="inlineStr">
-        <is>
-          <t>Política de acceso</t>
-        </is>
-      </c>
-      <c r="F570" t="inlineStr">
-        <is>
-          <t>Abierto solo clientes; edad mínima 12 años</t>
-        </is>
-      </c>
-      <c r="G570" t="inlineStr">
-        <is>
-          <t>Menores de 12 solo con padres/tutor; masajes con costo adicional</t>
-        </is>
-      </c>
-    </row>
-    <row r="571">
-      <c r="A571" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B571" t="inlineStr">
-        <is>
-          <t>Sonesta Arequipa</t>
-        </is>
-      </c>
-      <c r="C571" t="inlineStr">
-        <is>
-          <t>18-01</t>
-        </is>
-      </c>
-      <c r="D571" t="inlineStr">
-        <is>
-          <t>Restaurant</t>
-        </is>
-      </c>
-      <c r="E571" t="inlineStr">
-        <is>
-          <t>Descripción restaurante Micaela</t>
-        </is>
-      </c>
-      <c r="F571" t="inlineStr">
-        <is>
-          <t>Incluía capacidad, política de niños y tronas</t>
-        </is>
-      </c>
-      <c r="G571" t="inlineStr">
-        <is>
-          <t>Descripción simplificada (se retira info de capacidad y niños)</t>
-        </is>
-      </c>
-    </row>
-    <row r="572">
-      <c r="A572" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B572" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C572" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D572" t="inlineStr">
-        <is>
-          <t>Clasificación del hotel</t>
-        </is>
-      </c>
-      <c r="E572" t="inlineStr">
-        <is>
-          <t>Estrellas</t>
-        </is>
-      </c>
-      <c r="F572" t="inlineStr">
-        <is>
-          <t>5 estrellas</t>
-        </is>
-      </c>
-      <c r="G572" t="inlineStr">
-        <is>
-          <t>4 estrellas</t>
-        </is>
-      </c>
-    </row>
-    <row r="573">
-      <c r="A573" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B573" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C573" t="inlineStr">
-        <is>
-          <t>14-04</t>
-        </is>
-      </c>
-      <c r="D573" t="inlineStr">
-        <is>
-          <t>Smoking</t>
-        </is>
-      </c>
-      <c r="E573" t="inlineStr">
-        <is>
-          <t>Detectores de humo</t>
-        </is>
-      </c>
-      <c r="F573" t="inlineStr">
-        <is>
-          <t>Las habitaciones no están equipadas con detectores de humo</t>
-        </is>
-      </c>
-      <c r="G573" t="inlineStr">
-        <is>
-          <t>Las habitaciones están equipadas con detectores de humo</t>
-        </is>
-      </c>
-    </row>
-    <row r="574">
-      <c r="A574" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B574" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C574" t="inlineStr">
-        <is>
-          <t>15-06</t>
-        </is>
-      </c>
-      <c r="D574" t="inlineStr">
-        <is>
-          <t>Bathroom equipment</t>
-        </is>
-      </c>
-      <c r="E574" t="inlineStr">
-        <is>
-          <t>Artículos gratis / no disponibles</t>
-        </is>
-      </c>
-      <c r="F574" t="inlineStr">
-        <is>
-          <t>Lista distinta</t>
-        </is>
-      </c>
-      <c r="G574" t="inlineStr">
-        <is>
-          <t>Se agregan albornoz, pantuflas, gel de ducha, hisopos, cepillo y pasta de dientes; se recorta lista de no disponibles</t>
-        </is>
-      </c>
-    </row>
-    <row r="575">
-      <c r="A575" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B575" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C575" t="inlineStr">
-        <is>
-          <t>15-23</t>
-        </is>
-      </c>
-      <c r="D575" t="inlineStr">
-        <is>
-          <t>Extra bed</t>
-        </is>
-      </c>
-      <c r="E575" t="inlineStr">
-        <is>
-          <t>Precio cama extra</t>
-        </is>
-      </c>
-      <c r="F575" t="inlineStr">
-        <is>
-          <t>110000 COP/noche</t>
-        </is>
-      </c>
-      <c r="G575" t="inlineStr">
-        <is>
-          <t>Se elimina el precio; solo se indica correo de solicitud</t>
-        </is>
-      </c>
-    </row>
-    <row r="576">
-      <c r="A576" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B576" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C576" t="inlineStr">
-        <is>
-          <t>16-02</t>
-        </is>
-      </c>
-      <c r="D576" t="inlineStr">
-        <is>
-          <t>Contact staff</t>
-        </is>
-      </c>
-      <c r="E576" t="inlineStr">
-        <is>
-          <t>Teléfono gratuito</t>
-        </is>
-      </c>
-      <c r="F576" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="G576" t="inlineStr">
-        <is>
-          <t>+57 3052281127 (recepción, reserva y eventos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="577">
-      <c r="A577" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B577" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C577" t="inlineStr">
-        <is>
-          <t>10-04, 10-06</t>
-        </is>
-      </c>
-      <c r="D577" t="inlineStr">
-        <is>
-          <t>Reservation modification/cancellation</t>
-        </is>
-      </c>
-      <c r="E577" t="inlineStr">
-        <is>
-          <t>Correo</t>
-        </is>
-      </c>
-      <c r="F577" t="inlineStr">
-        <is>
-          <t>reservas.sonetabogota (typo)</t>
-        </is>
-      </c>
-      <c r="G577" t="inlineStr">
-        <is>
-          <t>reservas.sonestabogota@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="578">
-      <c r="A578" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B578" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C578" t="inlineStr">
-        <is>
-          <t>13-01</t>
-        </is>
-      </c>
-      <c r="D578" t="inlineStr">
-        <is>
-          <t>Parking</t>
-        </is>
-      </c>
-      <c r="E578" t="inlineStr">
-        <is>
-          <t>Política y parqueo de bicis</t>
-        </is>
-      </c>
-      <c r="F578" t="inlineStr">
-        <is>
-          <t>Gratuito para todos; sin parqueo de bicis</t>
-        </is>
-      </c>
-      <c r="G578" t="inlineStr">
-        <is>
-          <t>Gratuito solo para huéspedes (invitados pagan tarifa); sí hay parqueo de bicis</t>
-        </is>
-      </c>
-    </row>
-    <row r="579">
-      <c r="A579" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B579" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C579" t="inlineStr">
-        <is>
-          <t>15-61</t>
-        </is>
-      </c>
-      <c r="D579" t="inlineStr">
-        <is>
-          <t>Balcony &amp; windows</t>
-        </is>
-      </c>
-      <c r="E579" t="inlineStr">
-        <is>
-          <t>Balcón</t>
-        </is>
-      </c>
-      <c r="F579" t="inlineStr">
-        <is>
-          <t>Todas las habitaciones tienen balcón</t>
-        </is>
-      </c>
-      <c r="G579" t="inlineStr">
-        <is>
-          <t>Ninguna habitación tiene balcón; la suite tiene terraza</t>
-        </is>
-      </c>
-    </row>
-    <row r="580">
-      <c r="A580" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B580" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C580" t="inlineStr">
-        <is>
-          <t>16-10</t>
-        </is>
-      </c>
-      <c r="D580" t="inlineStr">
-        <is>
-          <t>Pets</t>
-        </is>
-      </c>
-      <c r="E580" t="inlineStr">
-        <is>
-          <t>Zonas restringidas</t>
-        </is>
-      </c>
-      <c r="F580" t="inlineStr">
-        <is>
-          <t>Lista extensa de zonas</t>
-        </is>
-      </c>
-      <c r="G580" t="inlineStr">
-        <is>
-          <t>Zonas públicas, salas de conferencias, gimnasio, Porterhouse y Cook's</t>
-        </is>
-      </c>
-    </row>
-    <row r="581">
-      <c r="A581" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B581" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C581" t="inlineStr">
-        <is>
-          <t>17-01</t>
-        </is>
-      </c>
-      <c r="D581" t="inlineStr">
-        <is>
-          <t>Bar</t>
-        </is>
-      </c>
-      <c r="E581" t="inlineStr">
-        <is>
-          <t>Nombre y horario</t>
-        </is>
-      </c>
-      <c r="F581" t="inlineStr">
-        <is>
-          <t>Cook's PorterHouse, 12:00-22:00 todos los días</t>
-        </is>
-      </c>
-      <c r="G581" t="inlineStr">
-        <is>
-          <t>PorterHouse, horario variable por día (hasta 22:00-22:30 según el día)</t>
-        </is>
-      </c>
-    </row>
-    <row r="582">
-      <c r="A582" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B582" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C582" t="inlineStr">
-        <is>
-          <t>17-11, 17-15</t>
-        </is>
-      </c>
-      <c r="D582" t="inlineStr">
-        <is>
-          <t>Spa reservation / hours</t>
-        </is>
-      </c>
-      <c r="E582" t="inlineStr">
-        <is>
-          <t>Nombre del servicio</t>
-        </is>
-      </c>
-      <c r="F582" t="inlineStr">
-        <is>
-          <t>Spa / Tratamiento de Spa</t>
-        </is>
-      </c>
-      <c r="G582" t="inlineStr">
-        <is>
-          <t>Sala de bienestar / Masaje; consultar disponibilidad por correo</t>
-        </is>
-      </c>
-    </row>
-    <row r="583">
-      <c r="A583" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B583" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C583" t="inlineStr">
-        <is>
-          <t>18-01</t>
-        </is>
-      </c>
-      <c r="D583" t="inlineStr">
-        <is>
-          <t>Restaurant</t>
-        </is>
-      </c>
-      <c r="E583" t="inlineStr">
-        <is>
-          <t>Nombre, horarios y política de niños</t>
-        </is>
-      </c>
-      <c r="F583" t="inlineStr">
-        <is>
-          <t>Cook's Porterhouse (no acepta niños); Cook's 6:00-10:00</t>
-        </is>
-      </c>
-      <c r="G583" t="inlineStr">
-        <is>
-          <t>Porterhouse (steak house, acepta niños, horario variable); Cook's 6:00-10:00 y 6:30-10:30 fines de semana</t>
-        </is>
-      </c>
-    </row>
-    <row r="584">
-      <c r="A584" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B584" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C584" t="inlineStr">
-        <is>
-          <t>18-08</t>
-        </is>
-      </c>
-      <c r="D584" t="inlineStr">
-        <is>
-          <t>Takeaway &amp; delivery</t>
-        </is>
-      </c>
-      <c r="E584" t="inlineStr">
-        <is>
-          <t>Catering</t>
-        </is>
-      </c>
-      <c r="F584" t="inlineStr">
-        <is>
-          <t>Se ofrecía catering</t>
-        </is>
-      </c>
-      <c r="G584" t="inlineStr">
-        <is>
-          <t>No hay catering; solo domicilios</t>
-        </is>
-      </c>
-    </row>
-    <row r="585">
-      <c r="A585" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B585" t="inlineStr">
-        <is>
-          <t>Sonesta Bogotá</t>
-        </is>
-      </c>
-      <c r="C585" t="inlineStr">
-        <is>
-          <t>18-26</t>
-        </is>
-      </c>
-      <c r="D585" t="inlineStr">
-        <is>
-          <t>Valentine's day</t>
-        </is>
-      </c>
-      <c r="E585" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="F585" t="inlineStr">
-        <is>
-          <t>Enlace a oferta específica</t>
-        </is>
-      </c>
-      <c r="G585" t="inlineStr">
-        <is>
-          <t>Información general de eventos de temporada</t>
-        </is>
-      </c>
-    </row>
-    <row r="586">
-      <c r="A586" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B586" t="inlineStr">
-        <is>
-          <t>Sonesta Pereira</t>
-        </is>
-      </c>
-      <c r="C586" t="inlineStr">
-        <is>
-          <t>12-01</t>
-        </is>
-      </c>
-      <c r="D586" t="inlineStr">
-        <is>
-          <t>Breakfast time</t>
-        </is>
-      </c>
-      <c r="E586" t="inlineStr">
-        <is>
-          <t>Horario</t>
-        </is>
-      </c>
-      <c r="F586" t="inlineStr">
-        <is>
-          <t>06:00 a 10:00</t>
-        </is>
-      </c>
-      <c r="G586" t="inlineStr">
-        <is>
-          <t>06:30 a 10:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="587">
-      <c r="A587" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B587" t="inlineStr">
-        <is>
-          <t>Sonesta Pereira</t>
-        </is>
-      </c>
-      <c r="C587" t="inlineStr">
-        <is>
-          <t>13-53</t>
-        </is>
-      </c>
-      <c r="D587" t="inlineStr">
-        <is>
-          <t>Taxi</t>
-        </is>
-      </c>
-      <c r="E587" t="inlineStr">
-        <is>
-          <t>Precio y correo</t>
-        </is>
-      </c>
-      <c r="F587" t="inlineStr">
-        <is>
-          <t>Aeropuerto 26000 COP, Centro 28000 COP, recepcion.sonestapereira@ghlhoteles.com</t>
-        </is>
-      </c>
-      <c r="G587" t="inlineStr">
-        <is>
-          <t>Aeropuerto 40000 COP, Centro 45000 COP, reservas.sonestapereira@ghlhoteles.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="588">
-      <c r="A588" t="inlineStr">
-        <is>
-          <t>Sep-26</t>
-        </is>
-      </c>
-      <c r="B588" t="inlineStr">
-        <is>
-          <t>Sonesta Pereira</t>
-        </is>
-      </c>
-      <c r="C588" t="inlineStr">
-        <is>
-          <t>18-01</t>
-        </is>
-      </c>
-      <c r="D588" t="inlineStr">
-        <is>
-          <t>Restaurant</t>
-        </is>
-      </c>
-      <c r="E588" t="inlineStr">
-        <is>
-          <t>Horario</t>
-        </is>
-      </c>
-      <c r="F588" t="inlineStr">
-        <is>
-          <t>06:00 a 22:00</t>
-        </is>
-      </c>
-      <c r="G588" t="inlineStr">
-        <is>
-          <t>06:30 a 22:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza contacto de Biohotel para Sep-26: Sofia Solano reemplaza a Pilar Narvaez
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6950,12 +6950,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Maria Del Pilar Narvaez</t>
+          <t>Sofia Solano</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>pilar.narvaez@ghlhoteles.com</t>
+          <t>sofia.solano@ghlhoteles.com</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -6966,6 +6966,11 @@
       <c r="G131" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Cambio de contacto: antes Maria Del Pilar Narvaez (pilar.narvaez@ghlhoteles.com)</t>
         </is>
       </c>
       <c r="K131" s="44" t="inlineStr">

</xml_diff>

<commit_message>
Registra a Sonesta Loja como sin modificaciones para Sep-26 (respondió 16/09)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -8428,14 +8428,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K166" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K166" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8855,23 +8865,23 @@
         <v>42</v>
       </c>
       <c r="C7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="I7">
@@ -8994,23 +9004,23 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" t="n">
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>█████████████░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
       <c r="I4" s="44" t="inlineStr">
@@ -9134,19 +9144,19 @@
         <v>168</v>
       </c>
       <c r="C8" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
         <v>56</v>
       </c>
       <c r="F8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4583333333333333</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Marca como Actualizado los 10 hoteles con modificaciones de Sep-26
Confirmado que los cambios de Arsenal, Geotel Calama, GHL Relax Club Hotel
el Puente, GHL Relax Hotel Sunrise, GHL Style Yopal, GHL Hotel Abadía
Plaza, Makani Luxury Wanderlust, Sonesta Arequipa, Sonesta Bogotá y
Sonesta Pereira ya quedaron aplicados en el chatbot (Velma). Se actualiza
fecha y estado en el HTML y el Excel, y el contador de "Actualizados en
chatbot" en Resumen por ciclo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -6931,9 +6931,14 @@
           <t>7 diálogos modificados: desayuno, tarifas, objetos perdidos, delivery, taxi, ascensor, teléfono de contacto</t>
         </is>
       </c>
-      <c r="K130" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K130" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7094,14 +7099,19 @@
           <t>11 diálogos modificados: contacto, pago, desayuno, cuna, lavandería, ocupación, horarios, gimnasio, ascensor, transporte</t>
         </is>
       </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="J134" t="inlineStr">
         <is>
           <t>Respuesta con formato informal — varios diálogos sin número claro o sin valor 'antes'; ver detalle. Diálogo 14-02 con respuesta poco clara ('NO ENTENDI')</t>
         </is>
       </c>
-      <c r="K134" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K134" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7462,9 +7472,14 @@
           <t>4 diálogos modificados: remodelación, day use, mascotas, piscina</t>
         </is>
       </c>
-      <c r="K143" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K143" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7593,9 +7608,14 @@
           <t>8 diálogos modificados: contacto, reservas, pago, day pass, check-in, desayuno, parqueadero, club infantil</t>
         </is>
       </c>
-      <c r="K146" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K146" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7761,14 +7781,19 @@
           <t>7 diálogos modificados: método de pago, check-in, check-out, desayuno, mascotas, spa</t>
         </is>
       </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="J150" t="inlineStr">
         <is>
           <t>Reporta que los ajustes enviados en ciclos anteriores no se ven reflejados en el chatbot — verificar</t>
         </is>
       </c>
-      <c r="K150" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K150" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7850,9 +7875,14 @@
           <t>4 diálogos modificados: cajero, mascotas, reservas restaurante, brunch</t>
         </is>
       </c>
-      <c r="K152" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K152" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -7981,14 +8011,19 @@
           <t>12 diálogos actualizados vía PDF adjunto: pases, recepción, check-in, parqueadero, muelle, niños, conserjería, objetos perdidos, transporte, eventos, boutique</t>
         </is>
       </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="J155" t="inlineStr">
         <is>
           <t>Correcciones enviadas solo en PDF adjunto, sin texto antes/después en el cuerpo del correo — valores 'antes' marcados como Verificar en correo</t>
         </is>
       </c>
-      <c r="K155" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K155" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8312,9 +8347,14 @@
           <t>9 diálogos modificados: lavandería, fumadores, baño, cama extra, empleo, propinas, reservas restaurante, spa, restaurante</t>
         </is>
       </c>
-      <c r="K163" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K163" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8359,9 +8399,14 @@
           <t>13 diálogos modificados: clasificación, fumadores, baño, cama extra, contacto, parqueadero, balcón, mascotas, bar, spa, restaurante, delivery, San Valentín</t>
         </is>
       </c>
-      <c r="K164" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K164" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8527,9 +8572,14 @@
           <t>3 diálogos modificados: desayuno, taxi, restaurante</t>
         </is>
       </c>
-      <c r="K168" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K168" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8927,7 @@
         <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Registra a Hotel Tequendama Bogotá, Sonesta Bucaramanga, Sonesta Osorno y GHL Style Barrancabermeja como sin modificaciones para Sep-26
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -7645,14 +7645,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K147" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K147" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -7823,14 +7833,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K151" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K151" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8137,14 +8157,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K158" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K158" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8520,14 +8550,24 @@
           <t>02/09/2026</t>
         </is>
       </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K167" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Confirmó sin cambios para septiembre</t>
+        </is>
+      </c>
+      <c r="K167" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -8915,23 +8955,23 @@
         <v>42</v>
       </c>
       <c r="C7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" t="n">
         <v>19</v>
-      </c>
-      <c r="D7" t="n">
-        <v>23</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
         <v>10</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="I7">
@@ -9054,28 +9094,28 @@
         <v>42</v>
       </c>
       <c r="C4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D4" t="n">
         <v>19</v>
-      </c>
-      <c r="D4" t="n">
-        <v>23</v>
       </c>
       <c r="E4" t="n">
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.5476190476190477</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I4" s="44" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>████████████████░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
+        <is>
+          <t>En progreso</t>
         </is>
       </c>
     </row>
@@ -9194,23 +9234,23 @@
         <v>168</v>
       </c>
       <c r="C8" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E8" t="n">
         <v>56</v>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4642857142857143</v>
+        <v>0.4880952380952381</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
+          <t>███████████████░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Abre el ciclo Octubre 2026 (Oct-26)
42 hoteles en HTML y Excel (Consolidado), color violeta, y nueva fila en
Dashboard cumplimiento (con TOTAL recalculado) y Resumen por ciclo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -201,8 +201,19 @@
       <color rgb="009D174D"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="004C1D95"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004C1D95"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -306,6 +317,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE7F3"/>
         <bgColor rgb="00FCE7F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE9FE"/>
+        <bgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -437,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -564,6 +581,13 @@
     <xf numFmtId="0" fontId="30" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -929,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8739,6 +8763,1560 @@
         </is>
       </c>
       <c r="K171" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Luis Saez</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>luis.saez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K172" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Biohotel</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Sofia Solano</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>sofia.solano@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K173" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Bioxury</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>calidad.bioxury@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K174" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Geotel Antofagasta</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Nelson Uriel Perez Ortiz</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>nelson.perez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K175" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Geotel Calama</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Katherine Mora</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>katherine.mora@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K176" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>GHL Collection 93</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>James Mendoza</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>james.mendoza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K177" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Armeria Real</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Saray Estrada</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Saray.estrada@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K178" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>GHL Collection Hamilton</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Wilson Bohorquez</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>andres.bohorquez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K179" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>GHL Grand Villavicencio</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Ingrid Mendez</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>jimena.mendez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K180" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>GHL Hotel Capital</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Maira Piza</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>maira.piza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K181" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>GHL Lago Titicaca</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Milagros Velazco Reyes</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>milagros.velazco@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K182" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>GHL Montería</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Jose Medina</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>mauricio.medina@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K183" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>GHL Portón Medellín</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Jose Fernando Villareal</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>jose.villareal@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K184" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>GHL Relax Club Hotel el Puente</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Maria Gomez</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>angelica.gomez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K185" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Corales de Indias</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Andres Narvaez</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>andres.narvaez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K186" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Costa Azul</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Marlis Marriaga</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>marlys.marriaga@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K187" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>GHL Relax Hotel Sunrise</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Juan Martinez</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>juan.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K188" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>GHL Style Barrancabermeja</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Luis Martinez</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>luis.martinez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K189" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>GHL Style Bogotá Occidente</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Leidy Cely</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>jrecepcion.bogotaoccidente@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K190" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>GHL Style Neiva</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Carlos Robayo</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>yobani.robayo@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K191" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>GHL Style Yopal</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Mafy Daniela Rodriguez</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>daniela.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K192" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Hotel Tequendama Bogotá</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Sara Judith Aguirre</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>sara.aguirre@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K193" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>GHL Hotel Abadía Plaza</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Katerine Ospina Gil</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>suprecepcion.abadiaplaza@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K194" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>GHL Hotel Grand Barranquilla</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Jose Carlos Ibañez</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>jose.ibanez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K195" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>LATAM XELA</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Gabriela Rodas</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>gabriela.rodas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K196" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Makani Luxury Wanderlust</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Jose Macea</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>jose.macea@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K197" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Sergio Víctor Alejandro Yevenes Escobar</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>sergio.yevenes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K198" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>San Lazaro Art</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Keilis Mercado</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>keilis.mercado@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K199" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Sonesta Bucaramanga</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Jeferson Reyes</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>jeferson.reyes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K200" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Sonesta Cali</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Lorena Figueroa</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>lorena.figueroa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K201" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Sonesta Cartagena</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Liliana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>liliana.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K202" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Sonesta Cusco</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Adolfo Alfaro</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>adolfo.alfaro@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K203" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Sonesta El Olivar</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Andrea Silvana Zevallos</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>andrea.zevallos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K204" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Sonesta Arequipa</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Tania Catacora</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>jefederecepcion.sonestaarequipa@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K205" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Sonesta Bogotá</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Catalina Rojas</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>catalina.rojas@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K206" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Sonesta Ibagué</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Wilmer Rodriguez</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>wilmer.rodriguez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K207" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Sonesta Loja</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Miryam Ramirez</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>miryam.ramirez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K208" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Sonesta Osorno</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Cristina Sanzana</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>cristina.sanzana@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K209" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Sonesta Pereira</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Edwar Pacanchique</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>edwar.pacanchique@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K210" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Sonesta Puno</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Delmy Nuñez</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>delmy.nunez@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K211" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Sonesta Yucay</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Monica Chirinos</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>monica.chirinos@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K212" s="44" t="inlineStr">
+        <is>
+          <t>Sin respuesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Sonesta Valledupar</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Emerson David Cotes</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>emerson.cotes@ghlhoteles.com</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K213" s="44" t="inlineStr">
         <is>
           <t>Sin respuesta</t>
         </is>
@@ -8768,7 +10346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8976,6 +10554,40 @@
       </c>
       <c r="I7">
         <f>IF(B7&gt;0,C7/B7,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>42</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="I8">
+        <f>IF(B8&gt;0,C8/B8,0)</f>
         <v/>
       </c>
     </row>
@@ -9003,7 +10615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9085,188 +10697,222 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="51" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Sep-26</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B5" t="n">
         <v>42</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C5" t="n">
         <v>23</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D5" t="n">
         <v>19</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E5" t="n">
         <v>10</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F5" t="n">
         <v>13</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G5" t="n">
         <v>0.5476190476190477</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>████████████████░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I4" s="46" t="inlineStr">
+      <c r="I5" s="46" t="inlineStr">
         <is>
           <t>En progreso</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Ago-26</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>42</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>22</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" s="20" t="n">
-        <v>0.4761904761904762</v>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I5" s="22" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>Ago-26</t>
         </is>
       </c>
       <c r="B6" s="19" t="n">
         <v>42</v>
       </c>
       <c r="C6" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>0.4761904761904762</v>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>██████████████░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D7" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E7" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F7" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G7" s="20" t="n">
         <v>0.3809523809523809</v>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>███████████░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I7" s="22" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>Jun-26</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="n">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
         <v>42</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C8" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D8" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E8" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G8" s="20" t="n">
         <v>0.5476190476190477</v>
       </c>
-      <c r="H7" s="25" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <t>████████████████░░░░░░░░░░░░░░</t>
         </is>
       </c>
-      <c r="I7" s="26" t="inlineStr">
+      <c r="I8" s="26" t="inlineStr">
         <is>
           <t>En progreso</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>168</v>
-      </c>
-      <c r="C8" t="n">
+      <c r="B9" t="n">
+        <v>210</v>
+      </c>
+      <c r="C9" t="n">
         <v>82</v>
       </c>
-      <c r="D8" t="n">
-        <v>86</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D9" t="n">
+        <v>128</v>
+      </c>
+      <c r="E9" t="n">
         <v>56</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F9" t="n">
         <v>26</v>
       </c>
-      <c r="G8" t="n">
-        <v>0.4880952380952381</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>███████████████░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="G9" t="n">
+        <v>0.3904761904761905</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>████████████░░░░░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>Nota: La barra de progreso refleja % de hoteles que respondieron el correo (con o sin modificaciones). Completo = 100% · En progreso = 50-99% · Pendiente = &lt; 50%</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A7"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A10:I10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualiza contacto de Sonesta Pereira para Oct-26: Luisa Ramírez reemplaza a Edwar Pacanchique
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -10187,12 +10187,12 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Edwar Pacanchique</t>
+          <t>Luisa Ramírez</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>edwar.pacanchique@ghlhoteles.com</t>
+          <t>jeferecepcion.sonestapereira@ghlhoteles.com</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -10203,6 +10203,11 @@
       <c r="G210" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>Cambio de contacto: antes Edwar Pacanchique (edwar.pacanchique@ghlhoteles.com)</t>
         </is>
       </c>
       <c r="K210" s="44" t="inlineStr">
@@ -10910,9 +10915,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A10:I10"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A10:I10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sonesta Bogotá Oct-26: agrega 15-48 del adjunto y actualiza notas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -10314,12 +10314,12 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>7 diálogos modificados: desayuno, solicitudes especiales, fumadores, baño, bar, gimnasio, restaurante</t>
+          <t>8 diálogos modificados: desayuno, solicitudes especiales, fumadores, baño, instalaciones eléctricas, bar, gimnasio, restaurante</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>ATENCIÓN: el correo trae además un adjunto reenviado (.eml) con otras modificaciones que el conector no permite leer — abrirlo en Outlook y completar (puede cambiar 12-01, 17-01, 18-01 o añadir más). El hotel solo reportó el 'después' en el cuerpo; el 'antes' se tomó del PDF original de octubre. 17-31: el texto no menciona 'gimnasio'</t>
+          <t>Texto del adjunto reenviado aportado por el usuario: confirma 12-01, 13-17, 14-04, 15-06, 17-01 y 17-31 (igual al cuerpo del correo) y agrega 15-48 (solo adaptadores eléctricos, sin mencionar cargador de móvil). 18-01 solo viene en el cuerpo del correo. 17-31: el texto no menciona 'gimnasio'. El 'antes' se tomó del PDF original de octubre</t>
         </is>
       </c>
       <c r="K206" s="46" t="inlineStr">
@@ -11209,7 +11209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H633"/>
+  <dimension ref="A1:H634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34561,27 +34561,27 @@
       </c>
       <c r="C621" s="41" t="inlineStr">
         <is>
-          <t>17-01</t>
+          <t>15-48</t>
         </is>
       </c>
       <c r="D621" s="41" t="inlineStr">
         <is>
-          <t>Bar</t>
+          <t>Electrical &amp; mobile phone facilities</t>
         </is>
       </c>
       <c r="E621" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Adaptadores eléctricos</t>
         </is>
       </c>
       <c r="F621" s="41" t="inlineStr">
         <is>
-          <t>Jue a sáb 12:00-22:30; domingo 12:00-21:00</t>
+          <t>⚠ Verificar en correo</t>
         </is>
       </c>
       <c r="G621" s="41" t="inlineStr">
         <is>
-          <t>Abierto 7/7: lunes a sábado 12:00-22:00; domingos y festivos 12:00-21:00</t>
+          <t>Adaptadores eléctricos: disponible gratuitamente</t>
         </is>
       </c>
     </row>
@@ -34598,27 +34598,27 @@
       </c>
       <c r="C622" s="41" t="inlineStr">
         <is>
-          <t>17-31</t>
+          <t>17-01</t>
         </is>
       </c>
       <c r="D622" s="41" t="inlineStr">
         <is>
-          <t>Fitness gym</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="E622" s="41" t="inlineStr">
         <is>
-          <t>Existencia</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F622" s="41" t="inlineStr">
         <is>
-          <t>No tenemos gimnasio</t>
+          <t>Jue a sáb 12:00-22:30; domingo 12:00-21:00</t>
         </is>
       </c>
       <c r="G622" s="41" t="inlineStr">
         <is>
-          <t>Espacio dotado para bienestar disponible 24 horas (⚠ Verificar en correo: no menciona ubicación ni precio)</t>
+          <t>Abierto 7/7: lunes a sábado 12:00-22:00; domingos y festivos 12:00-21:00</t>
         </is>
       </c>
     </row>
@@ -34635,27 +34635,27 @@
       </c>
       <c r="C623" s="41" t="inlineStr">
         <is>
-          <t>18-01</t>
+          <t>17-31</t>
         </is>
       </c>
       <c r="D623" s="41" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Fitness gym</t>
         </is>
       </c>
       <c r="E623" s="41" t="inlineStr">
         <is>
-          <t>Horarios</t>
+          <t>Existencia</t>
         </is>
       </c>
       <c r="F623" s="41" t="inlineStr">
         <is>
-          <t>Porterhouse jue-sáb 12:00-22:30, dom 12:00-21:00; Cook's 06:00-10:30</t>
+          <t>No tenemos gimnasio</t>
         </is>
       </c>
       <c r="G623" s="41" t="inlineStr">
         <is>
-          <t>Porterhouse lunes a sábado 12:00-22:00, domingos y festivos 12:00-21:00; Cook's 06:00-12:00</t>
+          <t>Espacio dotado para bienestar disponible 24 horas (⚠ Verificar en correo: no menciona ubicación ni precio)</t>
         </is>
       </c>
     </row>
@@ -34667,32 +34667,32 @@
       </c>
       <c r="B624" s="41" t="inlineStr">
         <is>
-          <t>GHL Relax Hotel Corales de Indias</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C624" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18-01</t>
         </is>
       </c>
       <c r="D624" s="41" t="inlineStr">
         <is>
-          <t>Varios</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="E624" s="41" t="inlineStr">
         <is>
-          <t>Ver adjunto</t>
+          <t>Horarios</t>
         </is>
       </c>
       <c r="F624" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Porterhouse jue-sáb 12:00-22:30, dom 12:00-21:00; Cook's 06:00-10:30</t>
         </is>
       </c>
       <c r="G624" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo (correcciones como anotaciones en 'Corales de Indias (003).pdf')</t>
+          <t>Porterhouse lunes a sábado 12:00-22:00, domingos y festivos 12:00-21:00; Cook's 06:00-12:00</t>
         </is>
       </c>
     </row>
@@ -34704,32 +34704,32 @@
       </c>
       <c r="B625" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>GHL Relax Hotel Corales de Indias</t>
         </is>
       </c>
       <c r="C625" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D625" s="41" t="inlineStr">
         <is>
-          <t>Check-in time</t>
+          <t>Varios</t>
         </is>
       </c>
       <c r="E625" s="41" t="inlineStr">
         <is>
-          <t>Tarifa early check-in (desde 06:00)</t>
+          <t>Ver adjunto</t>
         </is>
       </c>
       <c r="F625" s="41" t="inlineStr">
         <is>
-          <t>40 USD por habitación</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G625" s="41" t="inlineStr">
         <is>
-          <t>50 USD por habitación</t>
+          <t>⚠ Verificar en correo (correcciones como anotaciones en 'Corales de Indias (003).pdf')</t>
         </is>
       </c>
     </row>
@@ -34746,17 +34746,17 @@
       </c>
       <c r="C626" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D626" s="41" t="inlineStr">
         <is>
-          <t>Check-out time</t>
+          <t>Check-in time</t>
         </is>
       </c>
       <c r="E626" s="41" t="inlineStr">
         <is>
-          <t>Tarifa late check-out (hasta 15:00)</t>
+          <t>Tarifa early check-in (desde 06:00)</t>
         </is>
       </c>
       <c r="F626" s="41" t="inlineStr">
@@ -34783,27 +34783,27 @@
       </c>
       <c r="C627" s="41" t="inlineStr">
         <is>
-          <t>13-11</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D627" s="41" t="inlineStr">
         <is>
-          <t>Wifi &amp; Internet</t>
+          <t>Check-out time</t>
         </is>
       </c>
       <c r="E627" s="41" t="inlineStr">
         <is>
-          <t>Velocidad wifi dedicado</t>
+          <t>Tarifa late check-out (hasta 15:00)</t>
         </is>
       </c>
       <c r="F627" s="41" t="inlineStr">
         <is>
-          <t>Wifi dedicado de 60 megas ilimitado</t>
+          <t>40 USD por habitación</t>
         </is>
       </c>
       <c r="G627" s="41" t="inlineStr">
         <is>
-          <t>Wifi dedicado de 100 megas ilimitado</t>
+          <t>50 USD por habitación</t>
         </is>
       </c>
     </row>
@@ -34820,27 +34820,27 @@
       </c>
       <c r="C628" s="41" t="inlineStr">
         <is>
-          <t>13-21</t>
+          <t>13-11</t>
         </is>
       </c>
       <c r="D628" s="41" t="inlineStr">
         <is>
-          <t>Kids</t>
+          <t>Wifi &amp; Internet</t>
         </is>
       </c>
       <c r="E628" s="41" t="inlineStr">
         <is>
-          <t>Tarifa infantil de 13 a 18 años</t>
+          <t>Velocidad wifi dedicado</t>
         </is>
       </c>
       <c r="F628" s="41" t="inlineStr">
         <is>
-          <t>27 USD/noche</t>
+          <t>Wifi dedicado de 60 megas ilimitado</t>
         </is>
       </c>
       <c r="G628" s="41" t="inlineStr">
         <is>
-          <t>32.80 USD/noche</t>
+          <t>Wifi dedicado de 100 megas ilimitado</t>
         </is>
       </c>
     </row>
@@ -34857,27 +34857,27 @@
       </c>
       <c r="C629" s="41" t="inlineStr">
         <is>
-          <t>13-43</t>
+          <t>13-21</t>
         </is>
       </c>
       <c r="D629" s="41" t="inlineStr">
         <is>
-          <t>Laundry</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="E629" s="41" t="inlineStr">
         <is>
-          <t>Horario del servicio</t>
+          <t>Tarifa infantil de 13 a 18 años</t>
         </is>
       </c>
       <c r="F629" s="41" t="inlineStr">
         <is>
-          <t>Objetos dados antes de las 10:00 se devuelven el mismo día antes de las 19:00</t>
+          <t>27 USD/noche</t>
         </is>
       </c>
       <c r="G629" s="41" t="inlineStr">
         <is>
-          <t>Servicio de lavandería desde las 8:00 hasta las 16:00</t>
+          <t>32.80 USD/noche</t>
         </is>
       </c>
     </row>
@@ -34894,27 +34894,27 @@
       </c>
       <c r="C630" s="41" t="inlineStr">
         <is>
-          <t>13-50</t>
+          <t>13-43</t>
         </is>
       </c>
       <c r="D630" s="41" t="inlineStr">
         <is>
-          <t>Airport &amp; train station public transport</t>
+          <t>Laundry</t>
         </is>
       </c>
       <c r="E630" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto</t>
+          <t>Horario del servicio</t>
         </is>
       </c>
       <c r="F630" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto Internacional José Joaquín de Olmedo (GYE), 400 km</t>
+          <t>Objetos dados antes de las 10:00 se devuelven el mismo día antes de las 19:00</t>
         </is>
       </c>
       <c r="G630" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto Ciudad de Catamayo (LOH), Catamayo</t>
+          <t>Servicio de lavandería desde las 8:00 hasta las 16:00</t>
         </is>
       </c>
     </row>
@@ -34926,32 +34926,32 @@
       </c>
       <c r="B631" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cali</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C631" s="41" t="inlineStr">
         <is>
-          <t>15-48</t>
+          <t>13-50</t>
         </is>
       </c>
       <c r="D631" s="41" t="inlineStr">
         <is>
-          <t>Electrical &amp; mobile phone facilities</t>
+          <t>Airport &amp; train station public transport</t>
         </is>
       </c>
       <c r="E631" s="41" t="inlineStr">
         <is>
-          <t>Adaptadores y cargador de móvil</t>
+          <t>Aeropuerto</t>
         </is>
       </c>
       <c r="F631" s="41" t="inlineStr">
         <is>
-          <t>Disponibles gratuitamente</t>
+          <t>Aeropuerto Internacional José Joaquín de Olmedo (GYE), 400 km</t>
         </is>
       </c>
       <c r="G631" s="41" t="inlineStr">
         <is>
-          <t>No disponibles</t>
+          <t>Aeropuerto Ciudad de Catamayo (LOH), Catamayo</t>
         </is>
       </c>
     </row>
@@ -34968,27 +34968,27 @@
       </c>
       <c r="C632" s="41" t="inlineStr">
         <is>
-          <t>16-10</t>
+          <t>15-48</t>
         </is>
       </c>
       <c r="D632" s="41" t="inlineStr">
         <is>
-          <t>Pets</t>
+          <t>Electrical &amp; mobile phone facilities</t>
         </is>
       </c>
       <c r="E632" s="41" t="inlineStr">
         <is>
-          <t>Tasa animal de servicio/apoyo emocional y limpieza</t>
+          <t>Adaptadores y cargador de móvil</t>
         </is>
       </c>
       <c r="F632" s="41" t="inlineStr">
         <is>
-          <t>No es necesario abonar ninguna tasa</t>
+          <t>Disponibles gratuitamente</t>
         </is>
       </c>
       <c r="G632" s="41" t="inlineStr">
         <is>
-          <t>70000 COP/estancia</t>
+          <t>No disponibles</t>
         </is>
       </c>
     </row>
@@ -35005,25 +35005,62 @@
       </c>
       <c r="C633" s="41" t="inlineStr">
         <is>
+          <t>16-10</t>
+        </is>
+      </c>
+      <c r="D633" s="41" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="E633" s="41" t="inlineStr">
+        <is>
+          <t>Tasa animal de servicio/apoyo emocional y limpieza</t>
+        </is>
+      </c>
+      <c r="F633" s="41" t="inlineStr">
+        <is>
+          <t>No es necesario abonar ninguna tasa</t>
+        </is>
+      </c>
+      <c r="G633" s="41" t="inlineStr">
+        <is>
+          <t>70000 COP/estancia</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B634" s="41" t="inlineStr">
+        <is>
+          <t>Sonesta Cali</t>
+        </is>
+      </c>
+      <c r="C634" s="41" t="inlineStr">
+        <is>
           <t>17-34</t>
         </is>
       </c>
-      <c r="D633" s="41" t="inlineStr">
+      <c r="D634" s="41" t="inlineStr">
         <is>
           <t>Rooftop</t>
         </is>
       </c>
-      <c r="E633" s="41" t="inlineStr">
+      <c r="E634" s="41" t="inlineStr">
         <is>
           <t>Existencia del rooftop</t>
         </is>
       </c>
-      <c r="F633" s="41" t="inlineStr">
+      <c r="F634" s="41" t="inlineStr">
         <is>
           <t>Terraza con vistas, abierta todo el año</t>
         </is>
       </c>
-      <c r="G633" s="41" t="inlineStr">
+      <c r="G634" s="41" t="inlineStr">
         <is>
           <t>No disponemos de Rooftop</t>
         </is>

</xml_diff>

<commit_message>
Oct-26: registra Park Lake Luxury (11 cambios) y Geotel Antofagasta (sin cambios)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -454,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -586,6 +586,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -8950,14 +8953,24 @@
           <t>02/10/2026</t>
         </is>
       </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K175" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Reportó sin cambios para octubre</t>
+        </is>
+      </c>
+      <c r="K175" s="48" t="inlineStr">
+        <is>
+          <t>Sin modificaciones</t>
         </is>
       </c>
     </row>
@@ -9941,14 +9954,29 @@
           <t>02/10/2026</t>
         </is>
       </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K198" s="44" t="inlineStr">
-        <is>
-          <t>Sin respuesta</t>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>11 diálogos modificados: contacto eventos, pago en cuotas y online, late check-out, habitaciones, connecting, cama extra, bares</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Diálogo de Eventos sin número en el texto (se asume 16-02). 'Superio Superior' tal como lo escribió el hotel (posible typo). Cierra con: 'quedo atento y a disposición para seguir revisando cualquier otro punto'</t>
+        </is>
+      </c>
+      <c r="K198" s="46" t="inlineStr">
+        <is>
+          <t>Pendiente actualización</t>
         </is>
       </c>
     </row>
@@ -10852,23 +10880,23 @@
         <v>42</v>
       </c>
       <c r="C8" t="n">
+        <v>22</v>
+      </c>
+      <c r="D8" t="n">
         <v>20</v>
       </c>
-      <c r="D8" t="n">
-        <v>22</v>
-      </c>
       <c r="E8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="I8">
@@ -10991,28 +11019,28 @@
         <v>42</v>
       </c>
       <c r="C4" s="19" t="n">
+        <v>22</v>
+      </c>
+      <c r="D4" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="D4" s="19" t="n">
-        <v>22</v>
-      </c>
       <c r="E4" s="19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" s="20" t="n">
-        <v>0.4761904761904762</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>██████████████░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-      <c r="I4" s="52" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>████████████████░░░░░░░░░░░░░░</t>
+        </is>
+      </c>
+      <c r="I4" s="53" t="inlineStr">
+        <is>
+          <t>En progreso</t>
         </is>
       </c>
     </row>
@@ -11166,19 +11194,19 @@
         <v>210</v>
       </c>
       <c r="C9" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D9" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E9" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4857142857142857</v>
+        <v>0.4952380952380953</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -11209,7 +11237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H634"/>
+  <dimension ref="A1:H645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -35063,6 +35091,413 @@
       <c r="G634" s="41" t="inlineStr">
         <is>
           <t>No disponemos de Rooftop</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B635" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C635" s="41" t="inlineStr">
+        <is>
+          <t>16-02 (⚠ sin número en el texto)</t>
+        </is>
+      </c>
+      <c r="D635" s="41" t="inlineStr">
+        <is>
+          <t>Contact staff</t>
+        </is>
+      </c>
+      <c r="E635" s="41" t="inlineStr">
+        <is>
+          <t>Correo de Eventos</t>
+        </is>
+      </c>
+      <c r="F635" s="41" t="inlineStr">
+        <is>
+          <t>carolina.gutierrez@ghlhoteles.com (Tel +56 45 252 7200)</t>
+        </is>
+      </c>
+      <c r="G635" s="41" t="inlineStr">
+        <is>
+          <t>catherinne.zuniga@ghlhoteles.com (el teléfono y el gratuito +56 45 252 7200 no cambian)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B636" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C636" s="41" t="inlineStr">
+        <is>
+          <t>10-71</t>
+        </is>
+      </c>
+      <c r="D636" s="41" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="E636" s="41" t="inlineStr">
+        <is>
+          <t>Pago en cuotas</t>
+        </is>
+      </c>
+      <c r="F636" s="41" t="inlineStr">
+        <is>
+          <t>No aceptamos pago en cuotas</t>
+        </is>
+      </c>
+      <c r="G636" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo: el hotel indica que el texto le queda poco claro; aclarar</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B637" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C637" s="41" t="inlineStr">
+        <is>
+          <t>10-74</t>
+        </is>
+      </c>
+      <c r="D637" s="41" t="inlineStr">
+        <is>
+          <t>Online payment</t>
+        </is>
+      </c>
+      <c r="E637" s="41" t="inlineStr">
+        <is>
+          <t>Pago online</t>
+        </is>
+      </c>
+      <c r="F637" s="41" t="inlineStr">
+        <is>
+          <t>Lo sentimos, no aceptamos pago online</t>
+        </is>
+      </c>
+      <c r="G637" s="41" t="inlineStr">
+        <is>
+          <t>Sí aceptamos pago online, con link de pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B638" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C638" s="41" t="inlineStr">
+        <is>
+          <t>11-12</t>
+        </is>
+      </c>
+      <c r="D638" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="E638" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="F638" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G638" s="41" t="inlineStr">
+        <is>
+          <t>Sí hay opción de late check-out, con cargo del 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B639" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C639" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D639" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E639" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de habitaciones</t>
+        </is>
+      </c>
+      <c r="F639" s="41" t="inlineStr">
+        <is>
+          <t>King Deluxe (39 hab); Deluxe Twin (13 hab); Junior Suite (5 hab); Suite Presidencial (1 hab)</t>
+        </is>
+      </c>
+      <c r="G639" s="41" t="inlineStr">
+        <is>
+          <t>'Superio Superior' (39 hab, ⚠ nombre escrito así, posible typo); Superior Doble Doble (13); Junior Suite King (5); Suite (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B640" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C640" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D640" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E640" s="41" t="inlineStr">
+        <is>
+          <t>Habitaciones nuevas</t>
+        </is>
+      </c>
+      <c r="F640" s="41" t="inlineStr">
+        <is>
+          <t>Sin estos tipos</t>
+        </is>
+      </c>
+      <c r="G640" s="41" t="inlineStr">
+        <is>
+          <t>Agregar: Junior Superior (5 hab); Junior Suite Doble Doble (2 hab); Superior King (5 hab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B641" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C641" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D641" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E641" s="41" t="inlineStr">
+        <is>
+          <t>Total de habitaciones</t>
+        </is>
+      </c>
+      <c r="F641" s="41" t="inlineStr">
+        <is>
+          <t>Incluye la habitación 707</t>
+        </is>
+      </c>
+      <c r="G641" s="41" t="inlineStr">
+        <is>
+          <t>Descontar una habitación: la 707</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B642" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C642" s="41" t="inlineStr">
+        <is>
+          <t>14-02</t>
+        </is>
+      </c>
+      <c r="D642" s="41" t="inlineStr">
+        <is>
+          <t>Connecting &amp; close accommodation</t>
+        </is>
+      </c>
+      <c r="E642" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F642" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G642" s="41" t="inlineStr">
+        <is>
+          <t>Sí disponemos de opciones connecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B643" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C643" s="41" t="inlineStr">
+        <is>
+          <t>15-09, 15-21, 15-61, 17-43</t>
+        </is>
+      </c>
+      <c r="D643" s="41" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="E643" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de habitaciones</t>
+        </is>
+      </c>
+      <c r="F643" s="41" t="inlineStr">
+        <is>
+          <t>Nombres anteriores de habitación</t>
+        </is>
+      </c>
+      <c r="G643" s="41" t="inlineStr">
+        <is>
+          <t>Actualizar los nombres de habitaciones según el punto 14-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B644" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C644" s="41" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="D644" s="41" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="E644" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F644" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G644" s="41" t="inlineStr">
+        <is>
+          <t>Sí tenemos camas adicionales disponibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B645" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C645" s="41" t="inlineStr">
+        <is>
+          <t>17-01</t>
+        </is>
+      </c>
+      <c r="D645" s="41" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="E645" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de los bares</t>
+        </is>
+      </c>
+      <c r="F645" s="41" t="inlineStr">
+        <is>
+          <t>Equilibrium; Vertigo</t>
+        </is>
+      </c>
+      <c r="G645" s="41" t="inlineStr">
+        <is>
+          <t>Equilibrium lobby bar; Bar Lake</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oct-26: completa Sonesta Cartagena con capturas del PDF y confirma Collection 93, Biohotel, Sunrise y Capital
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -8866,7 +8866,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>CONTRADICCIÓN: el 04/10 (Ajustes ChatBot.pdf, respuesta a 'Diálogos desde Junio a la fecha') reportó estos cambios, pero el 18/10 Sofía confirmó 'en orden, no se debe realizar ningún ajuste' — confirmar con ella si siguen vigentes. Números 16-06, 16-10 y 17-43 venían truncados ('6 - 06', '6 - 10', '7 - 43') y se asumieron. 16-02 Eventos: el 'Ahora' viene rotulado Recepción con otro WhatsApp (+57 322 9736615). No respondió la ficha A&amp;B/Spa</t>
+          <t>Cambios del 04/10 (BIOHOT.pdf aportado por el usuario); el 18/10 Sofía había escrito 'en orden, no se debe realizar ningún ajuste' — se registran los cambios del documento. Números 6-06, 6-10 y 7-43 aparecen así en el PDF y se asumieron 16-06, 16-10 y 17-43. 16-02 Eventos: el 'Ahora' viene rotulado Recepción con otro WhatsApp (+57 322 9736615). No respondió la ficha A&amp;B/Spa</t>
         </is>
       </c>
       <c r="K173" s="46" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>Respuesta recibida el 05/10 fuera de la carpeta Octubre (el reenvío del 07/10 solo trae un .eml ilegible). Solo 19-01 traía número; los demás números se infirieron por contenido y orden del PDF — verificar. 13-45: el tiempo a pie sale mal porque el mapa apunta al hotel de Cota (se corrige con 19-01). Posible incoherencia: gimnasio en piso 6 vs '5 pisos' en 17-43</t>
+          <t>Respuesta recibida el 05/10 fuera de la carpeta Octubre; col93.pdf (aportado por el usuario) confirma los números de diálogo con capturas (10-71 y 16-10 sin encabezado visible, inferidos). 13-45: el tiempo a pie sale mal porque el mapa apunta al hotel de Cota (se corrige con 19-01). Posible incoherencia: gimnasio en piso 6 vs '5 pisos' en 17-43</t>
         </is>
       </c>
       <c r="K177" s="46" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>Llegó como reenvío de Valentina Gonzalez (14/10) de un Word enviado por Maira Piza (original 02/10, respuesta a 'Diálogos desde Junio a la fecha'). Desayuno sin número en el docx (se asumen 12-01/12-02). 10-05, 10-08, 10-32 y 10-33 sin valor 'antes'. 14-02 ambiguo ('no contamos con conectadas' pero conserva lista Standard/Twin/Junior Suite). 14-04: pasa de 0 COP a 200 USD, confirmar</t>
+          <t>Llegó como reenvío de Valentina Gonzalez (14/10) de un Word enviado por Maira Piza (original 02/10, respuesta a 'Diálogos desde Junio a la fecha'). Desayuno sin número en el docx (se asumen 12-01/12-02). 10-05, 10-08, 10-32 y 10-33 sin valor 'antes'. 14-02 ambiguo ('no contamos con conectadas' pero conserva lista Standard/Twin/Junior Suite). 14-04: pasa de 0 COP a 200 USD, confirmar CAPI.docx aportado por el usuario: 10-05, 10-08, 10-32 y 10-33 vienen sin marcas Antes/Ahora (texto único), el 'antes' sigue sin confirmar.</t>
         </is>
       </c>
       <c r="K181" s="46" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>Reenvía casi los mismos puntos ya aplicados en Sep-26 (16-02, 10-04, 10-06, 10-41, 10-71, 11-01, 12-01, 13-01, 13-21); solo el diálogo '0-26' (probable typo de 10-26) es nuevo y sin valor 'antes'. El hotel indicó que seguía revisando con calidad, puede llegar un segundo envío. En 10-41 pregunta si puede colocarse el flyer del pasadía en el enlace</t>
+          <t>Reenvía casi los mismos puntos ya aplicados en Sep-26 (16-02, 10-04, 10-06, 10-41, 10-71, 11-01, 12-01, 13-01, 13-21); solo el diálogo '0-26' (probable typo de 10-26) es nuevo y sin valor 'antes'. El hotel indicó que seguía revisando con calidad, puede llegar un segundo envío. En 10-41 pregunta si puede colocarse el flyer del pasadía en el enlace SUNRIS.docx aportado por el usuario coincide con el adjunto del correo (solo texto 'después').</t>
         </is>
       </c>
       <c r="K188" s="46" t="inlineStr">
@@ -10154,12 +10154,12 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Anotaciones sin número de diálogo: pagos, check-in/out, niños, spa, lavandería, transporte, fumadores, camas, mascotas</t>
+          <t>25 diálogos modificados: pagos, check-in/out, desayuno, niños, peluquería, lavandería, traslados, vuelos, fumadores, camas, mascotas, alcohol, actividades, piscina, boutique</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>Liliana respondió con anotaciones sueltas sobre el PDF sin indicar número de diálogo ni 'antes' — los números/campos son inferidos y deben verificarse en el PDF. Kenny Maturana (gerencia) había pedido el 06/10 revisar juntos. Otras anotaciones sin contexto: 'Esto no lo manejamos', 'Esto es sujeto a la disponibilidad', 'Sujeto a disponibilidad', 'Nosotros no prohibimos esto', 'No lo exigimos'. Pregunta sobre pago fraccionado con varias tarjetas: propone plasmar el procedimiento de pagos por WOMPI</t>
+          <t>Liliana respondió con anotaciones sobre capturas del PDF (SONCART.pdf aportado por el usuario). Números tomados de las capturas; '(inferido)' = la captura no mostraba el encabezado; sin número: puertas insonorizadas y horario de piscina; '-44 Alcohol policy' venía truncado. Pregunta abierta: 'Pago por otra persona' (propone plasmar procedimiento de pagos por WOMPI). Kenny Maturana (gerencia) pidió el 06/10 revisar juntos</t>
         </is>
       </c>
       <c r="K202" s="46" t="inlineStr">
@@ -11237,7 +11237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H645"/>
+  <dimension ref="A1:H652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33072,27 +33072,27 @@
       </c>
       <c r="C580" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>10-71 (inferido)</t>
         </is>
       </c>
       <c r="D580" s="41" t="inlineStr">
         <is>
-          <t>Payment method (inferido)</t>
+          <t>Payment method</t>
         </is>
       </c>
       <c r="E580" s="41" t="inlineStr">
         <is>
-          <t>Pago fraccionado con varias tarjetas</t>
+          <t>Pago con varias tarjetas</t>
         </is>
       </c>
       <c r="F580" s="41" t="inlineStr">
         <is>
-          <t>El huésped puede fraccionar su pago con varias tarjetas pagando en Recepción</t>
+          <t>No podemos dividir el pago entre diferentes tarjetas de crédito</t>
         </is>
       </c>
       <c r="G580" s="41" t="inlineStr">
         <is>
-          <t>Hotel pregunta a qué se refiere; propone plasmar el procedimiento de pagos por WOMPI</t>
+          <t>El huésped puede fraccionar su pago con varias tarjetas de crédito pagando en Recepción</t>
         </is>
       </c>
     </row>
@@ -33109,27 +33109,27 @@
       </c>
       <c r="C581" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>10-71 (inferido)</t>
         </is>
       </c>
       <c r="D581" s="41" t="inlineStr">
         <is>
-          <t>Check-in time (inferido)</t>
+          <t>Payment method</t>
         </is>
       </c>
       <c r="E581" s="41" t="inlineStr">
         <is>
-          <t>Early check-in</t>
+          <t>Pago por otra persona</t>
         </is>
       </c>
       <c r="F581" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>No aceptamos pagos hechos por otra persona</t>
         </is>
       </c>
       <c r="G581" s="41" t="inlineStr">
         <is>
-          <t>No cobramos early check-in; se sugiere cambiarlo por Web Check-in para agilizar el registro</t>
+          <t>⚠ Verificar en correo: el hotel pregunta a qué se refiere (¿el que paga debe hospedarse?) y propone plasmar el procedimiento de pagos por WOMPI</t>
         </is>
       </c>
     </row>
@@ -33146,27 +33146,27 @@
       </c>
       <c r="C582" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D582" s="41" t="inlineStr">
         <is>
-          <t>Check-out time (inferido)</t>
+          <t>Check-in time</t>
         </is>
       </c>
       <c r="E582" s="41" t="inlineStr">
         <is>
-          <t>Late check-out</t>
+          <t>Early check-in</t>
         </is>
       </c>
       <c r="F582" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Check-in anticipado desde las 12:00 por 50% adicional del precio de la habitación</t>
         </is>
       </c>
       <c r="G582" s="41" t="inlineStr">
         <is>
-          <t>Cada hora de late check-out cuesta 20.000 + impuestos, sujeta a disponibilidad</t>
+          <t>No cobramos early check-in</t>
         </is>
       </c>
     </row>
@@ -33183,27 +33183,27 @@
       </c>
       <c r="C583" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>11-03</t>
         </is>
       </c>
       <c r="D583" s="41" t="inlineStr">
         <is>
-          <t>Breakfast (inferido)</t>
+          <t>Online check-in</t>
         </is>
       </c>
       <c r="E583" s="41" t="inlineStr">
         <is>
-          <t>Reserva de desayuno</t>
+          <t>Check-in online</t>
         </is>
       </c>
       <c r="F583" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Lamentablemente, no ofrecemos la posibilidad de check-in online</t>
         </is>
       </c>
       <c r="G583" s="41" t="inlineStr">
         <is>
-          <t>No es necesario reservar para el desayuno</t>
+          <t>Cambiarlo por Web Check-in para agilizar el registro en recepción (texto nuevo no indicado)</t>
         </is>
       </c>
     </row>
@@ -33220,27 +33220,27 @@
       </c>
       <c r="C584" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D584" s="41" t="inlineStr">
         <is>
-          <t>Cancellation policy (inferido)</t>
+          <t>Check-out time</t>
         </is>
       </c>
       <c r="E584" s="41" t="inlineStr">
         <is>
-          <t>Condición</t>
+          <t>Tarifa late check-out</t>
         </is>
       </c>
       <c r="F584" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Late check-out hasta las 15:00 por 50% adicional del precio de la habitación</t>
         </is>
       </c>
       <c r="G584" s="41" t="inlineStr">
         <is>
-          <t>No reembolsable e intransferible</t>
+          <t>Cada hora de late check-out cuesta 20.000 + impuestos, sujeta a disponibilidad</t>
         </is>
       </c>
     </row>
@@ -33257,27 +33257,27 @@
       </c>
       <c r="C585" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>12-04</t>
         </is>
       </c>
       <c r="D585" s="41" t="inlineStr">
         <is>
-          <t>Kids (inferido)</t>
+          <t>Breakfast reservation</t>
         </is>
       </c>
       <c r="E585" s="41" t="inlineStr">
         <is>
-          <t>Tarifa niño</t>
+          <t>Reserva de desayuno</t>
         </is>
       </c>
       <c r="F585" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Realice su reserva para el desayuno en el siguiente link</t>
         </is>
       </c>
       <c r="G585" s="41" t="inlineStr">
         <is>
-          <t>65.000 + impuestos por noche</t>
+          <t>No es necesario reservar para el desayuno</t>
         </is>
       </c>
     </row>
@@ -33294,27 +33294,27 @@
       </c>
       <c r="C586" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>12-06</t>
         </is>
       </c>
       <c r="D586" s="41" t="inlineStr">
         <is>
-          <t>Spa (inferido)</t>
+          <t>Breakfast refundable</t>
         </is>
       </c>
       <c r="E586" s="41" t="inlineStr">
         <is>
-          <t>Peluquería</t>
+          <t>Reembolso</t>
         </is>
       </c>
       <c r="F586" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>El desayuno no es reembolsable</t>
         </is>
       </c>
       <c r="G586" s="41" t="inlineStr">
         <is>
-          <t>Spa que ofrece peluquería es externo</t>
+          <t>No reembolsable e intransferible</t>
         </is>
       </c>
     </row>
@@ -33331,27 +33331,27 @@
       </c>
       <c r="C587" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-21 (inferido)</t>
         </is>
       </c>
       <c r="D587" s="41" t="inlineStr">
         <is>
-          <t>Laundry (inferido)</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="E587" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Tarifa infantil 5-11 años</t>
         </is>
       </c>
       <c r="F587" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>50000 COP/noche</t>
         </is>
       </c>
       <c r="G587" s="41" t="inlineStr">
         <is>
-          <t>Prendas antes de las 10:00 am se entregan después de las 6:00 pm del mismo día</t>
+          <t>65.000 + impuestos por noche</t>
         </is>
       </c>
     </row>
@@ -33368,27 +33368,27 @@
       </c>
       <c r="C588" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-33</t>
         </is>
       </c>
       <c r="D588" s="41" t="inlineStr">
         <is>
-          <t>Airport transfer (inferido)</t>
+          <t>Hairdresser</t>
         </is>
       </c>
       <c r="E588" s="41" t="inlineStr">
         <is>
-          <t>Recogida internacional</t>
+          <t>Peluquería</t>
         </is>
       </c>
       <c r="F588" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>No disponemos de peluquería dentro de la propiedad</t>
         </is>
       </c>
       <c r="G588" s="41" t="inlineStr">
         <is>
-          <t>Tarifa 55.000</t>
+          <t>Tenemos un spa que ofrece servicio de peluquería, es externo</t>
         </is>
       </c>
     </row>
@@ -33405,27 +33405,27 @@
       </c>
       <c r="C589" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-43</t>
         </is>
       </c>
       <c r="D589" s="41" t="inlineStr">
         <is>
-          <t>Transport (inferido)</t>
+          <t>Laundry</t>
         </is>
       </c>
       <c r="E589" s="41" t="inlineStr">
         <is>
-          <t>Empresa de transporte</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F589" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Objetos dados antes de las 08:00 se devuelven el mismo día antes de las 08:00</t>
         </is>
       </c>
       <c r="G589" s="41" t="inlineStr">
         <is>
-          <t>KEMUEL, contacto 316 4115808</t>
+          <t>Se reciben prendas antes de las 10:00 am y se entregan después de las 6:00 pm del mismo día</t>
         </is>
       </c>
     </row>
@@ -33442,27 +33442,27 @@
       </c>
       <c r="C590" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-51</t>
         </is>
       </c>
       <c r="D590" s="41" t="inlineStr">
         <is>
-          <t>Smoking (inferido)</t>
+          <t>Private transfer</t>
         </is>
       </c>
       <c r="E590" s="41" t="inlineStr">
         <is>
-          <t>Multa</t>
+          <t>Recogida internacional</t>
         </is>
       </c>
       <c r="F590" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Transfer aeropuerto-hotel $40.000 COP hasta 3 personas (nacionales o internacionales); hotel-aeropuerto $25.000</t>
         </is>
       </c>
       <c r="G590" s="41" t="inlineStr">
         <is>
-          <t>Multa por fumar en habitaciones: 200 USD</t>
+          <t>Recogida internacional tarifa de 55.000</t>
         </is>
       </c>
     </row>
@@ -33479,27 +33479,27 @@
       </c>
       <c r="C591" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-55</t>
         </is>
       </c>
       <c r="D591" s="41" t="inlineStr">
         <is>
-          <t>Bedding (inferido)</t>
+          <t>Shuttle</t>
         </is>
       </c>
       <c r="E591" s="41" t="inlineStr">
         <is>
-          <t>Medidas de camas</t>
+          <t>Contacto de transporte</t>
         </is>
       </c>
       <c r="F591" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>No ofrecemos servicios de traslado</t>
         </is>
       </c>
       <c r="G591" s="41" t="inlineStr">
         <is>
-          <t>Standard y Superior King 2.00x2.00; Standard y Superior Twin 1.90x1.40; Standard Queen 1.90x1.60 a 1.90x1.80</t>
+          <t>Colocar el contacto de la empresa de transporte: KEMUEL, 316 4115808</t>
         </is>
       </c>
     </row>
@@ -33516,27 +33516,27 @@
       </c>
       <c r="C592" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>13-61</t>
         </is>
       </c>
       <c r="D592" s="41" t="inlineStr">
         <is>
-          <t>Soundproofing (inferido)</t>
+          <t>Flight, hotel packages, airlines &amp; airports</t>
         </is>
       </c>
       <c r="E592" s="41" t="inlineStr">
         <is>
-          <t>Puertas</t>
+          <t>Paquetes vuelo + hotel</t>
         </is>
       </c>
       <c r="F592" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Contamos con paquetes de vuelo + hotel para Colombia y Perú</t>
         </is>
       </c>
       <c r="G592" s="41" t="inlineStr">
         <is>
-          <t>Las puertas de las habitaciones NO son insonorizadas</t>
+          <t>Esto no lo manejamos (retirar)</t>
         </is>
       </c>
     </row>
@@ -33553,27 +33553,27 @@
       </c>
       <c r="C593" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>15-99 (inferido)</t>
         </is>
       </c>
       <c r="D593" s="41" t="inlineStr">
         <is>
-          <t>Floor arrangement (inferido)</t>
+          <t>Specific room request</t>
         </is>
       </c>
       <c r="E593" s="41" t="inlineStr">
         <is>
-          <t>Pisos altos</t>
+          <t>Solicitud de habitación</t>
         </is>
       </c>
       <c r="F593" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Solicitud por correo a calidad.sonestacartagena y reservas.sonestacartagena</t>
         </is>
       </c>
       <c r="G593" s="41" t="inlineStr">
         <is>
-          <t>Los pisos altos son sujetos a disponibilidad</t>
+          <t>Esto es sujeto a la disponibilidad</t>
         </is>
       </c>
     </row>
@@ -33590,27 +33590,27 @@
       </c>
       <c r="C594" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>14-04</t>
         </is>
       </c>
       <c r="D594" s="41" t="inlineStr">
         <is>
-          <t>Pets (inferido)</t>
+          <t>Smoking</t>
         </is>
       </c>
       <c r="E594" s="41" t="inlineStr">
         <is>
-          <t>Tarifa</t>
+          <t>Tarifa por fumar</t>
         </is>
       </c>
       <c r="F594" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Tarifa por limpieza de humo 0 COP</t>
         </is>
       </c>
       <c r="G594" s="41" t="inlineStr">
         <is>
-          <t>90.000 + impuestos por noche; animal de apoyo emocional sin cobro con documentación médica</t>
+          <t>Multa por fumar en las habitaciones de 200 USD</t>
         </is>
       </c>
     </row>
@@ -33627,27 +33627,27 @@
       </c>
       <c r="C595" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>15-21</t>
         </is>
       </c>
       <c r="D595" s="41" t="inlineStr">
         <is>
-          <t>Entertainment (inferido)</t>
+          <t>Bedding, pillow, mattress</t>
         </is>
       </c>
       <c r="E595" s="41" t="inlineStr">
         <is>
-          <t>Actividades</t>
+          <t>Medidas de camas</t>
         </is>
       </c>
       <c r="F595" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Estándar King: queen 200x160 + king 200x180 + extra king 200x200; Estándar Twin 2 dobles 200x140; Junior Suite king 200x180; King superior king 200x180; Twin superior doble 200x140</t>
         </is>
       </c>
       <c r="G595" s="41" t="inlineStr">
         <is>
-          <t>No tienen; solo piscina, bar y cancha de tenis</t>
+          <t>Standard y Superior King: king size 2.00x2.00; Standard y Superior Twin: dobles 1.90x1.40; Standard Queen: 1.90x1.60 a 1.90x1.80</t>
         </is>
       </c>
     </row>
@@ -33664,27 +33664,27 @@
       </c>
       <c r="C596" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>15-23</t>
         </is>
       </c>
       <c r="D596" s="41" t="inlineStr">
         <is>
-          <t>Horario (inferido)</t>
+          <t>Extra bed</t>
         </is>
       </c>
       <c r="E596" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Condición</t>
         </is>
       </c>
       <c r="F596" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Sí, con mucho gusto le podemos agregar una cama extra gratuitamente</t>
         </is>
       </c>
       <c r="G596" s="41" t="inlineStr">
         <is>
-          <t>8 am hasta las 8 pm</t>
+          <t>Sujeto a disponibilidad</t>
         </is>
       </c>
     </row>
@@ -33701,27 +33701,27 @@
       </c>
       <c r="C597" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>⚠ sin número</t>
         </is>
       </c>
       <c r="D597" s="41" t="inlineStr">
         <is>
-          <t>Boutique (inferido)</t>
+          <t>Soundproofing</t>
         </is>
       </c>
       <c r="E597" s="41" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Puertas</t>
         </is>
       </c>
       <c r="F597" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Puertas insonorizadas</t>
         </is>
       </c>
       <c r="G597" s="41" t="inlineStr">
         <is>
-          <t>Hay una boutique, pero es externa</t>
+          <t>Las puertas de las habitaciones NO son insonorizadas</t>
         </is>
       </c>
     </row>
@@ -33733,32 +33733,32 @@
       </c>
       <c r="B598" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C598" s="41" t="inlineStr">
         <is>
-          <t>13-11</t>
+          <t>17-43 (inferido)</t>
         </is>
       </c>
       <c r="D598" s="41" t="inlineStr">
         <is>
-          <t>Wifi &amp; Internet</t>
+          <t>Floor arrangement &amp; elevator</t>
         </is>
       </c>
       <c r="E598" s="41" t="inlineStr">
         <is>
-          <t>Cobertura piscina/playa y Ethernet</t>
+          <t>Pisos altos</t>
         </is>
       </c>
       <c r="F598" s="41" t="inlineStr">
         <is>
-          <t>Incluía 'las áreas de piscina y playa no tienen cobertura Wifi' y 'Ethernet (no se proporciona el cable)'</t>
+          <t>Pisos superiores (Standard King, Standard Twin, Junior Suite, Superior King y Superior Twin)</t>
         </is>
       </c>
       <c r="G598" s="41" t="inlineStr">
         <is>
-          <t>Se elimina la línea de piscina/playa; queda 'También hay conexión Ethernet en las habitaciones'</t>
+          <t>Los pisos altos son sujetos a disponibilidad</t>
         </is>
       </c>
     </row>
@@ -33770,32 +33770,32 @@
       </c>
       <c r="B599" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C599" s="41" t="inlineStr">
         <is>
-          <t>13-43</t>
+          <t>16-10 (inferido)</t>
         </is>
       </c>
       <c r="D599" s="41" t="inlineStr">
         <is>
-          <t>Laundry</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="E599" s="41" t="inlineStr">
         <is>
-          <t>Hora de devolución</t>
+          <t>Tarifa mascotas</t>
         </is>
       </c>
       <c r="F599" s="41" t="inlineStr">
         <is>
-          <t>Devuelve el mismo día antes de las 10:00</t>
+          <t>90000 COP/mascota; animal de apoyo emocional sin tasa</t>
         </is>
       </c>
       <c r="G599" s="41" t="inlineStr">
         <is>
-          <t>Devuelve el mismo día pasadas las 6:00 pm</t>
+          <t>90.000 + impuestos por noche; apoyo emocional no genera cobro y requiere documentación médica de entidades legalmente constituidas</t>
         </is>
       </c>
     </row>
@@ -33807,32 +33807,32 @@
       </c>
       <c r="B600" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C600" s="41" t="inlineStr">
         <is>
-          <t>15-06</t>
+          <t>⚠ '-44' (truncado)</t>
         </is>
       </c>
       <c r="D600" s="41" t="inlineStr">
         <is>
-          <t>Bathroom equipment</t>
+          <t>Alcohol policy</t>
         </is>
       </c>
       <c r="E600" s="41" t="inlineStr">
         <is>
-          <t>Artículos gratis a petición</t>
+          <t>Consumo de alcohol</t>
         </is>
       </c>
       <c r="F600" s="41" t="inlineStr">
         <is>
-          <t>Pantuflas, kit de afeitar, cepillo para el pelo y costurero</t>
+          <t>El consumo de alcohol está prohibido en habitaciones y zonas comunes, excepto en el restaurante</t>
         </is>
       </c>
       <c r="G600" s="41" t="inlineStr">
         <is>
-          <t>Pantuflas, kit de afeitar, kit dental y costurero</t>
+          <t>Nosotros no prohibimos esto</t>
         </is>
       </c>
     </row>
@@ -33844,32 +33844,32 @@
       </c>
       <c r="B601" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C601" s="41" t="inlineStr">
         <is>
-          <t>15-09</t>
+          <t>17-20</t>
         </is>
       </c>
       <c r="D601" s="41" t="inlineStr">
         <is>
-          <t>Shower, bathtub, jacuzzi, pool</t>
+          <t>Sport activities &amp; equipments</t>
         </is>
       </c>
       <c r="E601" s="41" t="inlineStr">
         <is>
-          <t>Junior Suite</t>
+          <t>Actividades</t>
         </is>
       </c>
       <c r="F601" s="41" t="inlineStr">
         <is>
-          <t>Junior Suite tiene ducha y bañera</t>
+          <t>Ofrecemos diversas actividades y entretenimiento</t>
         </is>
       </c>
       <c r="G601" s="41" t="inlineStr">
         <is>
-          <t>Junior Suite tiene ducha</t>
+          <t>NO tenemos esto, solo piscina, bar y cancha de tenis</t>
         </is>
       </c>
     </row>
@@ -33881,32 +33881,32 @@
       </c>
       <c r="B602" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C602" s="41" t="inlineStr">
         <is>
-          <t>16-06</t>
+          <t>17-61 (inferido)</t>
         </is>
       </c>
       <c r="D602" s="41" t="inlineStr">
         <is>
-          <t>Jobs &amp; internships</t>
+          <t>Swimming pool</t>
         </is>
       </c>
       <c r="E602" s="41" t="inlineStr">
         <is>
-          <t>Contacto RRHH</t>
+          <t>Gorro de baño</t>
         </is>
       </c>
       <c r="F602" s="41" t="inlineStr">
         <is>
-          <t>contactenos@ghlhoteles.com / +57 601 3139330</t>
+          <t>Gorro de baño: obligatorio</t>
         </is>
       </c>
       <c r="G602" s="41" t="inlineStr">
         <is>
-          <t>laydy.pauca@ghlhoteles.com / +51 945 739 960</t>
+          <t>No lo exigimos</t>
         </is>
       </c>
     </row>
@@ -33918,32 +33918,32 @@
       </c>
       <c r="B603" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C603" s="41" t="inlineStr">
         <is>
-          <t>16-25</t>
+          <t>⚠ sin número</t>
         </is>
       </c>
       <c r="D603" s="41" t="inlineStr">
         <is>
-          <t>Tips policy</t>
+          <t>Swimming pool hours</t>
         </is>
       </c>
       <c r="E603" s="41" t="inlineStr">
         <is>
-          <t>Política de propinas</t>
+          <t>Horario piscina</t>
         </is>
       </c>
       <c r="F603" s="41" t="inlineStr">
         <is>
-          <t>Incluía 'es costumbre dejar propina'</t>
+          <t>Abierto todos los días 08:00 - 22:00</t>
         </is>
       </c>
       <c r="G603" s="41" t="inlineStr">
         <is>
-          <t>Se elimina esa línea</t>
+          <t>8 am hasta las 8 pm</t>
         </is>
       </c>
     </row>
@@ -33955,32 +33955,32 @@
       </c>
       <c r="B604" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Arequipa</t>
+          <t>Sonesta Cartagena</t>
         </is>
       </c>
       <c r="C604" s="41" t="inlineStr">
         <is>
-          <t>18-01 (⚠ escrito '8-01' / '18 -01')</t>
+          <t>17-91</t>
         </is>
       </c>
       <c r="D604" s="41" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="E604" s="41" t="inlineStr">
         <is>
-          <t>Descripción restaurante Micaela</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="F604" s="41" t="inlineStr">
         <is>
-          <t>Incluía tipo de cocina, rango de precios, edad de niños, capacidad 45, tronas y código de vestimenta</t>
+          <t>No disponemos de tienda en las instalaciones</t>
         </is>
       </c>
       <c r="G604" s="41" t="inlineStr">
         <is>
-          <t>Descripción simplificada (abierto todo el año, 06:00-22:00, silla de ruedas, sin mascotas); texto duplicado en el correo</t>
+          <t>Hay una boutique, pero es externa</t>
         </is>
       </c>
     </row>
@@ -33992,32 +33992,32 @@
       </c>
       <c r="B605" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C605" s="41" t="inlineStr">
         <is>
-          <t>11-31</t>
+          <t>13-11</t>
         </is>
       </c>
       <c r="D605" s="41" t="inlineStr">
         <is>
-          <t>Front desk</t>
+          <t>Wifi &amp; Internet</t>
         </is>
       </c>
       <c r="E605" s="41" t="inlineStr">
         <is>
-          <t>Horario recepción</t>
+          <t>Cobertura piscina/playa y Ethernet</t>
         </is>
       </c>
       <c r="F605" s="41" t="inlineStr">
         <is>
-          <t>06:00 a 17:00</t>
+          <t>Incluía 'las áreas de piscina y playa no tienen cobertura Wifi' y 'Ethernet (no se proporciona el cable)'</t>
         </is>
       </c>
       <c r="G605" s="41" t="inlineStr">
         <is>
-          <t>24/7</t>
+          <t>Se elimina la línea de piscina/playa; queda 'También hay conexión Ethernet en las habitaciones'</t>
         </is>
       </c>
     </row>
@@ -34029,32 +34029,32 @@
       </c>
       <c r="B606" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C606" s="41" t="inlineStr">
         <is>
-          <t>12-01</t>
+          <t>13-43</t>
         </is>
       </c>
       <c r="D606" s="41" t="inlineStr">
         <is>
-          <t>Breakfast time</t>
+          <t>Laundry</t>
         </is>
       </c>
       <c r="E606" s="41" t="inlineStr">
         <is>
-          <t>Nombre restaurante (ortografía)</t>
+          <t>Hora de devolución</t>
         </is>
       </c>
       <c r="F606" s="41" t="inlineStr">
         <is>
-          <t>Restaurante Bornón</t>
+          <t>Devuelve el mismo día antes de las 10:00</t>
         </is>
       </c>
       <c r="G606" s="41" t="inlineStr">
         <is>
-          <t>Restaurante Borbón</t>
+          <t>Devuelve el mismo día pasadas las 6:00 pm</t>
         </is>
       </c>
     </row>
@@ -34066,32 +34066,32 @@
       </c>
       <c r="B607" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C607" s="41" t="inlineStr">
         <is>
-          <t>12-02</t>
+          <t>15-06</t>
         </is>
       </c>
       <c r="D607" s="41" t="inlineStr">
         <is>
-          <t>Breakfast rates</t>
+          <t>Bathroom equipment</t>
         </is>
       </c>
       <c r="E607" s="41" t="inlineStr">
         <is>
-          <t>Precio adulto y niño</t>
+          <t>Artículos gratis a petición</t>
         </is>
       </c>
       <c r="F607" s="41" t="inlineStr">
         <is>
-          <t>Adulto 35000 COP; niños 28000 COP</t>
+          <t>Pantuflas, kit de afeitar, cepillo para el pelo y costurero</t>
         </is>
       </c>
       <c r="G607" s="41" t="inlineStr">
         <is>
-          <t>Adulto 33.000 COP; niños 33.000 COP</t>
+          <t>Pantuflas, kit de afeitar, kit dental y costurero</t>
         </is>
       </c>
     </row>
@@ -34103,32 +34103,32 @@
       </c>
       <c r="B608" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C608" s="41" t="inlineStr">
         <is>
-          <t>13-01</t>
+          <t>15-09</t>
         </is>
       </c>
       <c r="D608" s="41" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Shower, bathtub, jacuzzi, pool</t>
         </is>
       </c>
       <c r="E608" s="41" t="inlineStr">
         <is>
-          <t>Parqueadero externo</t>
+          <t>Junior Suite</t>
         </is>
       </c>
       <c r="F608" s="41" t="inlineStr">
         <is>
-          <t>No tenemos parking</t>
+          <t>Junior Suite tiene ducha y bañera</t>
         </is>
       </c>
       <c r="G608" s="41" t="inlineStr">
         <is>
-          <t>Parking externo con tarifa especial para huéspedes $14.000 COP por día</t>
+          <t>Junior Suite tiene ducha</t>
         </is>
       </c>
     </row>
@@ -34140,32 +34140,32 @@
       </c>
       <c r="B609" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C609" s="41" t="inlineStr">
         <is>
-          <t>13-11</t>
+          <t>16-06</t>
         </is>
       </c>
       <c r="D609" s="41" t="inlineStr">
         <is>
-          <t>Wifi &amp; Internet</t>
+          <t>Jobs &amp; internships</t>
         </is>
       </c>
       <c r="E609" s="41" t="inlineStr">
         <is>
-          <t>Alta velocidad</t>
+          <t>Contacto RRHH</t>
         </is>
       </c>
       <c r="F609" s="41" t="inlineStr">
         <is>
-          <t>No hay internet de alta velocidad; sin cobertura en piscina/playa</t>
+          <t>contactenos@ghlhoteles.com / +57 601 3139330</t>
         </is>
       </c>
       <c r="G609" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo: 'hay internet de alta velocidad'; se elimina la línea de piscina/playa</t>
+          <t>laydy.pauca@ghlhoteles.com / +51 945 739 960</t>
         </is>
       </c>
     </row>
@@ -34177,32 +34177,32 @@
       </c>
       <c r="B610" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C610" s="41" t="inlineStr">
         <is>
-          <t>13-41</t>
+          <t>16-25</t>
         </is>
       </c>
       <c r="D610" s="41" t="inlineStr">
         <is>
-          <t>Concierge</t>
+          <t>Tips policy</t>
         </is>
       </c>
       <c r="E610" s="41" t="inlineStr">
         <is>
-          <t>Servicio</t>
+          <t>Política de propinas</t>
         </is>
       </c>
       <c r="F610" s="41" t="inlineStr">
         <is>
-          <t>Conserje 08:00-22:00, inglés y español</t>
+          <t>Incluía 'es costumbre dejar propina'</t>
         </is>
       </c>
       <c r="G610" s="41" t="inlineStr">
         <is>
-          <t>No ofrecemos servicio de conserje</t>
+          <t>Se elimina esa línea</t>
         </is>
       </c>
     </row>
@@ -34214,32 +34214,32 @@
       </c>
       <c r="B611" s="41" t="inlineStr">
         <is>
-          <t>GHL Hotel Abadía Plaza</t>
+          <t>Sonesta Arequipa</t>
         </is>
       </c>
       <c r="C611" s="41" t="inlineStr">
         <is>
-          <t>13-50</t>
+          <t>18-01 (⚠ escrito '8-01' / '18 -01')</t>
         </is>
       </c>
       <c r="D611" s="41" t="inlineStr">
         <is>
-          <t>Airport &amp; train station public transport</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="E611" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto</t>
+          <t>Descripción restaurante Micaela</t>
         </is>
       </c>
       <c r="F611" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto Internacional Rafael Núñez (CTG), 938 km</t>
+          <t>Incluía tipo de cocina, rango de precios, edad de niños, capacidad 45, tronas y código de vestimenta</t>
         </is>
       </c>
       <c r="G611" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo: 'Aeropuerto Internacional Matecaña' (texto cortado, falta distancia)</t>
+          <t>Descripción simplificada (abierto todo el año, 06:00-22:00, silla de ruedas, sin mascotas); texto duplicado en el correo</t>
         </is>
       </c>
     </row>
@@ -34256,27 +34256,27 @@
       </c>
       <c r="C612" s="41" t="inlineStr">
         <is>
-          <t>17-01</t>
+          <t>11-31</t>
         </is>
       </c>
       <c r="D612" s="41" t="inlineStr">
         <is>
-          <t>Bar</t>
+          <t>Front desk</t>
         </is>
       </c>
       <c r="E612" s="41" t="inlineStr">
         <is>
-          <t>Contenido</t>
+          <t>Horario recepción</t>
         </is>
       </c>
       <c r="F612" s="41" t="inlineStr">
         <is>
-          <t>No tenemos bar en el hotel</t>
+          <t>06:00 a 17:00</t>
         </is>
       </c>
       <c r="G612" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo: 'Contamos con espacios para trabajar: Coworking en el lobby y Café Lobby'</t>
+          <t>24/7</t>
         </is>
       </c>
     </row>
@@ -34293,27 +34293,27 @@
       </c>
       <c r="C613" s="41" t="inlineStr">
         <is>
-          <t>17-15</t>
+          <t>12-01</t>
         </is>
       </c>
       <c r="D613" s="41" t="inlineStr">
         <is>
-          <t>Spa hours</t>
+          <t>Breakfast time</t>
         </is>
       </c>
       <c r="E613" s="41" t="inlineStr">
         <is>
-          <t>Existencia del spa</t>
+          <t>Nombre restaurante (ortografía)</t>
         </is>
       </c>
       <c r="F613" s="41" t="inlineStr">
         <is>
-          <t>Spa 1 abierto todo el año, todos los días</t>
+          <t>Restaurante Bornón</t>
         </is>
       </c>
       <c r="G613" s="41" t="inlineStr">
         <is>
-          <t>No tenemos servicio de spa</t>
+          <t>Restaurante Borbón</t>
         </is>
       </c>
     </row>
@@ -34330,27 +34330,27 @@
       </c>
       <c r="C614" s="41" t="inlineStr">
         <is>
-          <t>18-08</t>
+          <t>12-02</t>
         </is>
       </c>
       <c r="D614" s="41" t="inlineStr">
         <is>
-          <t>Takeaway &amp; delivery</t>
+          <t>Breakfast rates</t>
         </is>
       </c>
       <c r="E614" s="41" t="inlineStr">
         <is>
-          <t>Domicilio</t>
+          <t>Precio adulto y niño</t>
         </is>
       </c>
       <c r="F614" s="41" t="inlineStr">
         <is>
-          <t>Domicilio 8h-18h previa solicitud, con cobro adicional</t>
+          <t>Adulto 35000 COP; niños 28000 COP</t>
         </is>
       </c>
       <c r="G614" s="41" t="inlineStr">
         <is>
-          <t>No tenemos domiciliario disponible</t>
+          <t>Adulto 33.000 COP; niños 33.000 COP</t>
         </is>
       </c>
     </row>
@@ -34367,27 +34367,27 @@
       </c>
       <c r="C615" s="41" t="inlineStr">
         <is>
-          <t>19-03</t>
+          <t>13-01</t>
         </is>
       </c>
       <c r="D615" s="41" t="inlineStr">
         <is>
-          <t>City center</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="E615" s="41" t="inlineStr">
         <is>
-          <t>Distancia al centro</t>
+          <t>Parqueadero externo</t>
         </is>
       </c>
       <c r="F615" s="41" t="inlineStr">
         <is>
-          <t>A 142 km del centro</t>
+          <t>No tenemos parking</t>
         </is>
       </c>
       <c r="G615" s="41" t="inlineStr">
         <is>
-          <t>A 2 cuadras del centro</t>
+          <t>Parking externo con tarifa especial para huéspedes $14.000 COP por día</t>
         </is>
       </c>
     </row>
@@ -34404,27 +34404,27 @@
       </c>
       <c r="C616" s="41" t="inlineStr">
         <is>
-          <t>20-21</t>
+          <t>13-11</t>
         </is>
       </c>
       <c r="D616" s="41" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>Wifi &amp; Internet</t>
         </is>
       </c>
       <c r="E616" s="41" t="inlineStr">
         <is>
-          <t>Correo y teléfono eventos</t>
+          <t>Alta velocidad</t>
         </is>
       </c>
       <c r="F616" s="41" t="inlineStr">
         <is>
-          <t>camila.dickens@ghlhoteles.com; +57 324 4547171</t>
+          <t>No hay internet de alta velocidad; sin cobertura en piscina/playa</t>
         </is>
       </c>
       <c r="G616" s="41" t="inlineStr">
         <is>
-          <t>eventos.abadiaplaza@ghlhoteles.com; +57 311 311 51 16</t>
+          <t>⚠ Verificar en correo: 'hay internet de alta velocidad'; se elimina la línea de piscina/playa</t>
         </is>
       </c>
     </row>
@@ -34436,32 +34436,32 @@
       </c>
       <c r="B617" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C617" s="41" t="inlineStr">
         <is>
-          <t>12-01</t>
+          <t>13-41</t>
         </is>
       </c>
       <c r="D617" s="41" t="inlineStr">
         <is>
-          <t>Breakfast time</t>
+          <t>Concierge</t>
         </is>
       </c>
       <c r="E617" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Servicio</t>
         </is>
       </c>
       <c r="F617" s="41" t="inlineStr">
         <is>
-          <t>Todos los días 06:00-10:00 y 06:30-10:30 fines de semana</t>
+          <t>Conserje 08:00-22:00, inglés y español</t>
         </is>
       </c>
       <c r="G617" s="41" t="inlineStr">
         <is>
-          <t>Lunes a viernes 06:00-10:00; sábados, domingos y festivos 06:30-10:30</t>
+          <t>No ofrecemos servicio de conserje</t>
         </is>
       </c>
     </row>
@@ -34473,32 +34473,32 @@
       </c>
       <c r="B618" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C618" s="41" t="inlineStr">
         <is>
-          <t>13-17</t>
+          <t>13-50</t>
         </is>
       </c>
       <c r="D618" s="41" t="inlineStr">
         <is>
-          <t>Special requests</t>
+          <t>Airport &amp; train station public transport</t>
         </is>
       </c>
       <c r="E618" s="41" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Aeropuerto</t>
         </is>
       </c>
       <c r="F618" s="41" t="inlineStr">
         <is>
-          <t>Pedimos disculpas por no poder atender peticiones especiales</t>
+          <t>Aeropuerto Internacional Rafael Núñez (CTG), 938 km</t>
         </is>
       </c>
       <c r="G618" s="41" t="inlineStr">
         <is>
-          <t>Puede contactarnos al correo reservas.sonestabogota@ghlhoteles.com</t>
+          <t>⚠ Verificar en correo: 'Aeropuerto Internacional Matecaña' (texto cortado, falta distancia)</t>
         </is>
       </c>
     </row>
@@ -34510,32 +34510,32 @@
       </c>
       <c r="B619" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C619" s="41" t="inlineStr">
         <is>
-          <t>14-04</t>
+          <t>17-01</t>
         </is>
       </c>
       <c r="D619" s="41" t="inlineStr">
         <is>
-          <t>Smoking</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="E619" s="41" t="inlineStr">
         <is>
-          <t>Tarifa limpieza por humo</t>
+          <t>Contenido</t>
         </is>
       </c>
       <c r="F619" s="41" t="inlineStr">
         <is>
-          <t>350000 COP</t>
+          <t>No tenemos bar en el hotel</t>
         </is>
       </c>
       <c r="G619" s="41" t="inlineStr">
         <is>
-          <t>Desodorización equivalente a USD 100 diarios, al cambio de la TRM del día</t>
+          <t>⚠ Verificar en correo: 'Contamos con espacios para trabajar: Coworking en el lobby y Café Lobby'</t>
         </is>
       </c>
     </row>
@@ -34547,32 +34547,32 @@
       </c>
       <c r="B620" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C620" s="41" t="inlineStr">
         <is>
-          <t>15-06</t>
+          <t>17-15</t>
         </is>
       </c>
       <c r="D620" s="41" t="inlineStr">
         <is>
-          <t>Bathroom equipment</t>
+          <t>Spa hours</t>
         </is>
       </c>
       <c r="E620" s="41" t="inlineStr">
         <is>
-          <t>Artículos a solicitud</t>
+          <t>Existencia del spa</t>
         </is>
       </c>
       <c r="F620" s="41" t="inlineStr">
         <is>
-          <t>Incluía cepillo y pasta de dientes en baño; no disponible: hisopos, cepillo de pelo, espejo, toallas de piscina</t>
+          <t>Spa 1 abierto todo el año, todos los días</t>
         </is>
       </c>
       <c r="G620" s="41" t="inlineStr">
         <is>
-          <t>Baño con secador, toallas, gel, champú, acondicionador y gorro; cepillo/pasta de dientes y kit de afeitar a solicitud marcando 1</t>
+          <t>No tenemos servicio de spa</t>
         </is>
       </c>
     </row>
@@ -34584,32 +34584,32 @@
       </c>
       <c r="B621" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C621" s="41" t="inlineStr">
         <is>
-          <t>15-48</t>
+          <t>18-08</t>
         </is>
       </c>
       <c r="D621" s="41" t="inlineStr">
         <is>
-          <t>Electrical &amp; mobile phone facilities</t>
+          <t>Takeaway &amp; delivery</t>
         </is>
       </c>
       <c r="E621" s="41" t="inlineStr">
         <is>
-          <t>Adaptadores eléctricos</t>
+          <t>Domicilio</t>
         </is>
       </c>
       <c r="F621" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Domicilio 8h-18h previa solicitud, con cobro adicional</t>
         </is>
       </c>
       <c r="G621" s="41" t="inlineStr">
         <is>
-          <t>Adaptadores eléctricos: disponible gratuitamente</t>
+          <t>No tenemos domiciliario disponible</t>
         </is>
       </c>
     </row>
@@ -34621,32 +34621,32 @@
       </c>
       <c r="B622" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C622" s="41" t="inlineStr">
         <is>
-          <t>17-01</t>
+          <t>19-03</t>
         </is>
       </c>
       <c r="D622" s="41" t="inlineStr">
         <is>
-          <t>Bar</t>
+          <t>City center</t>
         </is>
       </c>
       <c r="E622" s="41" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Distancia al centro</t>
         </is>
       </c>
       <c r="F622" s="41" t="inlineStr">
         <is>
-          <t>Jue a sáb 12:00-22:30; domingo 12:00-21:00</t>
+          <t>A 142 km del centro</t>
         </is>
       </c>
       <c r="G622" s="41" t="inlineStr">
         <is>
-          <t>Abierto 7/7: lunes a sábado 12:00-22:00; domingos y festivos 12:00-21:00</t>
+          <t>A 2 cuadras del centro</t>
         </is>
       </c>
     </row>
@@ -34658,32 +34658,32 @@
       </c>
       <c r="B623" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Bogotá</t>
+          <t>GHL Hotel Abadía Plaza</t>
         </is>
       </c>
       <c r="C623" s="41" t="inlineStr">
         <is>
-          <t>17-31</t>
+          <t>20-21</t>
         </is>
       </c>
       <c r="D623" s="41" t="inlineStr">
         <is>
-          <t>Fitness gym</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="E623" s="41" t="inlineStr">
         <is>
-          <t>Existencia</t>
+          <t>Correo y teléfono eventos</t>
         </is>
       </c>
       <c r="F623" s="41" t="inlineStr">
         <is>
-          <t>No tenemos gimnasio</t>
+          <t>camila.dickens@ghlhoteles.com; +57 324 4547171</t>
         </is>
       </c>
       <c r="G623" s="41" t="inlineStr">
         <is>
-          <t>Espacio dotado para bienestar disponible 24 horas (⚠ Verificar en correo: no menciona ubicación ni precio)</t>
+          <t>eventos.abadiaplaza@ghlhoteles.com; +57 311 311 51 16</t>
         </is>
       </c>
     </row>
@@ -34700,27 +34700,27 @@
       </c>
       <c r="C624" s="41" t="inlineStr">
         <is>
-          <t>18-01</t>
+          <t>12-01</t>
         </is>
       </c>
       <c r="D624" s="41" t="inlineStr">
         <is>
-          <t>Restaurant</t>
+          <t>Breakfast time</t>
         </is>
       </c>
       <c r="E624" s="41" t="inlineStr">
         <is>
-          <t>Horarios</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F624" s="41" t="inlineStr">
         <is>
-          <t>Porterhouse jue-sáb 12:00-22:30, dom 12:00-21:00; Cook's 06:00-10:30</t>
+          <t>Todos los días 06:00-10:00 y 06:30-10:30 fines de semana</t>
         </is>
       </c>
       <c r="G624" s="41" t="inlineStr">
         <is>
-          <t>Porterhouse lunes a sábado 12:00-22:00, domingos y festivos 12:00-21:00; Cook's 06:00-12:00</t>
+          <t>Lunes a viernes 06:00-10:00; sábados, domingos y festivos 06:30-10:30</t>
         </is>
       </c>
     </row>
@@ -34732,32 +34732,32 @@
       </c>
       <c r="B625" s="41" t="inlineStr">
         <is>
-          <t>GHL Relax Hotel Corales de Indias</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C625" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13-17</t>
         </is>
       </c>
       <c r="D625" s="41" t="inlineStr">
         <is>
-          <t>Varios</t>
+          <t>Special requests</t>
         </is>
       </c>
       <c r="E625" s="41" t="inlineStr">
         <is>
-          <t>Ver adjunto</t>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="F625" s="41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Pedimos disculpas por no poder atender peticiones especiales</t>
         </is>
       </c>
       <c r="G625" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo (correcciones como anotaciones en 'Corales de Indias (003).pdf')</t>
+          <t>Puede contactarnos al correo reservas.sonestabogota@ghlhoteles.com</t>
         </is>
       </c>
     </row>
@@ -34769,32 +34769,32 @@
       </c>
       <c r="B626" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C626" s="41" t="inlineStr">
         <is>
-          <t>11-01</t>
+          <t>14-04</t>
         </is>
       </c>
       <c r="D626" s="41" t="inlineStr">
         <is>
-          <t>Check-in time</t>
+          <t>Smoking</t>
         </is>
       </c>
       <c r="E626" s="41" t="inlineStr">
         <is>
-          <t>Tarifa early check-in (desde 06:00)</t>
+          <t>Tarifa limpieza por humo</t>
         </is>
       </c>
       <c r="F626" s="41" t="inlineStr">
         <is>
-          <t>40 USD por habitación</t>
+          <t>350000 COP</t>
         </is>
       </c>
       <c r="G626" s="41" t="inlineStr">
         <is>
-          <t>50 USD por habitación</t>
+          <t>Desodorización equivalente a USD 100 diarios, al cambio de la TRM del día</t>
         </is>
       </c>
     </row>
@@ -34806,32 +34806,32 @@
       </c>
       <c r="B627" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C627" s="41" t="inlineStr">
         <is>
-          <t>11-11</t>
+          <t>15-06</t>
         </is>
       </c>
       <c r="D627" s="41" t="inlineStr">
         <is>
-          <t>Check-out time</t>
+          <t>Bathroom equipment</t>
         </is>
       </c>
       <c r="E627" s="41" t="inlineStr">
         <is>
-          <t>Tarifa late check-out (hasta 15:00)</t>
+          <t>Artículos a solicitud</t>
         </is>
       </c>
       <c r="F627" s="41" t="inlineStr">
         <is>
-          <t>40 USD por habitación</t>
+          <t>Incluía cepillo y pasta de dientes en baño; no disponible: hisopos, cepillo de pelo, espejo, toallas de piscina</t>
         </is>
       </c>
       <c r="G627" s="41" t="inlineStr">
         <is>
-          <t>50 USD por habitación</t>
+          <t>Baño con secador, toallas, gel, champú, acondicionador y gorro; cepillo/pasta de dientes y kit de afeitar a solicitud marcando 1</t>
         </is>
       </c>
     </row>
@@ -34843,32 +34843,32 @@
       </c>
       <c r="B628" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C628" s="41" t="inlineStr">
         <is>
-          <t>13-11</t>
+          <t>15-48</t>
         </is>
       </c>
       <c r="D628" s="41" t="inlineStr">
         <is>
-          <t>Wifi &amp; Internet</t>
+          <t>Electrical &amp; mobile phone facilities</t>
         </is>
       </c>
       <c r="E628" s="41" t="inlineStr">
         <is>
-          <t>Velocidad wifi dedicado</t>
+          <t>Adaptadores eléctricos</t>
         </is>
       </c>
       <c r="F628" s="41" t="inlineStr">
         <is>
-          <t>Wifi dedicado de 60 megas ilimitado</t>
+          <t>⚠ Verificar en correo</t>
         </is>
       </c>
       <c r="G628" s="41" t="inlineStr">
         <is>
-          <t>Wifi dedicado de 100 megas ilimitado</t>
+          <t>Adaptadores eléctricos: disponible gratuitamente</t>
         </is>
       </c>
     </row>
@@ -34880,32 +34880,32 @@
       </c>
       <c r="B629" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C629" s="41" t="inlineStr">
         <is>
-          <t>13-21</t>
+          <t>17-01</t>
         </is>
       </c>
       <c r="D629" s="41" t="inlineStr">
         <is>
-          <t>Kids</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="E629" s="41" t="inlineStr">
         <is>
-          <t>Tarifa infantil de 13 a 18 años</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="F629" s="41" t="inlineStr">
         <is>
-          <t>27 USD/noche</t>
+          <t>Jue a sáb 12:00-22:30; domingo 12:00-21:00</t>
         </is>
       </c>
       <c r="G629" s="41" t="inlineStr">
         <is>
-          <t>32.80 USD/noche</t>
+          <t>Abierto 7/7: lunes a sábado 12:00-22:00; domingos y festivos 12:00-21:00</t>
         </is>
       </c>
     </row>
@@ -34917,32 +34917,32 @@
       </c>
       <c r="B630" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C630" s="41" t="inlineStr">
         <is>
-          <t>13-43</t>
+          <t>17-31</t>
         </is>
       </c>
       <c r="D630" s="41" t="inlineStr">
         <is>
-          <t>Laundry</t>
+          <t>Fitness gym</t>
         </is>
       </c>
       <c r="E630" s="41" t="inlineStr">
         <is>
-          <t>Horario del servicio</t>
+          <t>Existencia</t>
         </is>
       </c>
       <c r="F630" s="41" t="inlineStr">
         <is>
-          <t>Objetos dados antes de las 10:00 se devuelven el mismo día antes de las 19:00</t>
+          <t>No tenemos gimnasio</t>
         </is>
       </c>
       <c r="G630" s="41" t="inlineStr">
         <is>
-          <t>Servicio de lavandería desde las 8:00 hasta las 16:00</t>
+          <t>Espacio dotado para bienestar disponible 24 horas (⚠ Verificar en correo: no menciona ubicación ni precio)</t>
         </is>
       </c>
     </row>
@@ -34954,32 +34954,32 @@
       </c>
       <c r="B631" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Loja</t>
+          <t>Sonesta Bogotá</t>
         </is>
       </c>
       <c r="C631" s="41" t="inlineStr">
         <is>
-          <t>13-50</t>
+          <t>18-01</t>
         </is>
       </c>
       <c r="D631" s="41" t="inlineStr">
         <is>
-          <t>Airport &amp; train station public transport</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="E631" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto</t>
+          <t>Horarios</t>
         </is>
       </c>
       <c r="F631" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto Internacional José Joaquín de Olmedo (GYE), 400 km</t>
+          <t>Porterhouse jue-sáb 12:00-22:30, dom 12:00-21:00; Cook's 06:00-10:30</t>
         </is>
       </c>
       <c r="G631" s="41" t="inlineStr">
         <is>
-          <t>Aeropuerto Ciudad de Catamayo (LOH), Catamayo</t>
+          <t>Porterhouse lunes a sábado 12:00-22:00, domingos y festivos 12:00-21:00; Cook's 06:00-12:00</t>
         </is>
       </c>
     </row>
@@ -34991,32 +34991,32 @@
       </c>
       <c r="B632" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cali</t>
+          <t>GHL Relax Hotel Corales de Indias</t>
         </is>
       </c>
       <c r="C632" s="41" t="inlineStr">
         <is>
-          <t>15-48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D632" s="41" t="inlineStr">
         <is>
-          <t>Electrical &amp; mobile phone facilities</t>
+          <t>Varios</t>
         </is>
       </c>
       <c r="E632" s="41" t="inlineStr">
         <is>
-          <t>Adaptadores y cargador de móvil</t>
+          <t>Ver adjunto</t>
         </is>
       </c>
       <c r="F632" s="41" t="inlineStr">
         <is>
-          <t>Disponibles gratuitamente</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G632" s="41" t="inlineStr">
         <is>
-          <t>No disponibles</t>
+          <t>⚠ Verificar en correo (correcciones como anotaciones en 'Corales de Indias (003).pdf')</t>
         </is>
       </c>
     </row>
@@ -35028,32 +35028,32 @@
       </c>
       <c r="B633" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cali</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C633" s="41" t="inlineStr">
         <is>
-          <t>16-10</t>
+          <t>11-01</t>
         </is>
       </c>
       <c r="D633" s="41" t="inlineStr">
         <is>
-          <t>Pets</t>
+          <t>Check-in time</t>
         </is>
       </c>
       <c r="E633" s="41" t="inlineStr">
         <is>
-          <t>Tasa animal de servicio/apoyo emocional y limpieza</t>
+          <t>Tarifa early check-in (desde 06:00)</t>
         </is>
       </c>
       <c r="F633" s="41" t="inlineStr">
         <is>
-          <t>No es necesario abonar ninguna tasa</t>
+          <t>40 USD por habitación</t>
         </is>
       </c>
       <c r="G633" s="41" t="inlineStr">
         <is>
-          <t>70000 COP/estancia</t>
+          <t>50 USD por habitación</t>
         </is>
       </c>
     </row>
@@ -35065,32 +35065,32 @@
       </c>
       <c r="B634" s="41" t="inlineStr">
         <is>
-          <t>Sonesta Cali</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C634" s="41" t="inlineStr">
         <is>
-          <t>17-34</t>
+          <t>11-11</t>
         </is>
       </c>
       <c r="D634" s="41" t="inlineStr">
         <is>
-          <t>Rooftop</t>
+          <t>Check-out time</t>
         </is>
       </c>
       <c r="E634" s="41" t="inlineStr">
         <is>
-          <t>Existencia del rooftop</t>
+          <t>Tarifa late check-out (hasta 15:00)</t>
         </is>
       </c>
       <c r="F634" s="41" t="inlineStr">
         <is>
-          <t>Terraza con vistas, abierta todo el año</t>
+          <t>40 USD por habitación</t>
         </is>
       </c>
       <c r="G634" s="41" t="inlineStr">
         <is>
-          <t>No disponemos de Rooftop</t>
+          <t>50 USD por habitación</t>
         </is>
       </c>
     </row>
@@ -35102,32 +35102,32 @@
       </c>
       <c r="B635" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C635" s="41" t="inlineStr">
         <is>
-          <t>16-02 (⚠ sin número en el texto)</t>
+          <t>13-11</t>
         </is>
       </c>
       <c r="D635" s="41" t="inlineStr">
         <is>
-          <t>Contact staff</t>
+          <t>Wifi &amp; Internet</t>
         </is>
       </c>
       <c r="E635" s="41" t="inlineStr">
         <is>
-          <t>Correo de Eventos</t>
+          <t>Velocidad wifi dedicado</t>
         </is>
       </c>
       <c r="F635" s="41" t="inlineStr">
         <is>
-          <t>carolina.gutierrez@ghlhoteles.com (Tel +56 45 252 7200)</t>
+          <t>Wifi dedicado de 60 megas ilimitado</t>
         </is>
       </c>
       <c r="G635" s="41" t="inlineStr">
         <is>
-          <t>catherinne.zuniga@ghlhoteles.com (el teléfono y el gratuito +56 45 252 7200 no cambian)</t>
+          <t>Wifi dedicado de 100 megas ilimitado</t>
         </is>
       </c>
     </row>
@@ -35139,32 +35139,32 @@
       </c>
       <c r="B636" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C636" s="41" t="inlineStr">
         <is>
-          <t>10-71</t>
+          <t>13-21</t>
         </is>
       </c>
       <c r="D636" s="41" t="inlineStr">
         <is>
-          <t>Payment method</t>
+          <t>Kids</t>
         </is>
       </c>
       <c r="E636" s="41" t="inlineStr">
         <is>
-          <t>Pago en cuotas</t>
+          <t>Tarifa infantil de 13 a 18 años</t>
         </is>
       </c>
       <c r="F636" s="41" t="inlineStr">
         <is>
-          <t>No aceptamos pago en cuotas</t>
+          <t>27 USD/noche</t>
         </is>
       </c>
       <c r="G636" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo: el hotel indica que el texto le queda poco claro; aclarar</t>
+          <t>32.80 USD/noche</t>
         </is>
       </c>
     </row>
@@ -35176,32 +35176,32 @@
       </c>
       <c r="B637" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C637" s="41" t="inlineStr">
         <is>
-          <t>10-74</t>
+          <t>13-43</t>
         </is>
       </c>
       <c r="D637" s="41" t="inlineStr">
         <is>
-          <t>Online payment</t>
+          <t>Laundry</t>
         </is>
       </c>
       <c r="E637" s="41" t="inlineStr">
         <is>
-          <t>Pago online</t>
+          <t>Horario del servicio</t>
         </is>
       </c>
       <c r="F637" s="41" t="inlineStr">
         <is>
-          <t>Lo sentimos, no aceptamos pago online</t>
+          <t>Objetos dados antes de las 10:00 se devuelven el mismo día antes de las 19:00</t>
         </is>
       </c>
       <c r="G637" s="41" t="inlineStr">
         <is>
-          <t>Sí aceptamos pago online, con link de pago</t>
+          <t>Servicio de lavandería desde las 8:00 hasta las 16:00</t>
         </is>
       </c>
     </row>
@@ -35213,32 +35213,32 @@
       </c>
       <c r="B638" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Loja</t>
         </is>
       </c>
       <c r="C638" s="41" t="inlineStr">
         <is>
-          <t>11-12</t>
+          <t>13-50</t>
         </is>
       </c>
       <c r="D638" s="41" t="inlineStr">
         <is>
-          <t>Late check-out</t>
+          <t>Airport &amp; train station public transport</t>
         </is>
       </c>
       <c r="E638" s="41" t="inlineStr">
         <is>
-          <t>Late check-out</t>
+          <t>Aeropuerto</t>
         </is>
       </c>
       <c r="F638" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Aeropuerto Internacional José Joaquín de Olmedo (GYE), 400 km</t>
         </is>
       </c>
       <c r="G638" s="41" t="inlineStr">
         <is>
-          <t>Sí hay opción de late check-out, con cargo del 50%</t>
+          <t>Aeropuerto Ciudad de Catamayo (LOH), Catamayo</t>
         </is>
       </c>
     </row>
@@ -35250,32 +35250,32 @@
       </c>
       <c r="B639" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Cali</t>
         </is>
       </c>
       <c r="C639" s="41" t="inlineStr">
         <is>
-          <t>14-01</t>
+          <t>15-48</t>
         </is>
       </c>
       <c r="D639" s="41" t="inlineStr">
         <is>
-          <t>Accommodation</t>
+          <t>Electrical &amp; mobile phone facilities</t>
         </is>
       </c>
       <c r="E639" s="41" t="inlineStr">
         <is>
-          <t>Nombres de habitaciones</t>
+          <t>Adaptadores y cargador de móvil</t>
         </is>
       </c>
       <c r="F639" s="41" t="inlineStr">
         <is>
-          <t>King Deluxe (39 hab); Deluxe Twin (13 hab); Junior Suite (5 hab); Suite Presidencial (1 hab)</t>
+          <t>Disponibles gratuitamente</t>
         </is>
       </c>
       <c r="G639" s="41" t="inlineStr">
         <is>
-          <t>'Superio Superior' (39 hab, ⚠ nombre escrito así, posible typo); Superior Doble Doble (13); Junior Suite King (5); Suite (1)</t>
+          <t>No disponibles</t>
         </is>
       </c>
     </row>
@@ -35287,32 +35287,32 @@
       </c>
       <c r="B640" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Cali</t>
         </is>
       </c>
       <c r="C640" s="41" t="inlineStr">
         <is>
-          <t>14-01</t>
+          <t>16-10</t>
         </is>
       </c>
       <c r="D640" s="41" t="inlineStr">
         <is>
-          <t>Accommodation</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="E640" s="41" t="inlineStr">
         <is>
-          <t>Habitaciones nuevas</t>
+          <t>Tasa animal de servicio/apoyo emocional y limpieza</t>
         </is>
       </c>
       <c r="F640" s="41" t="inlineStr">
         <is>
-          <t>Sin estos tipos</t>
+          <t>No es necesario abonar ninguna tasa</t>
         </is>
       </c>
       <c r="G640" s="41" t="inlineStr">
         <is>
-          <t>Agregar: Junior Superior (5 hab); Junior Suite Doble Doble (2 hab); Superior King (5 hab)</t>
+          <t>70000 COP/estancia</t>
         </is>
       </c>
     </row>
@@ -35324,32 +35324,32 @@
       </c>
       <c r="B641" s="41" t="inlineStr">
         <is>
-          <t>Park Lake Luxury</t>
+          <t>Sonesta Cali</t>
         </is>
       </c>
       <c r="C641" s="41" t="inlineStr">
         <is>
-          <t>14-01</t>
+          <t>17-34</t>
         </is>
       </c>
       <c r="D641" s="41" t="inlineStr">
         <is>
-          <t>Accommodation</t>
+          <t>Rooftop</t>
         </is>
       </c>
       <c r="E641" s="41" t="inlineStr">
         <is>
-          <t>Total de habitaciones</t>
+          <t>Existencia del rooftop</t>
         </is>
       </c>
       <c r="F641" s="41" t="inlineStr">
         <is>
-          <t>Incluye la habitación 707</t>
+          <t>Terraza con vistas, abierta todo el año</t>
         </is>
       </c>
       <c r="G641" s="41" t="inlineStr">
         <is>
-          <t>Descontar una habitación: la 707</t>
+          <t>No disponemos de Rooftop</t>
         </is>
       </c>
     </row>
@@ -35366,27 +35366,27 @@
       </c>
       <c r="C642" s="41" t="inlineStr">
         <is>
-          <t>14-02</t>
+          <t>16-02 (⚠ sin número en el texto)</t>
         </is>
       </c>
       <c r="D642" s="41" t="inlineStr">
         <is>
-          <t>Connecting &amp; close accommodation</t>
+          <t>Contact staff</t>
         </is>
       </c>
       <c r="E642" s="41" t="inlineStr">
         <is>
-          <t>Disponibilidad</t>
+          <t>Correo de Eventos</t>
         </is>
       </c>
       <c r="F642" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>carolina.gutierrez@ghlhoteles.com (Tel +56 45 252 7200)</t>
         </is>
       </c>
       <c r="G642" s="41" t="inlineStr">
         <is>
-          <t>Sí disponemos de opciones connecting</t>
+          <t>catherinne.zuniga@ghlhoteles.com (el teléfono y el gratuito +56 45 252 7200 no cambian)</t>
         </is>
       </c>
     </row>
@@ -35403,27 +35403,27 @@
       </c>
       <c r="C643" s="41" t="inlineStr">
         <is>
-          <t>15-09, 15-21, 15-61, 17-43</t>
+          <t>10-71</t>
         </is>
       </c>
       <c r="D643" s="41" t="inlineStr">
         <is>
-          <t>Varios</t>
+          <t>Payment method</t>
         </is>
       </c>
       <c r="E643" s="41" t="inlineStr">
         <is>
-          <t>Nombres de habitaciones</t>
+          <t>Pago en cuotas</t>
         </is>
       </c>
       <c r="F643" s="41" t="inlineStr">
         <is>
-          <t>Nombres anteriores de habitación</t>
+          <t>No aceptamos pago en cuotas</t>
         </is>
       </c>
       <c r="G643" s="41" t="inlineStr">
         <is>
-          <t>Actualizar los nombres de habitaciones según el punto 14-01</t>
+          <t>⚠ Verificar en correo: el hotel indica que el texto le queda poco claro; aclarar</t>
         </is>
       </c>
     </row>
@@ -35440,27 +35440,27 @@
       </c>
       <c r="C644" s="41" t="inlineStr">
         <is>
-          <t>15-23</t>
+          <t>10-74</t>
         </is>
       </c>
       <c r="D644" s="41" t="inlineStr">
         <is>
-          <t>Extra bed</t>
+          <t>Online payment</t>
         </is>
       </c>
       <c r="E644" s="41" t="inlineStr">
         <is>
-          <t>Disponibilidad</t>
+          <t>Pago online</t>
         </is>
       </c>
       <c r="F644" s="41" t="inlineStr">
         <is>
-          <t>⚠ Verificar en correo</t>
+          <t>Lo sentimos, no aceptamos pago online</t>
         </is>
       </c>
       <c r="G644" s="41" t="inlineStr">
         <is>
-          <t>Sí tenemos camas adicionales disponibles</t>
+          <t>Sí aceptamos pago online, con link de pago</t>
         </is>
       </c>
     </row>
@@ -35477,25 +35477,284 @@
       </c>
       <c r="C645" s="41" t="inlineStr">
         <is>
+          <t>11-12</t>
+        </is>
+      </c>
+      <c r="D645" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="E645" s="41" t="inlineStr">
+        <is>
+          <t>Late check-out</t>
+        </is>
+      </c>
+      <c r="F645" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G645" s="41" t="inlineStr">
+        <is>
+          <t>Sí hay opción de late check-out, con cargo del 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B646" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C646" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D646" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E646" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de habitaciones</t>
+        </is>
+      </c>
+      <c r="F646" s="41" t="inlineStr">
+        <is>
+          <t>King Deluxe (39 hab); Deluxe Twin (13 hab); Junior Suite (5 hab); Suite Presidencial (1 hab)</t>
+        </is>
+      </c>
+      <c r="G646" s="41" t="inlineStr">
+        <is>
+          <t>'Superio Superior' (39 hab, ⚠ nombre escrito así, posible typo); Superior Doble Doble (13); Junior Suite King (5); Suite (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B647" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C647" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D647" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E647" s="41" t="inlineStr">
+        <is>
+          <t>Habitaciones nuevas</t>
+        </is>
+      </c>
+      <c r="F647" s="41" t="inlineStr">
+        <is>
+          <t>Sin estos tipos</t>
+        </is>
+      </c>
+      <c r="G647" s="41" t="inlineStr">
+        <is>
+          <t>Agregar: Junior Superior (5 hab); Junior Suite Doble Doble (2 hab); Superior King (5 hab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B648" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C648" s="41" t="inlineStr">
+        <is>
+          <t>14-01</t>
+        </is>
+      </c>
+      <c r="D648" s="41" t="inlineStr">
+        <is>
+          <t>Accommodation</t>
+        </is>
+      </c>
+      <c r="E648" s="41" t="inlineStr">
+        <is>
+          <t>Total de habitaciones</t>
+        </is>
+      </c>
+      <c r="F648" s="41" t="inlineStr">
+        <is>
+          <t>Incluye la habitación 707</t>
+        </is>
+      </c>
+      <c r="G648" s="41" t="inlineStr">
+        <is>
+          <t>Descontar una habitación: la 707</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B649" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C649" s="41" t="inlineStr">
+        <is>
+          <t>14-02</t>
+        </is>
+      </c>
+      <c r="D649" s="41" t="inlineStr">
+        <is>
+          <t>Connecting &amp; close accommodation</t>
+        </is>
+      </c>
+      <c r="E649" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F649" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G649" s="41" t="inlineStr">
+        <is>
+          <t>Sí disponemos de opciones connecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B650" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C650" s="41" t="inlineStr">
+        <is>
+          <t>15-09, 15-21, 15-61, 17-43</t>
+        </is>
+      </c>
+      <c r="D650" s="41" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="E650" s="41" t="inlineStr">
+        <is>
+          <t>Nombres de habitaciones</t>
+        </is>
+      </c>
+      <c r="F650" s="41" t="inlineStr">
+        <is>
+          <t>Nombres anteriores de habitación</t>
+        </is>
+      </c>
+      <c r="G650" s="41" t="inlineStr">
+        <is>
+          <t>Actualizar los nombres de habitaciones según el punto 14-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B651" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C651" s="41" t="inlineStr">
+        <is>
+          <t>15-23</t>
+        </is>
+      </c>
+      <c r="D651" s="41" t="inlineStr">
+        <is>
+          <t>Extra bed</t>
+        </is>
+      </c>
+      <c r="E651" s="41" t="inlineStr">
+        <is>
+          <t>Disponibilidad</t>
+        </is>
+      </c>
+      <c r="F651" s="41" t="inlineStr">
+        <is>
+          <t>⚠ Verificar en correo</t>
+        </is>
+      </c>
+      <c r="G651" s="41" t="inlineStr">
+        <is>
+          <t>Sí tenemos camas adicionales disponibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="50" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B652" s="41" t="inlineStr">
+        <is>
+          <t>Park Lake Luxury</t>
+        </is>
+      </c>
+      <c r="C652" s="41" t="inlineStr">
+        <is>
           <t>17-01</t>
         </is>
       </c>
-      <c r="D645" s="41" t="inlineStr">
+      <c r="D652" s="41" t="inlineStr">
         <is>
           <t>Bar</t>
         </is>
       </c>
-      <c r="E645" s="41" t="inlineStr">
+      <c r="E652" s="41" t="inlineStr">
         <is>
           <t>Nombres de los bares</t>
         </is>
       </c>
-      <c r="F645" s="41" t="inlineStr">
+      <c r="F652" s="41" t="inlineStr">
         <is>
           <t>Equilibrium; Vertigo</t>
         </is>
       </c>
-      <c r="G645" s="41" t="inlineStr">
+      <c r="G652" s="41" t="inlineStr">
         <is>
           <t>Equilibrium lobby bar; Bar Lake</t>
         </is>

</xml_diff>

<commit_message>
Marca como Actualizado 16 hoteles de Oct-26 aplicados en el chatbot
Corales de Indias se mantiene Pendiente (sus correcciones están como
anotaciones en PDF sin transcribir).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
+++ b/Base_Maestra_Consolidada_Dialogos_Chatbot.xlsx
@@ -8812,14 +8812,19 @@
           <t>6 diálogos modificados: ventajas reserva directa, agencias de viaje, lavandería, cajero, teléfono de contacto, marketing</t>
         </is>
       </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr">
         <is>
           <t>Teléfono +57 316 0107651 (15-26, 15-61, 15-62, 17-44) ya se había reportado en Sep-26 (marcado Actualizado) pero el PDF de octubre aún mostraba el teléfono anterior — verificar que quedó aplicado en el chatbot</t>
         </is>
       </c>
-      <c r="K172" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K172" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8864,14 +8869,19 @@
           <t>14 diálogos modificados: contacto, check-in, desayuno, room service, mascotas, spa, gimnasio</t>
         </is>
       </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr">
         <is>
           <t>Cambios del 04/10 (BIOHOT.pdf aportado por el usuario); el 18/10 Sofía había escrito 'en orden, no se debe realizar ningún ajuste' — se registran los cambios del documento. Números 6-06, 6-10 y 7-43 aparecen así en el PDF y se asumieron 16-06, 16-10 y 17-43. 16-02 Eventos: el 'Ahora' viene rotulado Recepción con otro WhatsApp (+57 322 9736615). No respondió la ficha A&amp;B/Spa</t>
         </is>
       </c>
-      <c r="K173" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K173" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -8916,14 +8926,19 @@
           <t>3 diálogos modificados: check-in anticipado, lavandería, camas</t>
         </is>
       </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr">
         <is>
           <t>Respuesta de Andres Bohorquez (jefe de recepción). En 10-71 solo cambia la ortografía 'Diners' a 'Dinners' (no registrado, probable error). En 11-02 el texto visible del enlace es reservas.bioxury@ghlhoteles.com pero el href oculto sigue siendo reservas2.sunrise — confirmar. 15-21: Queen 140x200 es medida poco usual</t>
         </is>
       </c>
-      <c r="K174" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K174" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9052,14 +9067,19 @@
           <t>18 diálogos modificados: ubicación, contacto, pago, check-in, desayuno, parqueadero, traslados, habitaciones, camas, aire, gimnasio, restaurante</t>
         </is>
       </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr">
         <is>
           <t>Respuesta recibida el 05/10 fuera de la carpeta Octubre; col93.pdf (aportado por el usuario) confirma los números de diálogo con capturas (10-71 y 16-10 sin encabezado visible, inferidos). 13-45: el tiempo a pie sale mal porque el mapa apunta al hotel de Cota (se corrige con 19-01). Posible incoherencia: gimnasio en piso 6 vs '5 pisos' en 17-43</t>
         </is>
       </c>
-      <c r="K177" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K177" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9225,14 +9245,19 @@
           <t>20 diálogos modificados: reservas, descuentos, wifi, traslado, conectadas, fumadores, cama extra, balcón, visitas, spa, gimnasio, brunch, desayuno</t>
         </is>
       </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J181" t="inlineStr">
         <is>
           <t>Llegó como reenvío de Valentina Gonzalez (14/10) de un Word enviado por Maira Piza (original 02/10, respuesta a 'Diálogos desde Junio a la fecha'). Desayuno sin número en el docx (se asumen 12-01/12-02). 10-05, 10-08, 10-32 y 10-33 sin valor 'antes'. 14-02 ambiguo ('no contamos con conectadas' pero conserva lista Standard/Twin/Junior Suite). 14-04: pasa de 0 COP a 200 USD, confirmar CAPI.docx aportado por el usuario: 10-05, 10-08, 10-32 y 10-33 vienen sin marcas Antes/Ahora (texto único), el 'antes' sigue sin confirmar.</t>
         </is>
       </c>
-      <c r="K181" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K181" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9388,14 +9413,19 @@
           <t>5 diálogos modificados: remodelación, check-in, mascotas, pisos, piscina</t>
         </is>
       </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J185" t="inlineStr">
         <is>
           <t>Diálogo de mascotas sin número en el correo (se asume 16-10, el mismo de Sep-26). 17-43: dice Superior Twin en 'Planta baja - Planta Alta' pero mantiene '1 planta' (posible incoherencia). Nota informativa de la firma aún dice febrero a octubre. Adicional: ficha Restaurante Mangos (Km 2 vía Girardot - Melgar, Ricaurte; WhatsApp +57 3214693086; reservas.cubelpuente@ghlhoteles.com; teléfono '+57 214693086' y campo 'hotel' en blanco) — verificar</t>
         </is>
       </c>
-      <c r="K185" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K185" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9492,14 +9522,19 @@
           <t>1 diálogo modificado: taxi</t>
         </is>
       </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J187" t="inlineStr">
         <is>
           <t>En 13-53 también agregan el texto 'Horario de atención de 6:30 a.m. a 9:00 p.m.', idéntico al ejemplo del correo original (posible copia involuntaria) — NO registrado, confirmar con el hotel. Adicional: ficha Restaurante Yaharo (Km 19 vía Ciénaga, Santa Marta; tel 6054237074 - 6054237075; WhatsApp +57 3174588115; reservas.costaazul@ghlhoteles.com)</t>
         </is>
       </c>
-      <c r="K187" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K187" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9544,14 +9579,19 @@
           <t>1 diálogo modificado: planes tarifarios y upgrade (10-26)</t>
         </is>
       </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J188" t="inlineStr">
         <is>
           <t>Reenvía casi los mismos puntos ya aplicados en Sep-26 (16-02, 10-04, 10-06, 10-41, 10-71, 11-01, 12-01, 13-01, 13-21); solo el diálogo '0-26' (probable typo de 10-26) es nuevo y sin valor 'antes'. El hotel indicó que seguía revisando con calidad, puede llegar un segundo envío. En 10-41 pregunta si puede colocarse el flyer del pasadía en el enlace SUNRIS.docx aportado por el usuario coincide con el adjunto del correo (solo texto 'después').</t>
         </is>
       </c>
-      <c r="K188" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K188" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9596,14 +9636,19 @@
           <t>3 diálogos modificados: contacto, check-out, desayuno</t>
         </is>
       </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J189" t="inlineStr">
         <is>
           <t>Respondió Geraldine Centeno (recepcionista). Nombre del restaurante 'Yariguíes' normalizado (salió partido en el PDF); precio late check-out sube de 50.000 a 95.200 COP, validar</t>
         </is>
       </c>
-      <c r="K189" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K189" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9806,14 +9851,19 @@
           <t>12 diálogos modificados: recepción, desayuno, parqueadero, wifi, conserjería, aeropuerto, bar, spa, domicilio, centro, eventos</t>
         </is>
       </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J194" t="inlineStr">
         <is>
           <t>13-11: el 'después' quedó 'hay internet de alta velocidad' (posible typo). 13-50: texto cortado, falta la distancia. 17-01: el texto nuevo habla de coworking/café, no de bar (¿diálogo equivocado?). 12-02: niño sube a 33.000, igual al adulto. Adicional: ficha Restaurante Borbón (Cra. 8 # 21-67 esquina, Pereira; tel 606 349 68 70; WhatsApp +57 311 311 51 16; eventos.abadiaplaza@ghlhoteles.com)</t>
         </is>
       </c>
-      <c r="K194" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K194" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -9969,14 +10019,19 @@
           <t>11 diálogos modificados: contacto eventos, pago en cuotas y online, late check-out, habitaciones, connecting, cama extra, bares</t>
         </is>
       </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J198" t="inlineStr">
         <is>
           <t>Diálogo de Eventos sin número en el texto (se asume 16-02). 'Superio Superior' tal como lo escribió el hotel (posible typo). Cierra con: 'quedo atento y a disposición para seguir revisando cualquier otro punto'</t>
         </is>
       </c>
-      <c r="K198" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K198" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10105,14 +10160,19 @@
           <t>3 diálogos modificados: instalaciones eléctricas, mascotas, rooftop</t>
         </is>
       </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J201" t="inlineStr">
         <is>
           <t>16-10: el bloque 'Tasas' aparece dos veces; en el primero sigue 'no es necesario abonar tasa' y en el segundo 70000 COP/estancia — confirmar texto vigente</t>
         </is>
       </c>
-      <c r="K201" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K201" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10157,14 +10217,19 @@
           <t>25 diálogos modificados: pagos, check-in/out, desayuno, niños, peluquería, lavandería, traslados, vuelos, fumadores, camas, mascotas, alcohol, actividades, piscina, boutique</t>
         </is>
       </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J202" t="inlineStr">
         <is>
           <t>Liliana respondió con anotaciones sobre capturas del PDF (SONCART.pdf aportado por el usuario). Números tomados de las capturas; '(inferido)' = la captura no mostraba el encabezado; sin número: puertas insonorizadas y horario de piscina; '-44 Alcohol policy' venía truncado. Pregunta abierta: 'Pago por otra persona' (propone plasmar procedimiento de pagos por WOMPI). Kenny Maturana (gerencia) pidió el 06/10 revisar juntos</t>
         </is>
       </c>
-      <c r="K202" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K202" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10293,14 +10358,19 @@
           <t>7 diálogos modificados: wifi, lavandería, baño, ducha, empleo, propinas, restaurante</t>
         </is>
       </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J205" t="inlineStr">
         <is>
           <t>El 'antes' de 13-43, 16-06, 16-25 y 18-01 es el texto anterior a los cambios que ya reportó en Sep-26 (marcado Actualizado) — verificar que aquellos cambios sí quedaron aplicados. 16-06: el teléfono de RRHH ahora es +51 945 739 960 (en Sep dijo +51 054 308 777). El 'después' de 18-01 viene con líneas duplicadas. Adicional: fichas A&amp;B/Spa de Restaurante Micaela, Restobar Arcadia, Café Lobby bar y Sauna y Spa (City Towers, Torre Norte; WhatsApp Micaela/Arcadia +51 945 739 921, Spa +51 945 739 960; reservas restaurante.sonestaarequipa@ghlhoteles.com, spa recepcion1.sonestaarequipa@ghlhoteles.com)</t>
         </is>
       </c>
-      <c r="K205" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K205" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10345,14 +10415,19 @@
           <t>8 diálogos modificados: desayuno, solicitudes especiales, fumadores, baño, instalaciones eléctricas, bar, gimnasio, restaurante</t>
         </is>
       </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J206" t="inlineStr">
         <is>
           <t>Texto del adjunto reenviado aportado por el usuario: confirma 12-01, 13-17, 14-04, 15-06, 17-01 y 17-31 (igual al cuerpo del correo) y agrega 15-48 (solo adaptadores eléctricos, sin mencionar cargador de móvil). 18-01 solo viene en el cuerpo del correo. 17-31: el texto no menciona 'gimnasio'. El 'antes' se tomó del PDF original de octubre</t>
         </is>
       </c>
-      <c r="K206" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K206" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10434,14 +10509,19 @@
           <t>6 diálogos modificados: check-in, check-out, wifi, niños, lavandería, aeropuerto</t>
         </is>
       </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
       <c r="J208" t="inlineStr">
         <is>
           <t>13-11: el 'después' trae solo el párrafo del wifi dedicado de 100 megas (¿se mantiene la lista genérica?). Adicional: ficha Restaurante CASA LOJANA (4.º piso, Av. Zoilo Rodríguez y Antisana, Loja; tel (+593) 07 2579000; WhatsApp (+593) 999359283; casalojana@sonestaloja.com y ayb@sonestaloja.com)</t>
         </is>
       </c>
-      <c r="K208" s="46" t="inlineStr">
-        <is>
-          <t>Pendiente actualización</t>
+      <c r="K208" s="47" t="inlineStr">
+        <is>
+          <t>Actualizado</t>
         </is>
       </c>
     </row>
@@ -10892,7 +10972,7 @@
         <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>

</xml_diff>